<commit_message>
docs: update Test-Case file.xlsx
</commit_message>
<xml_diff>
--- a/Test-Case file.xlsx
+++ b/Test-Case file.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30516"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="332" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AE206F57-99A4-4130-A4C4-16491696909B}"/>
+  <xr:revisionPtr revIDLastSave="347" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5994A0C-0D4C-4F8C-8366-04A23CCE3D92}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="84">
   <si>
     <t>Functionality</t>
   </si>
@@ -238,9 +238,6 @@
 2. Confirm 'YES' is shown as the current gesture.</t>
   </si>
   <si>
-    <t>fail</t>
-  </si>
-  <si>
     <t>Open hand recognized as HELP</t>
   </si>
   <si>
@@ -250,6 +247,20 @@
   <si>
     <t>1. Show a HELP gesture hand sign.
 2. Confirm 'HELP' is shown as the current gesture.</t>
+  </si>
+  <si>
+    <t>Open hand recognized as FOOD</t>
+  </si>
+  <si>
+    <t>A  closed front palm with open/straight thumb and pinky finger
+ is classified as the FOOD gesture.</t>
+  </si>
+  <si>
+    <t>1. Show a FOOD gesture hand sign.
+2. Confirm 'FOOD' is shown as the current gesture.</t>
+  </si>
+  <si>
+    <t>fail</t>
   </si>
   <si>
     <t xml:space="preserve"> </t>
@@ -313,7 +324,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -332,6 +343,18 @@
       <color rgb="FF1E1B2E"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1E1B2E"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -342,12 +365,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -383,11 +406,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD8CDB3"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -405,20 +437,8 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -429,10 +449,23 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -777,16 +810,16 @@
       <c r="H1" s="5"/>
     </row>
     <row r="2" spans="1:8" ht="54" customHeight="1">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="D2" s="10" t="s">
         <v>7</v>
       </c>
       <c r="E2" s="5"/>
@@ -795,16 +828,16 @@
       <c r="H2" s="5"/>
     </row>
     <row r="3" spans="1:8" ht="36">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" s="10" t="s">
         <v>11</v>
       </c>
       <c r="E3" s="5"/>
@@ -813,16 +846,16 @@
       <c r="H3" s="5"/>
     </row>
     <row r="4" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E4" s="5"/>
@@ -831,16 +864,16 @@
       <c r="H4" s="5"/>
     </row>
     <row r="5" spans="1:8" ht="39" customHeight="1">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="C5" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="D5" s="10" t="s">
         <v>19</v>
       </c>
       <c r="E5" s="5"/>
@@ -1149,7 +1182,7 @@
       <c r="C2" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="8" t="s">
         <v>47</v>
       </c>
       <c r="E2" t="s">
@@ -1166,7 +1199,7 @@
       <c r="C3" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="7" t="s">
         <v>52</v>
       </c>
       <c r="E3" t="s">
@@ -1183,7 +1216,7 @@
       <c r="C4" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="7" t="s">
         <v>56</v>
       </c>
       <c r="E4" t="s">
@@ -1200,11 +1233,11 @@
       <c r="C5" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="7" t="s">
         <v>59</v>
       </c>
       <c r="E5" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="30.75">
@@ -1212,36 +1245,47 @@
         <v>49</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C6" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="D6" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="E6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="30.75">
+      <c r="A7" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="E6" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="12"/>
+      <c r="C7" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="E7" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
-      <c r="D8" s="12"/>
+      <c r="D8" s="8"/>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="6" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C29" s="6"/>
       <c r="D29" s="6"/>
@@ -1253,7 +1297,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65FDA647-655C-4116-8B17-6F3C6FAE8C07}">
-  <dimension ref="A1:P65"/>
+  <dimension ref="A1:SF65"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
@@ -1262,7 +1306,7 @@
     <col min="4" max="4" width="64.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:500">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1276,61 +1320,2053 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="60">
-      <c r="A2" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="D2" s="8" t="s">
+    <row r="2" spans="1:500" ht="36">
+      <c r="A2" s="11" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="72">
-      <c r="A3" s="7" t="s">
+      <c r="B2" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="C2" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="D2" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="E2" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="14"/>
+      <c r="K2" s="14"/>
+      <c r="L2" s="14"/>
+      <c r="M2" s="14"/>
+      <c r="N2" s="14"/>
+      <c r="O2" s="14"/>
+      <c r="P2" s="14"/>
+      <c r="Q2" s="14"/>
+      <c r="R2" s="14"/>
+      <c r="S2" s="14"/>
+      <c r="T2" s="14"/>
+      <c r="U2" s="14"/>
+      <c r="V2" s="14"/>
+      <c r="W2" s="14"/>
+      <c r="X2" s="14"/>
+      <c r="Y2" s="14"/>
+      <c r="Z2" s="14"/>
+      <c r="AA2" s="14"/>
+      <c r="AB2" s="14"/>
+      <c r="AC2" s="14"/>
+      <c r="AD2" s="14"/>
+      <c r="AE2" s="14"/>
+      <c r="AF2" s="14"/>
+      <c r="AG2" s="14"/>
+      <c r="AH2" s="14"/>
+      <c r="AI2" s="14"/>
+      <c r="AJ2" s="14"/>
+      <c r="AK2" s="14"/>
+      <c r="AL2" s="14"/>
+      <c r="AM2" s="14"/>
+      <c r="AN2" s="14"/>
+      <c r="AO2" s="14"/>
+      <c r="AP2" s="14"/>
+      <c r="AQ2" s="14"/>
+      <c r="AR2" s="14"/>
+      <c r="AS2" s="14"/>
+      <c r="AT2" s="14"/>
+      <c r="AU2" s="14"/>
+      <c r="AV2" s="14"/>
+      <c r="AW2" s="14"/>
+      <c r="AX2" s="14"/>
+      <c r="AY2" s="14"/>
+      <c r="AZ2" s="14"/>
+      <c r="BA2" s="14"/>
+      <c r="BB2" s="14"/>
+      <c r="BC2" s="14"/>
+      <c r="BD2" s="14"/>
+      <c r="BE2" s="14"/>
+      <c r="BF2" s="14"/>
+      <c r="BG2" s="14"/>
+      <c r="BH2" s="14"/>
+      <c r="BI2" s="14"/>
+      <c r="BJ2" s="14"/>
+      <c r="BK2" s="14"/>
+      <c r="BL2" s="14"/>
+      <c r="BM2" s="14"/>
+      <c r="BN2" s="14"/>
+      <c r="BO2" s="14"/>
+      <c r="BP2" s="14"/>
+      <c r="BQ2" s="14"/>
+      <c r="BR2" s="14"/>
+      <c r="BS2" s="14"/>
+      <c r="BT2" s="14"/>
+      <c r="BU2" s="14"/>
+      <c r="BV2" s="14"/>
+      <c r="BW2" s="14"/>
+      <c r="BX2" s="14"/>
+      <c r="BY2" s="14"/>
+      <c r="BZ2" s="14"/>
+      <c r="CA2" s="14"/>
+      <c r="CB2" s="14"/>
+      <c r="CC2" s="14"/>
+      <c r="CD2" s="14"/>
+      <c r="CE2" s="14"/>
+      <c r="CF2" s="14"/>
+      <c r="CG2" s="14"/>
+      <c r="CH2" s="14"/>
+      <c r="CI2" s="14"/>
+      <c r="CJ2" s="14"/>
+      <c r="CK2" s="14"/>
+      <c r="CL2" s="14"/>
+      <c r="CM2" s="14"/>
+      <c r="CN2" s="14"/>
+      <c r="CO2" s="14"/>
+      <c r="CP2" s="14"/>
+      <c r="CQ2" s="14"/>
+      <c r="CR2" s="14"/>
+      <c r="CS2" s="14"/>
+      <c r="CT2" s="14"/>
+      <c r="CU2" s="14"/>
+      <c r="CV2" s="14"/>
+      <c r="CW2" s="14"/>
+      <c r="CX2" s="14"/>
+      <c r="CY2" s="14"/>
+      <c r="CZ2" s="14"/>
+      <c r="DA2" s="14"/>
+      <c r="DB2" s="14"/>
+      <c r="DC2" s="14"/>
+      <c r="DD2" s="14"/>
+      <c r="DE2" s="14"/>
+      <c r="DF2" s="14"/>
+      <c r="DG2" s="14"/>
+      <c r="DH2" s="14"/>
+      <c r="DI2" s="14"/>
+      <c r="DJ2" s="14"/>
+      <c r="DK2" s="14"/>
+      <c r="DL2" s="14"/>
+      <c r="DM2" s="14"/>
+      <c r="DN2" s="14"/>
+      <c r="DO2" s="14"/>
+      <c r="DP2" s="14"/>
+      <c r="DQ2" s="14"/>
+      <c r="DR2" s="14"/>
+      <c r="DS2" s="14"/>
+      <c r="DT2" s="14"/>
+      <c r="DU2" s="14"/>
+      <c r="DV2" s="14"/>
+      <c r="DW2" s="14"/>
+      <c r="DX2" s="14"/>
+      <c r="DY2" s="14"/>
+      <c r="DZ2" s="14"/>
+      <c r="EA2" s="14"/>
+      <c r="EB2" s="14"/>
+      <c r="EC2" s="14"/>
+      <c r="ED2" s="14"/>
+      <c r="EE2" s="14"/>
+      <c r="EF2" s="14"/>
+      <c r="EG2" s="14"/>
+      <c r="EH2" s="14"/>
+      <c r="EI2" s="14"/>
+      <c r="EJ2" s="14"/>
+      <c r="EK2" s="14"/>
+      <c r="EL2" s="14"/>
+      <c r="EM2" s="14"/>
+      <c r="EN2" s="14"/>
+      <c r="EO2" s="14"/>
+      <c r="EP2" s="14"/>
+      <c r="EQ2" s="14"/>
+      <c r="ER2" s="14"/>
+      <c r="ES2" s="14"/>
+      <c r="ET2" s="14"/>
+      <c r="EU2" s="14"/>
+      <c r="EV2" s="14"/>
+      <c r="EW2" s="14"/>
+      <c r="EX2" s="14"/>
+      <c r="EY2" s="14"/>
+      <c r="EZ2" s="14"/>
+      <c r="FA2" s="14"/>
+      <c r="FB2" s="14"/>
+      <c r="FC2" s="14"/>
+      <c r="FD2" s="14"/>
+      <c r="FE2" s="14"/>
+      <c r="FF2" s="14"/>
+      <c r="FG2" s="14"/>
+      <c r="FH2" s="14"/>
+      <c r="FI2" s="14"/>
+      <c r="FJ2" s="14"/>
+      <c r="FK2" s="14"/>
+      <c r="FL2" s="14"/>
+      <c r="FM2" s="14"/>
+      <c r="FN2" s="14"/>
+      <c r="FO2" s="14"/>
+      <c r="FP2" s="14"/>
+      <c r="FQ2" s="14"/>
+      <c r="FR2" s="14"/>
+      <c r="FS2" s="14"/>
+      <c r="FT2" s="14"/>
+      <c r="FU2" s="14"/>
+      <c r="FV2" s="14"/>
+      <c r="FW2" s="14"/>
+      <c r="FX2" s="14"/>
+      <c r="FY2" s="14"/>
+      <c r="FZ2" s="14"/>
+      <c r="GA2" s="14"/>
+      <c r="GB2" s="14"/>
+      <c r="GC2" s="14"/>
+      <c r="GD2" s="14"/>
+      <c r="GE2" s="14"/>
+      <c r="GF2" s="14"/>
+      <c r="GG2" s="14"/>
+      <c r="GH2" s="14"/>
+      <c r="GI2" s="14"/>
+      <c r="GJ2" s="14"/>
+      <c r="GK2" s="14"/>
+      <c r="GL2" s="14"/>
+      <c r="GM2" s="14"/>
+      <c r="GN2" s="14"/>
+      <c r="GO2" s="14"/>
+      <c r="GP2" s="14"/>
+      <c r="GQ2" s="14"/>
+      <c r="GR2" s="14"/>
+      <c r="GS2" s="14"/>
+      <c r="GT2" s="14"/>
+      <c r="GU2" s="14"/>
+      <c r="GV2" s="14"/>
+      <c r="GW2" s="14"/>
+      <c r="GX2" s="14"/>
+      <c r="GY2" s="14"/>
+      <c r="GZ2" s="14"/>
+      <c r="HA2" s="14"/>
+      <c r="HB2" s="14"/>
+      <c r="HC2" s="14"/>
+      <c r="HD2" s="14"/>
+      <c r="HE2" s="14"/>
+      <c r="HF2" s="14"/>
+      <c r="HG2" s="14"/>
+      <c r="HH2" s="14"/>
+      <c r="HI2" s="14"/>
+      <c r="HJ2" s="14"/>
+      <c r="HK2" s="14"/>
+      <c r="HL2" s="14"/>
+      <c r="HM2" s="14"/>
+      <c r="HN2" s="14"/>
+      <c r="HO2" s="14"/>
+      <c r="HP2" s="14"/>
+      <c r="HQ2" s="14"/>
+      <c r="HR2" s="14"/>
+      <c r="HS2" s="14"/>
+      <c r="HT2" s="14"/>
+      <c r="HU2" s="14"/>
+      <c r="HV2" s="14"/>
+      <c r="HW2" s="14"/>
+      <c r="HX2" s="14"/>
+      <c r="HY2" s="14"/>
+      <c r="HZ2" s="14"/>
+      <c r="IA2" s="14"/>
+      <c r="IB2" s="14"/>
+      <c r="IC2" s="14"/>
+      <c r="ID2" s="14"/>
+      <c r="IE2" s="14"/>
+      <c r="IF2" s="14"/>
+      <c r="IG2" s="14"/>
+      <c r="IH2" s="14"/>
+      <c r="II2" s="14"/>
+      <c r="IJ2" s="14"/>
+      <c r="IK2" s="14"/>
+      <c r="IL2" s="14"/>
+      <c r="IM2" s="14"/>
+      <c r="IN2" s="14"/>
+      <c r="IO2" s="14"/>
+      <c r="IP2" s="14"/>
+      <c r="IQ2" s="14"/>
+      <c r="IR2" s="14"/>
+      <c r="IS2" s="14"/>
+      <c r="IT2" s="14"/>
+      <c r="IU2" s="14"/>
+      <c r="IV2" s="14"/>
+      <c r="IW2" s="14"/>
+      <c r="IX2" s="14"/>
+      <c r="IY2" s="14"/>
+      <c r="IZ2" s="14"/>
+      <c r="JA2" s="14"/>
+      <c r="JB2" s="14"/>
+      <c r="JC2" s="14"/>
+      <c r="JD2" s="14"/>
+      <c r="JE2" s="14"/>
+      <c r="JF2" s="14"/>
+      <c r="JG2" s="14"/>
+      <c r="JH2" s="14"/>
+      <c r="JI2" s="14"/>
+      <c r="JJ2" s="14"/>
+      <c r="JK2" s="14"/>
+      <c r="JL2" s="14"/>
+      <c r="JM2" s="14"/>
+      <c r="JN2" s="14"/>
+      <c r="JO2" s="14"/>
+      <c r="JP2" s="14"/>
+      <c r="JQ2" s="14"/>
+      <c r="JR2" s="14"/>
+      <c r="JS2" s="14"/>
+      <c r="JT2" s="14"/>
+      <c r="JU2" s="14"/>
+      <c r="JV2" s="14"/>
+      <c r="JW2" s="14"/>
+      <c r="JX2" s="14"/>
+      <c r="JY2" s="14"/>
+      <c r="JZ2" s="14"/>
+      <c r="KA2" s="14"/>
+      <c r="KB2" s="14"/>
+      <c r="KC2" s="14"/>
+      <c r="KD2" s="14"/>
+      <c r="KE2" s="14"/>
+      <c r="KF2" s="14"/>
+      <c r="KG2" s="14"/>
+      <c r="KH2" s="14"/>
+      <c r="KI2" s="14"/>
+      <c r="KJ2" s="14"/>
+      <c r="KK2" s="14"/>
+      <c r="KL2" s="14"/>
+      <c r="KM2" s="14"/>
+      <c r="KN2" s="14"/>
+      <c r="KO2" s="14"/>
+      <c r="KP2" s="14"/>
+      <c r="KQ2" s="14"/>
+      <c r="KR2" s="14"/>
+      <c r="KS2" s="14"/>
+      <c r="KT2" s="14"/>
+      <c r="KU2" s="14"/>
+      <c r="KV2" s="14"/>
+      <c r="KW2" s="14"/>
+      <c r="KX2" s="14"/>
+      <c r="KY2" s="14"/>
+      <c r="KZ2" s="14"/>
+      <c r="LA2" s="14"/>
+      <c r="LB2" s="14"/>
+      <c r="LC2" s="14"/>
+      <c r="LD2" s="14"/>
+      <c r="LE2" s="14"/>
+      <c r="LF2" s="14"/>
+      <c r="LG2" s="14"/>
+      <c r="LH2" s="14"/>
+      <c r="LI2" s="14"/>
+      <c r="LJ2" s="14"/>
+      <c r="LK2" s="14"/>
+      <c r="LL2" s="14"/>
+      <c r="LM2" s="14"/>
+      <c r="LN2" s="14"/>
+      <c r="LO2" s="14"/>
+      <c r="LP2" s="14"/>
+      <c r="LQ2" s="14"/>
+      <c r="LR2" s="14"/>
+      <c r="LS2" s="14"/>
+      <c r="LT2" s="14"/>
+      <c r="LU2" s="14"/>
+      <c r="LV2" s="14"/>
+      <c r="LW2" s="14"/>
+      <c r="LX2" s="14"/>
+      <c r="LY2" s="14"/>
+      <c r="LZ2" s="14"/>
+      <c r="MA2" s="14"/>
+      <c r="MB2" s="14"/>
+      <c r="MC2" s="14"/>
+      <c r="MD2" s="14"/>
+      <c r="ME2" s="14"/>
+      <c r="MF2" s="14"/>
+      <c r="MG2" s="14"/>
+      <c r="MH2" s="14"/>
+      <c r="MI2" s="14"/>
+      <c r="MJ2" s="14"/>
+      <c r="MK2" s="14"/>
+      <c r="ML2" s="14"/>
+      <c r="MM2" s="14"/>
+      <c r="MN2" s="14"/>
+      <c r="MO2" s="14"/>
+      <c r="MP2" s="14"/>
+      <c r="MQ2" s="14"/>
+      <c r="MR2" s="14"/>
+      <c r="MS2" s="14"/>
+      <c r="MT2" s="14"/>
+      <c r="MU2" s="14"/>
+      <c r="MV2" s="14"/>
+      <c r="MW2" s="14"/>
+      <c r="MX2" s="14"/>
+      <c r="MY2" s="14"/>
+      <c r="MZ2" s="14"/>
+      <c r="NA2" s="14"/>
+      <c r="NB2" s="14"/>
+      <c r="NC2" s="14"/>
+      <c r="ND2" s="14"/>
+      <c r="NE2" s="14"/>
+      <c r="NF2" s="14"/>
+      <c r="NG2" s="14"/>
+      <c r="NH2" s="14"/>
+      <c r="NI2" s="14"/>
+      <c r="NJ2" s="14"/>
+      <c r="NK2" s="14"/>
+      <c r="NL2" s="14"/>
+      <c r="NM2" s="14"/>
+      <c r="NN2" s="14"/>
+      <c r="NO2" s="14"/>
+      <c r="NP2" s="14"/>
+      <c r="NQ2" s="14"/>
+      <c r="NR2" s="14"/>
+      <c r="NS2" s="14"/>
+      <c r="NT2" s="14"/>
+      <c r="NU2" s="14"/>
+      <c r="NV2" s="14"/>
+      <c r="NW2" s="14"/>
+      <c r="NX2" s="14"/>
+      <c r="NY2" s="14"/>
+      <c r="NZ2" s="14"/>
+      <c r="OA2" s="14"/>
+      <c r="OB2" s="14"/>
+      <c r="OC2" s="14"/>
+      <c r="OD2" s="14"/>
+      <c r="OE2" s="14"/>
+      <c r="OF2" s="14"/>
+      <c r="OG2" s="14"/>
+      <c r="OH2" s="14"/>
+      <c r="OI2" s="14"/>
+      <c r="OJ2" s="14"/>
+      <c r="OK2" s="14"/>
+      <c r="OL2" s="14"/>
+      <c r="OM2" s="14"/>
+      <c r="ON2" s="14"/>
+      <c r="OO2" s="14"/>
+      <c r="OP2" s="14"/>
+      <c r="OQ2" s="14"/>
+      <c r="OR2" s="14"/>
+      <c r="OS2" s="14"/>
+      <c r="OT2" s="14"/>
+      <c r="OU2" s="14"/>
+      <c r="OV2" s="14"/>
+      <c r="OW2" s="14"/>
+      <c r="OX2" s="14"/>
+      <c r="OY2" s="14"/>
+      <c r="OZ2" s="14"/>
+      <c r="PA2" s="14"/>
+      <c r="PB2" s="14"/>
+      <c r="PC2" s="14"/>
+      <c r="PD2" s="14"/>
+      <c r="PE2" s="14"/>
+      <c r="PF2" s="14"/>
+      <c r="PG2" s="14"/>
+      <c r="PH2" s="14"/>
+      <c r="PI2" s="14"/>
+      <c r="PJ2" s="14"/>
+      <c r="PK2" s="14"/>
+      <c r="PL2" s="14"/>
+      <c r="PM2" s="14"/>
+      <c r="PN2" s="14"/>
+      <c r="PO2" s="14"/>
+      <c r="PP2" s="14"/>
+      <c r="PQ2" s="14"/>
+      <c r="PR2" s="14"/>
+      <c r="PS2" s="14"/>
+      <c r="PT2" s="14"/>
+      <c r="PU2" s="14"/>
+      <c r="PV2" s="14"/>
+      <c r="PW2" s="14"/>
+      <c r="PX2" s="14"/>
+      <c r="PY2" s="14"/>
+      <c r="PZ2" s="14"/>
+      <c r="QA2" s="14"/>
+      <c r="QB2" s="14"/>
+      <c r="QC2" s="14"/>
+      <c r="QD2" s="14"/>
+      <c r="QE2" s="14"/>
+      <c r="QF2" s="14"/>
+      <c r="QG2" s="14"/>
+      <c r="QH2" s="14"/>
+      <c r="QI2" s="14"/>
+      <c r="QJ2" s="14"/>
+      <c r="QK2" s="14"/>
+      <c r="QL2" s="14"/>
+      <c r="QM2" s="14"/>
+      <c r="QN2" s="14"/>
+      <c r="QO2" s="14"/>
+      <c r="QP2" s="14"/>
+      <c r="QQ2" s="14"/>
+      <c r="QR2" s="14"/>
+      <c r="QS2" s="14"/>
+      <c r="QT2" s="14"/>
+      <c r="QU2" s="14"/>
+      <c r="QV2" s="14"/>
+      <c r="QW2" s="14"/>
+      <c r="QX2" s="14"/>
+      <c r="QY2" s="14"/>
+      <c r="QZ2" s="14"/>
+      <c r="RA2" s="14"/>
+      <c r="RB2" s="14"/>
+      <c r="RC2" s="14"/>
+      <c r="RD2" s="14"/>
+      <c r="RE2" s="14"/>
+      <c r="RF2" s="14"/>
+      <c r="RG2" s="14"/>
+      <c r="RH2" s="14"/>
+      <c r="RI2" s="14"/>
+      <c r="RJ2" s="14"/>
+      <c r="RK2" s="14"/>
+      <c r="RL2" s="14"/>
+      <c r="RM2" s="14"/>
+      <c r="RN2" s="14"/>
+      <c r="RO2" s="14"/>
+      <c r="RP2" s="14"/>
+      <c r="RQ2" s="14"/>
+      <c r="RR2" s="14"/>
+      <c r="RS2" s="14"/>
+      <c r="RT2" s="14"/>
+      <c r="RU2" s="14"/>
+      <c r="RV2" s="14"/>
+      <c r="RW2" s="14"/>
+      <c r="RX2" s="14"/>
+      <c r="RY2" s="14"/>
+      <c r="RZ2" s="14"/>
+      <c r="SA2" s="14"/>
+      <c r="SB2" s="14"/>
+      <c r="SC2" s="14"/>
+      <c r="SD2" s="14"/>
+      <c r="SE2" s="14"/>
+      <c r="SF2" s="14"/>
+    </row>
+    <row r="3" spans="1:500" ht="36">
+      <c r="A3" s="11" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="24">
+      <c r="B3" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="14"/>
+      <c r="L3" s="14"/>
+      <c r="M3" s="14"/>
+      <c r="N3" s="14"/>
+      <c r="O3" s="14"/>
+      <c r="P3" s="14"/>
+      <c r="Q3" s="14"/>
+      <c r="R3" s="14"/>
+      <c r="S3" s="14"/>
+      <c r="T3" s="14"/>
+      <c r="U3" s="14"/>
+      <c r="V3" s="14"/>
+      <c r="W3" s="14"/>
+      <c r="X3" s="14"/>
+      <c r="Y3" s="14"/>
+      <c r="Z3" s="14"/>
+      <c r="AA3" s="14"/>
+      <c r="AB3" s="14"/>
+      <c r="AC3" s="14"/>
+      <c r="AD3" s="14"/>
+      <c r="AE3" s="14"/>
+      <c r="AF3" s="14"/>
+      <c r="AG3" s="14"/>
+      <c r="AH3" s="14"/>
+      <c r="AI3" s="14"/>
+      <c r="AJ3" s="14"/>
+      <c r="AK3" s="14"/>
+      <c r="AL3" s="14"/>
+      <c r="AM3" s="14"/>
+      <c r="AN3" s="14"/>
+      <c r="AO3" s="14"/>
+      <c r="AP3" s="14"/>
+      <c r="AQ3" s="14"/>
+      <c r="AR3" s="14"/>
+      <c r="AS3" s="14"/>
+      <c r="AT3" s="14"/>
+      <c r="AU3" s="14"/>
+      <c r="AV3" s="14"/>
+      <c r="AW3" s="14"/>
+      <c r="AX3" s="14"/>
+      <c r="AY3" s="14"/>
+      <c r="AZ3" s="14"/>
+      <c r="BA3" s="14"/>
+      <c r="BB3" s="14"/>
+      <c r="BC3" s="14"/>
+      <c r="BD3" s="14"/>
+      <c r="BE3" s="14"/>
+      <c r="BF3" s="14"/>
+      <c r="BG3" s="14"/>
+      <c r="BH3" s="14"/>
+      <c r="BI3" s="14"/>
+      <c r="BJ3" s="14"/>
+      <c r="BK3" s="14"/>
+      <c r="BL3" s="14"/>
+      <c r="BM3" s="14"/>
+      <c r="BN3" s="14"/>
+      <c r="BO3" s="14"/>
+      <c r="BP3" s="14"/>
+      <c r="BQ3" s="14"/>
+      <c r="BR3" s="14"/>
+      <c r="BS3" s="14"/>
+      <c r="BT3" s="14"/>
+      <c r="BU3" s="14"/>
+      <c r="BV3" s="14"/>
+      <c r="BW3" s="14"/>
+      <c r="BX3" s="14"/>
+      <c r="BY3" s="14"/>
+      <c r="BZ3" s="14"/>
+      <c r="CA3" s="14"/>
+      <c r="CB3" s="14"/>
+      <c r="CC3" s="14"/>
+      <c r="CD3" s="14"/>
+      <c r="CE3" s="14"/>
+      <c r="CF3" s="14"/>
+      <c r="CG3" s="14"/>
+      <c r="CH3" s="14"/>
+      <c r="CI3" s="14"/>
+      <c r="CJ3" s="14"/>
+      <c r="CK3" s="14"/>
+      <c r="CL3" s="14"/>
+      <c r="CM3" s="14"/>
+      <c r="CN3" s="14"/>
+      <c r="CO3" s="14"/>
+      <c r="CP3" s="14"/>
+      <c r="CQ3" s="14"/>
+      <c r="CR3" s="14"/>
+      <c r="CS3" s="14"/>
+      <c r="CT3" s="14"/>
+      <c r="CU3" s="14"/>
+      <c r="CV3" s="14"/>
+      <c r="CW3" s="14"/>
+      <c r="CX3" s="14"/>
+      <c r="CY3" s="14"/>
+      <c r="CZ3" s="14"/>
+      <c r="DA3" s="14"/>
+      <c r="DB3" s="14"/>
+      <c r="DC3" s="14"/>
+      <c r="DD3" s="14"/>
+      <c r="DE3" s="14"/>
+      <c r="DF3" s="14"/>
+      <c r="DG3" s="14"/>
+      <c r="DH3" s="14"/>
+      <c r="DI3" s="14"/>
+      <c r="DJ3" s="14"/>
+      <c r="DK3" s="14"/>
+      <c r="DL3" s="14"/>
+      <c r="DM3" s="14"/>
+      <c r="DN3" s="14"/>
+      <c r="DO3" s="14"/>
+      <c r="DP3" s="14"/>
+      <c r="DQ3" s="14"/>
+      <c r="DR3" s="14"/>
+      <c r="DS3" s="14"/>
+      <c r="DT3" s="14"/>
+      <c r="DU3" s="14"/>
+      <c r="DV3" s="14"/>
+      <c r="DW3" s="14"/>
+      <c r="DX3" s="14"/>
+      <c r="DY3" s="14"/>
+      <c r="DZ3" s="14"/>
+      <c r="EA3" s="14"/>
+      <c r="EB3" s="14"/>
+      <c r="EC3" s="14"/>
+      <c r="ED3" s="14"/>
+      <c r="EE3" s="14"/>
+      <c r="EF3" s="14"/>
+      <c r="EG3" s="14"/>
+      <c r="EH3" s="14"/>
+      <c r="EI3" s="14"/>
+      <c r="EJ3" s="14"/>
+      <c r="EK3" s="14"/>
+      <c r="EL3" s="14"/>
+      <c r="EM3" s="14"/>
+      <c r="EN3" s="14"/>
+      <c r="EO3" s="14"/>
+      <c r="EP3" s="14"/>
+      <c r="EQ3" s="14"/>
+      <c r="ER3" s="14"/>
+      <c r="ES3" s="14"/>
+      <c r="ET3" s="14"/>
+      <c r="EU3" s="14"/>
+      <c r="EV3" s="14"/>
+      <c r="EW3" s="14"/>
+      <c r="EX3" s="14"/>
+      <c r="EY3" s="14"/>
+      <c r="EZ3" s="14"/>
+      <c r="FA3" s="14"/>
+      <c r="FB3" s="14"/>
+      <c r="FC3" s="14"/>
+      <c r="FD3" s="14"/>
+      <c r="FE3" s="14"/>
+      <c r="FF3" s="14"/>
+      <c r="FG3" s="14"/>
+      <c r="FH3" s="14"/>
+      <c r="FI3" s="14"/>
+      <c r="FJ3" s="14"/>
+      <c r="FK3" s="14"/>
+      <c r="FL3" s="14"/>
+      <c r="FM3" s="14"/>
+      <c r="FN3" s="14"/>
+      <c r="FO3" s="14"/>
+      <c r="FP3" s="14"/>
+      <c r="FQ3" s="14"/>
+      <c r="FR3" s="14"/>
+      <c r="FS3" s="14"/>
+      <c r="FT3" s="14"/>
+      <c r="FU3" s="14"/>
+      <c r="FV3" s="14"/>
+      <c r="FW3" s="14"/>
+      <c r="FX3" s="14"/>
+      <c r="FY3" s="14"/>
+      <c r="FZ3" s="14"/>
+      <c r="GA3" s="14"/>
+      <c r="GB3" s="14"/>
+      <c r="GC3" s="14"/>
+      <c r="GD3" s="14"/>
+      <c r="GE3" s="14"/>
+      <c r="GF3" s="14"/>
+      <c r="GG3" s="14"/>
+      <c r="GH3" s="14"/>
+      <c r="GI3" s="14"/>
+      <c r="GJ3" s="14"/>
+      <c r="GK3" s="14"/>
+      <c r="GL3" s="14"/>
+      <c r="GM3" s="14"/>
+      <c r="GN3" s="14"/>
+      <c r="GO3" s="14"/>
+      <c r="GP3" s="14"/>
+      <c r="GQ3" s="14"/>
+      <c r="GR3" s="14"/>
+      <c r="GS3" s="14"/>
+      <c r="GT3" s="14"/>
+      <c r="GU3" s="14"/>
+      <c r="GV3" s="14"/>
+      <c r="GW3" s="14"/>
+      <c r="GX3" s="14"/>
+      <c r="GY3" s="14"/>
+      <c r="GZ3" s="14"/>
+      <c r="HA3" s="14"/>
+      <c r="HB3" s="14"/>
+      <c r="HC3" s="14"/>
+      <c r="HD3" s="14"/>
+      <c r="HE3" s="14"/>
+      <c r="HF3" s="14"/>
+      <c r="HG3" s="14"/>
+      <c r="HH3" s="14"/>
+      <c r="HI3" s="14"/>
+      <c r="HJ3" s="14"/>
+      <c r="HK3" s="14"/>
+      <c r="HL3" s="14"/>
+      <c r="HM3" s="14"/>
+      <c r="HN3" s="14"/>
+      <c r="HO3" s="14"/>
+      <c r="HP3" s="14"/>
+      <c r="HQ3" s="14"/>
+      <c r="HR3" s="14"/>
+      <c r="HS3" s="14"/>
+      <c r="HT3" s="14"/>
+      <c r="HU3" s="14"/>
+      <c r="HV3" s="14"/>
+      <c r="HW3" s="14"/>
+      <c r="HX3" s="14"/>
+      <c r="HY3" s="14"/>
+      <c r="HZ3" s="14"/>
+      <c r="IA3" s="14"/>
+      <c r="IB3" s="14"/>
+      <c r="IC3" s="14"/>
+      <c r="ID3" s="14"/>
+      <c r="IE3" s="14"/>
+      <c r="IF3" s="14"/>
+      <c r="IG3" s="14"/>
+      <c r="IH3" s="14"/>
+      <c r="II3" s="14"/>
+      <c r="IJ3" s="14"/>
+      <c r="IK3" s="14"/>
+      <c r="IL3" s="14"/>
+      <c r="IM3" s="14"/>
+      <c r="IN3" s="14"/>
+      <c r="IO3" s="14"/>
+      <c r="IP3" s="14"/>
+      <c r="IQ3" s="14"/>
+      <c r="IR3" s="14"/>
+      <c r="IS3" s="14"/>
+      <c r="IT3" s="14"/>
+      <c r="IU3" s="14"/>
+      <c r="IV3" s="14"/>
+      <c r="IW3" s="14"/>
+      <c r="IX3" s="14"/>
+      <c r="IY3" s="14"/>
+      <c r="IZ3" s="14"/>
+      <c r="JA3" s="14"/>
+      <c r="JB3" s="14"/>
+      <c r="JC3" s="14"/>
+      <c r="JD3" s="14"/>
+      <c r="JE3" s="14"/>
+      <c r="JF3" s="14"/>
+      <c r="JG3" s="14"/>
+      <c r="JH3" s="14"/>
+      <c r="JI3" s="14"/>
+      <c r="JJ3" s="14"/>
+      <c r="JK3" s="14"/>
+      <c r="JL3" s="14"/>
+      <c r="JM3" s="14"/>
+      <c r="JN3" s="14"/>
+      <c r="JO3" s="14"/>
+      <c r="JP3" s="14"/>
+      <c r="JQ3" s="14"/>
+      <c r="JR3" s="14"/>
+      <c r="JS3" s="14"/>
+      <c r="JT3" s="14"/>
+      <c r="JU3" s="14"/>
+      <c r="JV3" s="14"/>
+      <c r="JW3" s="14"/>
+      <c r="JX3" s="14"/>
+      <c r="JY3" s="14"/>
+      <c r="JZ3" s="14"/>
+      <c r="KA3" s="14"/>
+      <c r="KB3" s="14"/>
+      <c r="KC3" s="14"/>
+      <c r="KD3" s="14"/>
+      <c r="KE3" s="14"/>
+      <c r="KF3" s="14"/>
+      <c r="KG3" s="14"/>
+      <c r="KH3" s="14"/>
+      <c r="KI3" s="14"/>
+      <c r="KJ3" s="14"/>
+      <c r="KK3" s="14"/>
+      <c r="KL3" s="14"/>
+      <c r="KM3" s="14"/>
+      <c r="KN3" s="14"/>
+      <c r="KO3" s="14"/>
+      <c r="KP3" s="14"/>
+      <c r="KQ3" s="14"/>
+      <c r="KR3" s="14"/>
+      <c r="KS3" s="14"/>
+      <c r="KT3" s="14"/>
+      <c r="KU3" s="14"/>
+      <c r="KV3" s="14"/>
+      <c r="KW3" s="14"/>
+      <c r="KX3" s="14"/>
+      <c r="KY3" s="14"/>
+      <c r="KZ3" s="14"/>
+      <c r="LA3" s="14"/>
+      <c r="LB3" s="14"/>
+      <c r="LC3" s="14"/>
+      <c r="LD3" s="14"/>
+      <c r="LE3" s="14"/>
+      <c r="LF3" s="14"/>
+      <c r="LG3" s="14"/>
+      <c r="LH3" s="14"/>
+      <c r="LI3" s="14"/>
+      <c r="LJ3" s="14"/>
+      <c r="LK3" s="14"/>
+      <c r="LL3" s="14"/>
+      <c r="LM3" s="14"/>
+      <c r="LN3" s="14"/>
+      <c r="LO3" s="14"/>
+      <c r="LP3" s="14"/>
+      <c r="LQ3" s="14"/>
+      <c r="LR3" s="14"/>
+      <c r="LS3" s="14"/>
+      <c r="LT3" s="14"/>
+      <c r="LU3" s="14"/>
+      <c r="LV3" s="14"/>
+      <c r="LW3" s="14"/>
+      <c r="LX3" s="14"/>
+      <c r="LY3" s="14"/>
+      <c r="LZ3" s="14"/>
+      <c r="MA3" s="14"/>
+      <c r="MB3" s="14"/>
+      <c r="MC3" s="14"/>
+      <c r="MD3" s="14"/>
+      <c r="ME3" s="14"/>
+      <c r="MF3" s="14"/>
+      <c r="MG3" s="14"/>
+      <c r="MH3" s="14"/>
+      <c r="MI3" s="14"/>
+      <c r="MJ3" s="14"/>
+      <c r="MK3" s="14"/>
+      <c r="ML3" s="14"/>
+      <c r="MM3" s="14"/>
+      <c r="MN3" s="14"/>
+      <c r="MO3" s="14"/>
+      <c r="MP3" s="14"/>
+      <c r="MQ3" s="14"/>
+      <c r="MR3" s="14"/>
+      <c r="MS3" s="14"/>
+      <c r="MT3" s="14"/>
+      <c r="MU3" s="14"/>
+      <c r="MV3" s="14"/>
+      <c r="MW3" s="14"/>
+      <c r="MX3" s="14"/>
+      <c r="MY3" s="14"/>
+      <c r="MZ3" s="14"/>
+      <c r="NA3" s="14"/>
+      <c r="NB3" s="14"/>
+      <c r="NC3" s="14"/>
+      <c r="ND3" s="14"/>
+      <c r="NE3" s="14"/>
+      <c r="NF3" s="14"/>
+      <c r="NG3" s="14"/>
+      <c r="NH3" s="14"/>
+      <c r="NI3" s="14"/>
+      <c r="NJ3" s="14"/>
+      <c r="NK3" s="14"/>
+      <c r="NL3" s="14"/>
+      <c r="NM3" s="14"/>
+      <c r="NN3" s="14"/>
+      <c r="NO3" s="14"/>
+      <c r="NP3" s="14"/>
+      <c r="NQ3" s="14"/>
+      <c r="NR3" s="14"/>
+      <c r="NS3" s="14"/>
+      <c r="NT3" s="14"/>
+      <c r="NU3" s="14"/>
+      <c r="NV3" s="14"/>
+      <c r="NW3" s="14"/>
+      <c r="NX3" s="14"/>
+      <c r="NY3" s="14"/>
+      <c r="NZ3" s="14"/>
+      <c r="OA3" s="14"/>
+      <c r="OB3" s="14"/>
+      <c r="OC3" s="14"/>
+      <c r="OD3" s="14"/>
+      <c r="OE3" s="14"/>
+      <c r="OF3" s="14"/>
+      <c r="OG3" s="14"/>
+      <c r="OH3" s="14"/>
+      <c r="OI3" s="14"/>
+      <c r="OJ3" s="14"/>
+      <c r="OK3" s="14"/>
+      <c r="OL3" s="14"/>
+      <c r="OM3" s="14"/>
+      <c r="ON3" s="14"/>
+      <c r="OO3" s="14"/>
+      <c r="OP3" s="14"/>
+      <c r="OQ3" s="14"/>
+      <c r="OR3" s="14"/>
+      <c r="OS3" s="14"/>
+      <c r="OT3" s="14"/>
+      <c r="OU3" s="14"/>
+      <c r="OV3" s="14"/>
+      <c r="OW3" s="14"/>
+      <c r="OX3" s="14"/>
+      <c r="OY3" s="14"/>
+      <c r="OZ3" s="14"/>
+      <c r="PA3" s="14"/>
+      <c r="PB3" s="14"/>
+      <c r="PC3" s="14"/>
+      <c r="PD3" s="14"/>
+      <c r="PE3" s="14"/>
+      <c r="PF3" s="14"/>
+      <c r="PG3" s="14"/>
+      <c r="PH3" s="14"/>
+      <c r="PI3" s="14"/>
+      <c r="PJ3" s="14"/>
+      <c r="PK3" s="14"/>
+      <c r="PL3" s="14"/>
+      <c r="PM3" s="14"/>
+      <c r="PN3" s="14"/>
+      <c r="PO3" s="14"/>
+      <c r="PP3" s="14"/>
+      <c r="PQ3" s="14"/>
+      <c r="PR3" s="14"/>
+      <c r="PS3" s="14"/>
+      <c r="PT3" s="14"/>
+      <c r="PU3" s="14"/>
+      <c r="PV3" s="14"/>
+      <c r="PW3" s="14"/>
+      <c r="PX3" s="14"/>
+      <c r="PY3" s="14"/>
+      <c r="PZ3" s="14"/>
+      <c r="QA3" s="14"/>
+      <c r="QB3" s="14"/>
+      <c r="QC3" s="14"/>
+      <c r="QD3" s="14"/>
+      <c r="QE3" s="14"/>
+      <c r="QF3" s="14"/>
+      <c r="QG3" s="14"/>
+      <c r="QH3" s="14"/>
+      <c r="QI3" s="14"/>
+      <c r="QJ3" s="14"/>
+      <c r="QK3" s="14"/>
+      <c r="QL3" s="14"/>
+      <c r="QM3" s="14"/>
+      <c r="QN3" s="14"/>
+      <c r="QO3" s="14"/>
+      <c r="QP3" s="14"/>
+      <c r="QQ3" s="14"/>
+      <c r="QR3" s="14"/>
+      <c r="QS3" s="14"/>
+      <c r="QT3" s="14"/>
+      <c r="QU3" s="14"/>
+      <c r="QV3" s="14"/>
+      <c r="QW3" s="14"/>
+      <c r="QX3" s="14"/>
+      <c r="QY3" s="14"/>
+      <c r="QZ3" s="14"/>
+      <c r="RA3" s="14"/>
+      <c r="RB3" s="14"/>
+      <c r="RC3" s="14"/>
+      <c r="RD3" s="14"/>
+      <c r="RE3" s="14"/>
+      <c r="RF3" s="14"/>
+      <c r="RG3" s="14"/>
+      <c r="RH3" s="14"/>
+      <c r="RI3" s="14"/>
+      <c r="RJ3" s="14"/>
+      <c r="RK3" s="14"/>
+      <c r="RL3" s="14"/>
+      <c r="RM3" s="14"/>
+      <c r="RN3" s="14"/>
+      <c r="RO3" s="14"/>
+      <c r="RP3" s="14"/>
+      <c r="RQ3" s="14"/>
+      <c r="RR3" s="14"/>
+      <c r="RS3" s="14"/>
+      <c r="RT3" s="14"/>
+      <c r="RU3" s="14"/>
+      <c r="RV3" s="14"/>
+      <c r="RW3" s="14"/>
+      <c r="RX3" s="14"/>
+      <c r="RY3" s="14"/>
+      <c r="RZ3" s="14"/>
+      <c r="SA3" s="14"/>
+      <c r="SB3" s="14"/>
+      <c r="SC3" s="14"/>
+      <c r="SD3" s="14"/>
+      <c r="SE3" s="14"/>
+      <c r="SF3" s="14"/>
+    </row>
+    <row r="4" spans="1:500" ht="24">
       <c r="A4" s="15" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="36">
-      <c r="A5" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="C5" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="E4" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="14"/>
+      <c r="K4" s="14"/>
+      <c r="L4" s="14"/>
+      <c r="M4" s="14"/>
+      <c r="N4" s="14"/>
+      <c r="O4" s="14"/>
+      <c r="P4" s="14"/>
+      <c r="Q4" s="14"/>
+      <c r="R4" s="14"/>
+      <c r="S4" s="14"/>
+      <c r="T4" s="14"/>
+      <c r="U4" s="14"/>
+      <c r="V4" s="14"/>
+      <c r="W4" s="14"/>
+      <c r="X4" s="14"/>
+      <c r="Y4" s="14"/>
+      <c r="Z4" s="14"/>
+      <c r="AA4" s="14"/>
+      <c r="AB4" s="14"/>
+      <c r="AC4" s="14"/>
+      <c r="AD4" s="14"/>
+      <c r="AE4" s="14"/>
+      <c r="AF4" s="14"/>
+      <c r="AG4" s="14"/>
+      <c r="AH4" s="14"/>
+      <c r="AI4" s="14"/>
+      <c r="AJ4" s="14"/>
+      <c r="AK4" s="14"/>
+      <c r="AL4" s="14"/>
+      <c r="AM4" s="14"/>
+      <c r="AN4" s="14"/>
+      <c r="AO4" s="14"/>
+      <c r="AP4" s="14"/>
+      <c r="AQ4" s="14"/>
+      <c r="AR4" s="14"/>
+      <c r="AS4" s="14"/>
+      <c r="AT4" s="14"/>
+      <c r="AU4" s="14"/>
+      <c r="AV4" s="14"/>
+      <c r="AW4" s="14"/>
+      <c r="AX4" s="14"/>
+      <c r="AY4" s="14"/>
+      <c r="AZ4" s="14"/>
+      <c r="BA4" s="14"/>
+      <c r="BB4" s="14"/>
+      <c r="BC4" s="14"/>
+      <c r="BD4" s="14"/>
+      <c r="BE4" s="14"/>
+      <c r="BF4" s="14"/>
+      <c r="BG4" s="14"/>
+      <c r="BH4" s="14"/>
+      <c r="BI4" s="14"/>
+      <c r="BJ4" s="14"/>
+      <c r="BK4" s="14"/>
+      <c r="BL4" s="14"/>
+      <c r="BM4" s="14"/>
+      <c r="BN4" s="14"/>
+      <c r="BO4" s="14"/>
+      <c r="BP4" s="14"/>
+      <c r="BQ4" s="14"/>
+      <c r="BR4" s="14"/>
+      <c r="BS4" s="14"/>
+      <c r="BT4" s="14"/>
+      <c r="BU4" s="14"/>
+      <c r="BV4" s="14"/>
+      <c r="BW4" s="14"/>
+      <c r="BX4" s="14"/>
+      <c r="BY4" s="14"/>
+      <c r="BZ4" s="14"/>
+      <c r="CA4" s="14"/>
+      <c r="CB4" s="14"/>
+      <c r="CC4" s="14"/>
+      <c r="CD4" s="14"/>
+      <c r="CE4" s="14"/>
+      <c r="CF4" s="14"/>
+      <c r="CG4" s="14"/>
+      <c r="CH4" s="14"/>
+      <c r="CI4" s="14"/>
+      <c r="CJ4" s="14"/>
+      <c r="CK4" s="14"/>
+      <c r="CL4" s="14"/>
+      <c r="CM4" s="14"/>
+      <c r="CN4" s="14"/>
+      <c r="CO4" s="14"/>
+      <c r="CP4" s="14"/>
+      <c r="CQ4" s="14"/>
+      <c r="CR4" s="14"/>
+      <c r="CS4" s="14"/>
+      <c r="CT4" s="14"/>
+      <c r="CU4" s="14"/>
+      <c r="CV4" s="14"/>
+      <c r="CW4" s="14"/>
+      <c r="CX4" s="14"/>
+      <c r="CY4" s="14"/>
+      <c r="CZ4" s="14"/>
+      <c r="DA4" s="14"/>
+      <c r="DB4" s="14"/>
+      <c r="DC4" s="14"/>
+      <c r="DD4" s="14"/>
+      <c r="DE4" s="14"/>
+      <c r="DF4" s="14"/>
+      <c r="DG4" s="14"/>
+      <c r="DH4" s="14"/>
+      <c r="DI4" s="14"/>
+      <c r="DJ4" s="14"/>
+      <c r="DK4" s="14"/>
+      <c r="DL4" s="14"/>
+      <c r="DM4" s="14"/>
+      <c r="DN4" s="14"/>
+      <c r="DO4" s="14"/>
+      <c r="DP4" s="14"/>
+      <c r="DQ4" s="14"/>
+      <c r="DR4" s="14"/>
+      <c r="DS4" s="14"/>
+      <c r="DT4" s="14"/>
+      <c r="DU4" s="14"/>
+      <c r="DV4" s="14"/>
+      <c r="DW4" s="14"/>
+      <c r="DX4" s="14"/>
+      <c r="DY4" s="14"/>
+      <c r="DZ4" s="14"/>
+      <c r="EA4" s="14"/>
+      <c r="EB4" s="14"/>
+      <c r="EC4" s="14"/>
+      <c r="ED4" s="14"/>
+      <c r="EE4" s="14"/>
+      <c r="EF4" s="14"/>
+      <c r="EG4" s="14"/>
+      <c r="EH4" s="14"/>
+      <c r="EI4" s="14"/>
+      <c r="EJ4" s="14"/>
+      <c r="EK4" s="14"/>
+      <c r="EL4" s="14"/>
+      <c r="EM4" s="14"/>
+      <c r="EN4" s="14"/>
+      <c r="EO4" s="14"/>
+      <c r="EP4" s="14"/>
+      <c r="EQ4" s="14"/>
+      <c r="ER4" s="14"/>
+      <c r="ES4" s="14"/>
+      <c r="ET4" s="14"/>
+      <c r="EU4" s="14"/>
+      <c r="EV4" s="14"/>
+      <c r="EW4" s="14"/>
+      <c r="EX4" s="14"/>
+      <c r="EY4" s="14"/>
+      <c r="EZ4" s="14"/>
+      <c r="FA4" s="14"/>
+      <c r="FB4" s="14"/>
+      <c r="FC4" s="14"/>
+      <c r="FD4" s="14"/>
+      <c r="FE4" s="14"/>
+      <c r="FF4" s="14"/>
+      <c r="FG4" s="14"/>
+      <c r="FH4" s="14"/>
+      <c r="FI4" s="14"/>
+      <c r="FJ4" s="14"/>
+      <c r="FK4" s="14"/>
+      <c r="FL4" s="14"/>
+      <c r="FM4" s="14"/>
+      <c r="FN4" s="14"/>
+      <c r="FO4" s="14"/>
+      <c r="FP4" s="14"/>
+      <c r="FQ4" s="14"/>
+      <c r="FR4" s="14"/>
+      <c r="FS4" s="14"/>
+      <c r="FT4" s="14"/>
+      <c r="FU4" s="14"/>
+      <c r="FV4" s="14"/>
+      <c r="FW4" s="14"/>
+      <c r="FX4" s="14"/>
+      <c r="FY4" s="14"/>
+      <c r="FZ4" s="14"/>
+      <c r="GA4" s="14"/>
+      <c r="GB4" s="14"/>
+      <c r="GC4" s="14"/>
+      <c r="GD4" s="14"/>
+      <c r="GE4" s="14"/>
+      <c r="GF4" s="14"/>
+      <c r="GG4" s="14"/>
+      <c r="GH4" s="14"/>
+      <c r="GI4" s="14"/>
+      <c r="GJ4" s="14"/>
+      <c r="GK4" s="14"/>
+      <c r="GL4" s="14"/>
+      <c r="GM4" s="14"/>
+      <c r="GN4" s="14"/>
+      <c r="GO4" s="14"/>
+      <c r="GP4" s="14"/>
+      <c r="GQ4" s="14"/>
+      <c r="GR4" s="14"/>
+      <c r="GS4" s="14"/>
+      <c r="GT4" s="14"/>
+      <c r="GU4" s="14"/>
+      <c r="GV4" s="14"/>
+      <c r="GW4" s="14"/>
+      <c r="GX4" s="14"/>
+      <c r="GY4" s="14"/>
+      <c r="GZ4" s="14"/>
+      <c r="HA4" s="14"/>
+      <c r="HB4" s="14"/>
+      <c r="HC4" s="14"/>
+      <c r="HD4" s="14"/>
+      <c r="HE4" s="14"/>
+      <c r="HF4" s="14"/>
+      <c r="HG4" s="14"/>
+      <c r="HH4" s="14"/>
+      <c r="HI4" s="14"/>
+      <c r="HJ4" s="14"/>
+      <c r="HK4" s="14"/>
+      <c r="HL4" s="14"/>
+      <c r="HM4" s="14"/>
+      <c r="HN4" s="14"/>
+      <c r="HO4" s="14"/>
+      <c r="HP4" s="14"/>
+      <c r="HQ4" s="14"/>
+      <c r="HR4" s="14"/>
+      <c r="HS4" s="14"/>
+      <c r="HT4" s="14"/>
+      <c r="HU4" s="14"/>
+      <c r="HV4" s="14"/>
+      <c r="HW4" s="14"/>
+      <c r="HX4" s="14"/>
+      <c r="HY4" s="14"/>
+      <c r="HZ4" s="14"/>
+      <c r="IA4" s="14"/>
+      <c r="IB4" s="14"/>
+      <c r="IC4" s="14"/>
+      <c r="ID4" s="14"/>
+      <c r="IE4" s="14"/>
+      <c r="IF4" s="14"/>
+      <c r="IG4" s="14"/>
+      <c r="IH4" s="14"/>
+      <c r="II4" s="14"/>
+      <c r="IJ4" s="14"/>
+      <c r="IK4" s="14"/>
+      <c r="IL4" s="14"/>
+      <c r="IM4" s="14"/>
+      <c r="IN4" s="14"/>
+      <c r="IO4" s="14"/>
+      <c r="IP4" s="14"/>
+      <c r="IQ4" s="14"/>
+      <c r="IR4" s="14"/>
+      <c r="IS4" s="14"/>
+      <c r="IT4" s="14"/>
+      <c r="IU4" s="14"/>
+      <c r="IV4" s="14"/>
+      <c r="IW4" s="14"/>
+      <c r="IX4" s="14"/>
+      <c r="IY4" s="14"/>
+      <c r="IZ4" s="14"/>
+      <c r="JA4" s="14"/>
+      <c r="JB4" s="14"/>
+      <c r="JC4" s="14"/>
+      <c r="JD4" s="14"/>
+      <c r="JE4" s="14"/>
+      <c r="JF4" s="14"/>
+      <c r="JG4" s="14"/>
+      <c r="JH4" s="14"/>
+      <c r="JI4" s="14"/>
+      <c r="JJ4" s="14"/>
+      <c r="JK4" s="14"/>
+      <c r="JL4" s="14"/>
+      <c r="JM4" s="14"/>
+      <c r="JN4" s="14"/>
+      <c r="JO4" s="14"/>
+      <c r="JP4" s="14"/>
+      <c r="JQ4" s="14"/>
+      <c r="JR4" s="14"/>
+      <c r="JS4" s="14"/>
+      <c r="JT4" s="14"/>
+      <c r="JU4" s="14"/>
+      <c r="JV4" s="14"/>
+      <c r="JW4" s="14"/>
+      <c r="JX4" s="14"/>
+      <c r="JY4" s="14"/>
+      <c r="JZ4" s="14"/>
+      <c r="KA4" s="14"/>
+      <c r="KB4" s="14"/>
+      <c r="KC4" s="14"/>
+      <c r="KD4" s="14"/>
+      <c r="KE4" s="14"/>
+      <c r="KF4" s="14"/>
+      <c r="KG4" s="14"/>
+      <c r="KH4" s="14"/>
+      <c r="KI4" s="14"/>
+      <c r="KJ4" s="14"/>
+      <c r="KK4" s="14"/>
+      <c r="KL4" s="14"/>
+      <c r="KM4" s="14"/>
+      <c r="KN4" s="14"/>
+      <c r="KO4" s="14"/>
+      <c r="KP4" s="14"/>
+      <c r="KQ4" s="14"/>
+      <c r="KR4" s="14"/>
+      <c r="KS4" s="14"/>
+      <c r="KT4" s="14"/>
+      <c r="KU4" s="14"/>
+      <c r="KV4" s="14"/>
+      <c r="KW4" s="14"/>
+      <c r="KX4" s="14"/>
+      <c r="KY4" s="14"/>
+      <c r="KZ4" s="14"/>
+      <c r="LA4" s="14"/>
+      <c r="LB4" s="14"/>
+      <c r="LC4" s="14"/>
+      <c r="LD4" s="14"/>
+      <c r="LE4" s="14"/>
+      <c r="LF4" s="14"/>
+      <c r="LG4" s="14"/>
+      <c r="LH4" s="14"/>
+      <c r="LI4" s="14"/>
+      <c r="LJ4" s="14"/>
+      <c r="LK4" s="14"/>
+      <c r="LL4" s="14"/>
+      <c r="LM4" s="14"/>
+      <c r="LN4" s="14"/>
+      <c r="LO4" s="14"/>
+      <c r="LP4" s="14"/>
+      <c r="LQ4" s="14"/>
+      <c r="LR4" s="14"/>
+      <c r="LS4" s="14"/>
+      <c r="LT4" s="14"/>
+      <c r="LU4" s="14"/>
+      <c r="LV4" s="14"/>
+      <c r="LW4" s="14"/>
+      <c r="LX4" s="14"/>
+      <c r="LY4" s="14"/>
+      <c r="LZ4" s="14"/>
+      <c r="MA4" s="14"/>
+      <c r="MB4" s="14"/>
+      <c r="MC4" s="14"/>
+      <c r="MD4" s="14"/>
+      <c r="ME4" s="14"/>
+      <c r="MF4" s="14"/>
+      <c r="MG4" s="14"/>
+      <c r="MH4" s="14"/>
+      <c r="MI4" s="14"/>
+      <c r="MJ4" s="14"/>
+      <c r="MK4" s="14"/>
+      <c r="ML4" s="14"/>
+      <c r="MM4" s="14"/>
+      <c r="MN4" s="14"/>
+      <c r="MO4" s="14"/>
+      <c r="MP4" s="14"/>
+      <c r="MQ4" s="14"/>
+      <c r="MR4" s="14"/>
+      <c r="MS4" s="14"/>
+      <c r="MT4" s="14"/>
+      <c r="MU4" s="14"/>
+      <c r="MV4" s="14"/>
+      <c r="MW4" s="14"/>
+      <c r="MX4" s="14"/>
+      <c r="MY4" s="14"/>
+      <c r="MZ4" s="14"/>
+      <c r="NA4" s="14"/>
+      <c r="NB4" s="14"/>
+      <c r="NC4" s="14"/>
+      <c r="ND4" s="14"/>
+      <c r="NE4" s="14"/>
+      <c r="NF4" s="14"/>
+      <c r="NG4" s="14"/>
+      <c r="NH4" s="14"/>
+      <c r="NI4" s="14"/>
+      <c r="NJ4" s="14"/>
+      <c r="NK4" s="14"/>
+      <c r="NL4" s="14"/>
+      <c r="NM4" s="14"/>
+      <c r="NN4" s="14"/>
+      <c r="NO4" s="14"/>
+      <c r="NP4" s="14"/>
+      <c r="NQ4" s="14"/>
+      <c r="NR4" s="14"/>
+      <c r="NS4" s="14"/>
+      <c r="NT4" s="14"/>
+      <c r="NU4" s="14"/>
+      <c r="NV4" s="14"/>
+      <c r="NW4" s="14"/>
+      <c r="NX4" s="14"/>
+      <c r="NY4" s="14"/>
+      <c r="NZ4" s="14"/>
+      <c r="OA4" s="14"/>
+      <c r="OB4" s="14"/>
+      <c r="OC4" s="14"/>
+      <c r="OD4" s="14"/>
+      <c r="OE4" s="14"/>
+      <c r="OF4" s="14"/>
+      <c r="OG4" s="14"/>
+      <c r="OH4" s="14"/>
+      <c r="OI4" s="14"/>
+      <c r="OJ4" s="14"/>
+      <c r="OK4" s="14"/>
+      <c r="OL4" s="14"/>
+      <c r="OM4" s="14"/>
+      <c r="ON4" s="14"/>
+      <c r="OO4" s="14"/>
+      <c r="OP4" s="14"/>
+      <c r="OQ4" s="14"/>
+      <c r="OR4" s="14"/>
+      <c r="OS4" s="14"/>
+      <c r="OT4" s="14"/>
+      <c r="OU4" s="14"/>
+      <c r="OV4" s="14"/>
+      <c r="OW4" s="14"/>
+      <c r="OX4" s="14"/>
+      <c r="OY4" s="14"/>
+      <c r="OZ4" s="14"/>
+      <c r="PA4" s="14"/>
+      <c r="PB4" s="14"/>
+      <c r="PC4" s="14"/>
+      <c r="PD4" s="14"/>
+      <c r="PE4" s="14"/>
+      <c r="PF4" s="14"/>
+      <c r="PG4" s="14"/>
+      <c r="PH4" s="14"/>
+      <c r="PI4" s="14"/>
+      <c r="PJ4" s="14"/>
+      <c r="PK4" s="14"/>
+      <c r="PL4" s="14"/>
+      <c r="PM4" s="14"/>
+      <c r="PN4" s="14"/>
+      <c r="PO4" s="14"/>
+      <c r="PP4" s="14"/>
+      <c r="PQ4" s="14"/>
+      <c r="PR4" s="14"/>
+      <c r="PS4" s="14"/>
+      <c r="PT4" s="14"/>
+      <c r="PU4" s="14"/>
+      <c r="PV4" s="14"/>
+      <c r="PW4" s="14"/>
+      <c r="PX4" s="14"/>
+      <c r="PY4" s="14"/>
+      <c r="PZ4" s="14"/>
+      <c r="QA4" s="14"/>
+      <c r="QB4" s="14"/>
+      <c r="QC4" s="14"/>
+      <c r="QD4" s="14"/>
+      <c r="QE4" s="14"/>
+      <c r="QF4" s="14"/>
+      <c r="QG4" s="14"/>
+      <c r="QH4" s="14"/>
+      <c r="QI4" s="14"/>
+      <c r="QJ4" s="14"/>
+      <c r="QK4" s="14"/>
+      <c r="QL4" s="14"/>
+      <c r="QM4" s="14"/>
+      <c r="QN4" s="14"/>
+      <c r="QO4" s="14"/>
+      <c r="QP4" s="14"/>
+      <c r="QQ4" s="14"/>
+      <c r="QR4" s="14"/>
+      <c r="QS4" s="14"/>
+      <c r="QT4" s="14"/>
+      <c r="QU4" s="14"/>
+      <c r="QV4" s="14"/>
+      <c r="QW4" s="14"/>
+      <c r="QX4" s="14"/>
+      <c r="QY4" s="14"/>
+      <c r="QZ4" s="14"/>
+      <c r="RA4" s="14"/>
+      <c r="RB4" s="14"/>
+      <c r="RC4" s="14"/>
+      <c r="RD4" s="14"/>
+      <c r="RE4" s="14"/>
+      <c r="RF4" s="14"/>
+      <c r="RG4" s="14"/>
+      <c r="RH4" s="14"/>
+      <c r="RI4" s="14"/>
+      <c r="RJ4" s="14"/>
+      <c r="RK4" s="14"/>
+      <c r="RL4" s="14"/>
+      <c r="RM4" s="14"/>
+      <c r="RN4" s="14"/>
+      <c r="RO4" s="14"/>
+      <c r="RP4" s="14"/>
+      <c r="RQ4" s="14"/>
+      <c r="RR4" s="14"/>
+      <c r="RS4" s="14"/>
+      <c r="RT4" s="14"/>
+      <c r="RU4" s="14"/>
+      <c r="RV4" s="14"/>
+      <c r="RW4" s="14"/>
+      <c r="RX4" s="14"/>
+      <c r="RY4" s="14"/>
+      <c r="RZ4" s="14"/>
+      <c r="SA4" s="14"/>
+      <c r="SB4" s="14"/>
+      <c r="SC4" s="14"/>
+      <c r="SD4" s="14"/>
+      <c r="SE4" s="14"/>
+      <c r="SF4" s="14"/>
+    </row>
+    <row r="5" spans="1:500" ht="36">
+      <c r="A5" s="15" t="s">
         <v>80</v>
       </c>
+      <c r="B5" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="E5" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="14"/>
+      <c r="K5" s="14"/>
+      <c r="L5" s="14"/>
+      <c r="M5" s="14"/>
+      <c r="N5" s="14"/>
+      <c r="O5" s="14"/>
+      <c r="P5" s="14"/>
+      <c r="Q5" s="14"/>
+      <c r="R5" s="14"/>
+      <c r="S5" s="14"/>
+      <c r="T5" s="14"/>
+      <c r="U5" s="14"/>
+      <c r="V5" s="14"/>
+      <c r="W5" s="14"/>
+      <c r="X5" s="14"/>
+      <c r="Y5" s="14"/>
+      <c r="Z5" s="14"/>
+      <c r="AA5" s="14"/>
+      <c r="AB5" s="14"/>
+      <c r="AC5" s="14"/>
+      <c r="AD5" s="14"/>
+      <c r="AE5" s="14"/>
+      <c r="AF5" s="14"/>
+      <c r="AG5" s="14"/>
+      <c r="AH5" s="14"/>
+      <c r="AI5" s="14"/>
+      <c r="AJ5" s="14"/>
+      <c r="AK5" s="14"/>
+      <c r="AL5" s="14"/>
+      <c r="AM5" s="14"/>
+      <c r="AN5" s="14"/>
+      <c r="AO5" s="14"/>
+      <c r="AP5" s="14"/>
+      <c r="AQ5" s="14"/>
+      <c r="AR5" s="14"/>
+      <c r="AS5" s="14"/>
+      <c r="AT5" s="14"/>
+      <c r="AU5" s="14"/>
+      <c r="AV5" s="14"/>
+      <c r="AW5" s="14"/>
+      <c r="AX5" s="14"/>
+      <c r="AY5" s="14"/>
+      <c r="AZ5" s="14"/>
+      <c r="BA5" s="14"/>
+      <c r="BB5" s="14"/>
+      <c r="BC5" s="14"/>
+      <c r="BD5" s="14"/>
+      <c r="BE5" s="14"/>
+      <c r="BF5" s="14"/>
+      <c r="BG5" s="14"/>
+      <c r="BH5" s="14"/>
+      <c r="BI5" s="14"/>
+      <c r="BJ5" s="14"/>
+      <c r="BK5" s="14"/>
+      <c r="BL5" s="14"/>
+      <c r="BM5" s="14"/>
+      <c r="BN5" s="14"/>
+      <c r="BO5" s="14"/>
+      <c r="BP5" s="14"/>
+      <c r="BQ5" s="14"/>
+      <c r="BR5" s="14"/>
+      <c r="BS5" s="14"/>
+      <c r="BT5" s="14"/>
+      <c r="BU5" s="14"/>
+      <c r="BV5" s="14"/>
+      <c r="BW5" s="14"/>
+      <c r="BX5" s="14"/>
+      <c r="BY5" s="14"/>
+      <c r="BZ5" s="14"/>
+      <c r="CA5" s="14"/>
+      <c r="CB5" s="14"/>
+      <c r="CC5" s="14"/>
+      <c r="CD5" s="14"/>
+      <c r="CE5" s="14"/>
+      <c r="CF5" s="14"/>
+      <c r="CG5" s="14"/>
+      <c r="CH5" s="14"/>
+      <c r="CI5" s="14"/>
+      <c r="CJ5" s="14"/>
+      <c r="CK5" s="14"/>
+      <c r="CL5" s="14"/>
+      <c r="CM5" s="14"/>
+      <c r="CN5" s="14"/>
+      <c r="CO5" s="14"/>
+      <c r="CP5" s="14"/>
+      <c r="CQ5" s="14"/>
+      <c r="CR5" s="14"/>
+      <c r="CS5" s="14"/>
+      <c r="CT5" s="14"/>
+      <c r="CU5" s="14"/>
+      <c r="CV5" s="14"/>
+      <c r="CW5" s="14"/>
+      <c r="CX5" s="14"/>
+      <c r="CY5" s="14"/>
+      <c r="CZ5" s="14"/>
+      <c r="DA5" s="14"/>
+      <c r="DB5" s="14"/>
+      <c r="DC5" s="14"/>
+      <c r="DD5" s="14"/>
+      <c r="DE5" s="14"/>
+      <c r="DF5" s="14"/>
+      <c r="DG5" s="14"/>
+      <c r="DH5" s="14"/>
+      <c r="DI5" s="14"/>
+      <c r="DJ5" s="14"/>
+      <c r="DK5" s="14"/>
+      <c r="DL5" s="14"/>
+      <c r="DM5" s="14"/>
+      <c r="DN5" s="14"/>
+      <c r="DO5" s="14"/>
+      <c r="DP5" s="14"/>
+      <c r="DQ5" s="14"/>
+      <c r="DR5" s="14"/>
+      <c r="DS5" s="14"/>
+      <c r="DT5" s="14"/>
+      <c r="DU5" s="14"/>
+      <c r="DV5" s="14"/>
+      <c r="DW5" s="14"/>
+      <c r="DX5" s="14"/>
+      <c r="DY5" s="14"/>
+      <c r="DZ5" s="14"/>
+      <c r="EA5" s="14"/>
+      <c r="EB5" s="14"/>
+      <c r="EC5" s="14"/>
+      <c r="ED5" s="14"/>
+      <c r="EE5" s="14"/>
+      <c r="EF5" s="14"/>
+      <c r="EG5" s="14"/>
+      <c r="EH5" s="14"/>
+      <c r="EI5" s="14"/>
+      <c r="EJ5" s="14"/>
+      <c r="EK5" s="14"/>
+      <c r="EL5" s="14"/>
+      <c r="EM5" s="14"/>
+      <c r="EN5" s="14"/>
+      <c r="EO5" s="14"/>
+      <c r="EP5" s="14"/>
+      <c r="EQ5" s="14"/>
+      <c r="ER5" s="14"/>
+      <c r="ES5" s="14"/>
+      <c r="ET5" s="14"/>
+      <c r="EU5" s="14"/>
+      <c r="EV5" s="14"/>
+      <c r="EW5" s="14"/>
+      <c r="EX5" s="14"/>
+      <c r="EY5" s="14"/>
+      <c r="EZ5" s="14"/>
+      <c r="FA5" s="14"/>
+      <c r="FB5" s="14"/>
+      <c r="FC5" s="14"/>
+      <c r="FD5" s="14"/>
+      <c r="FE5" s="14"/>
+      <c r="FF5" s="14"/>
+      <c r="FG5" s="14"/>
+      <c r="FH5" s="14"/>
+      <c r="FI5" s="14"/>
+      <c r="FJ5" s="14"/>
+      <c r="FK5" s="14"/>
+      <c r="FL5" s="14"/>
+      <c r="FM5" s="14"/>
+      <c r="FN5" s="14"/>
+      <c r="FO5" s="14"/>
+      <c r="FP5" s="14"/>
+      <c r="FQ5" s="14"/>
+      <c r="FR5" s="14"/>
+      <c r="FS5" s="14"/>
+      <c r="FT5" s="14"/>
+      <c r="FU5" s="14"/>
+      <c r="FV5" s="14"/>
+      <c r="FW5" s="14"/>
+      <c r="FX5" s="14"/>
+      <c r="FY5" s="14"/>
+      <c r="FZ5" s="14"/>
+      <c r="GA5" s="14"/>
+      <c r="GB5" s="14"/>
+      <c r="GC5" s="14"/>
+      <c r="GD5" s="14"/>
+      <c r="GE5" s="14"/>
+      <c r="GF5" s="14"/>
+      <c r="GG5" s="14"/>
+      <c r="GH5" s="14"/>
+      <c r="GI5" s="14"/>
+      <c r="GJ5" s="14"/>
+      <c r="GK5" s="14"/>
+      <c r="GL5" s="14"/>
+      <c r="GM5" s="14"/>
+      <c r="GN5" s="14"/>
+      <c r="GO5" s="14"/>
+      <c r="GP5" s="14"/>
+      <c r="GQ5" s="14"/>
+      <c r="GR5" s="14"/>
+      <c r="GS5" s="14"/>
+      <c r="GT5" s="14"/>
+      <c r="GU5" s="14"/>
+      <c r="GV5" s="14"/>
+      <c r="GW5" s="14"/>
+      <c r="GX5" s="14"/>
+      <c r="GY5" s="14"/>
+      <c r="GZ5" s="14"/>
+      <c r="HA5" s="14"/>
+      <c r="HB5" s="14"/>
+      <c r="HC5" s="14"/>
+      <c r="HD5" s="14"/>
+      <c r="HE5" s="14"/>
+      <c r="HF5" s="14"/>
+      <c r="HG5" s="14"/>
+      <c r="HH5" s="14"/>
+      <c r="HI5" s="14"/>
+      <c r="HJ5" s="14"/>
+      <c r="HK5" s="14"/>
+      <c r="HL5" s="14"/>
+      <c r="HM5" s="14"/>
+      <c r="HN5" s="14"/>
+      <c r="HO5" s="14"/>
+      <c r="HP5" s="14"/>
+      <c r="HQ5" s="14"/>
+      <c r="HR5" s="14"/>
+      <c r="HS5" s="14"/>
+      <c r="HT5" s="14"/>
+      <c r="HU5" s="14"/>
+      <c r="HV5" s="14"/>
+      <c r="HW5" s="14"/>
+      <c r="HX5" s="14"/>
+      <c r="HY5" s="14"/>
+      <c r="HZ5" s="14"/>
+      <c r="IA5" s="14"/>
+      <c r="IB5" s="14"/>
+      <c r="IC5" s="14"/>
+      <c r="ID5" s="14"/>
+      <c r="IE5" s="14"/>
+      <c r="IF5" s="14"/>
+      <c r="IG5" s="14"/>
+      <c r="IH5" s="14"/>
+      <c r="II5" s="14"/>
+      <c r="IJ5" s="14"/>
+      <c r="IK5" s="14"/>
+      <c r="IL5" s="14"/>
+      <c r="IM5" s="14"/>
+      <c r="IN5" s="14"/>
+      <c r="IO5" s="14"/>
+      <c r="IP5" s="14"/>
+      <c r="IQ5" s="14"/>
+      <c r="IR5" s="14"/>
+      <c r="IS5" s="14"/>
+      <c r="IT5" s="14"/>
+      <c r="IU5" s="14"/>
+      <c r="IV5" s="14"/>
+      <c r="IW5" s="14"/>
+      <c r="IX5" s="14"/>
+      <c r="IY5" s="14"/>
+      <c r="IZ5" s="14"/>
+      <c r="JA5" s="14"/>
+      <c r="JB5" s="14"/>
+      <c r="JC5" s="14"/>
+      <c r="JD5" s="14"/>
+      <c r="JE5" s="14"/>
+      <c r="JF5" s="14"/>
+      <c r="JG5" s="14"/>
+      <c r="JH5" s="14"/>
+      <c r="JI5" s="14"/>
+      <c r="JJ5" s="14"/>
+      <c r="JK5" s="14"/>
+      <c r="JL5" s="14"/>
+      <c r="JM5" s="14"/>
+      <c r="JN5" s="14"/>
+      <c r="JO5" s="14"/>
+      <c r="JP5" s="14"/>
+      <c r="JQ5" s="14"/>
+      <c r="JR5" s="14"/>
+      <c r="JS5" s="14"/>
+      <c r="JT5" s="14"/>
+      <c r="JU5" s="14"/>
+      <c r="JV5" s="14"/>
+      <c r="JW5" s="14"/>
+      <c r="JX5" s="14"/>
+      <c r="JY5" s="14"/>
+      <c r="JZ5" s="14"/>
+      <c r="KA5" s="14"/>
+      <c r="KB5" s="14"/>
+      <c r="KC5" s="14"/>
+      <c r="KD5" s="14"/>
+      <c r="KE5" s="14"/>
+      <c r="KF5" s="14"/>
+      <c r="KG5" s="14"/>
+      <c r="KH5" s="14"/>
+      <c r="KI5" s="14"/>
+      <c r="KJ5" s="14"/>
+      <c r="KK5" s="14"/>
+      <c r="KL5" s="14"/>
+      <c r="KM5" s="14"/>
+      <c r="KN5" s="14"/>
+      <c r="KO5" s="14"/>
+      <c r="KP5" s="14"/>
+      <c r="KQ5" s="14"/>
+      <c r="KR5" s="14"/>
+      <c r="KS5" s="14"/>
+      <c r="KT5" s="14"/>
+      <c r="KU5" s="14"/>
+      <c r="KV5" s="14"/>
+      <c r="KW5" s="14"/>
+      <c r="KX5" s="14"/>
+      <c r="KY5" s="14"/>
+      <c r="KZ5" s="14"/>
+      <c r="LA5" s="14"/>
+      <c r="LB5" s="14"/>
+      <c r="LC5" s="14"/>
+      <c r="LD5" s="14"/>
+      <c r="LE5" s="14"/>
+      <c r="LF5" s="14"/>
+      <c r="LG5" s="14"/>
+      <c r="LH5" s="14"/>
+      <c r="LI5" s="14"/>
+      <c r="LJ5" s="14"/>
+      <c r="LK5" s="14"/>
+      <c r="LL5" s="14"/>
+      <c r="LM5" s="14"/>
+      <c r="LN5" s="14"/>
+      <c r="LO5" s="14"/>
+      <c r="LP5" s="14"/>
+      <c r="LQ5" s="14"/>
+      <c r="LR5" s="14"/>
+      <c r="LS5" s="14"/>
+      <c r="LT5" s="14"/>
+      <c r="LU5" s="14"/>
+      <c r="LV5" s="14"/>
+      <c r="LW5" s="14"/>
+      <c r="LX5" s="14"/>
+      <c r="LY5" s="14"/>
+      <c r="LZ5" s="14"/>
+      <c r="MA5" s="14"/>
+      <c r="MB5" s="14"/>
+      <c r="MC5" s="14"/>
+      <c r="MD5" s="14"/>
+      <c r="ME5" s="14"/>
+      <c r="MF5" s="14"/>
+      <c r="MG5" s="14"/>
+      <c r="MH5" s="14"/>
+      <c r="MI5" s="14"/>
+      <c r="MJ5" s="14"/>
+      <c r="MK5" s="14"/>
+      <c r="ML5" s="14"/>
+      <c r="MM5" s="14"/>
+      <c r="MN5" s="14"/>
+      <c r="MO5" s="14"/>
+      <c r="MP5" s="14"/>
+      <c r="MQ5" s="14"/>
+      <c r="MR5" s="14"/>
+      <c r="MS5" s="14"/>
+      <c r="MT5" s="14"/>
+      <c r="MU5" s="14"/>
+      <c r="MV5" s="14"/>
+      <c r="MW5" s="14"/>
+      <c r="MX5" s="14"/>
+      <c r="MY5" s="14"/>
+      <c r="MZ5" s="14"/>
+      <c r="NA5" s="14"/>
+      <c r="NB5" s="14"/>
+      <c r="NC5" s="14"/>
+      <c r="ND5" s="14"/>
+      <c r="NE5" s="14"/>
+      <c r="NF5" s="14"/>
+      <c r="NG5" s="14"/>
+      <c r="NH5" s="14"/>
+      <c r="NI5" s="14"/>
+      <c r="NJ5" s="14"/>
+      <c r="NK5" s="14"/>
+      <c r="NL5" s="14"/>
+      <c r="NM5" s="14"/>
+      <c r="NN5" s="14"/>
+      <c r="NO5" s="14"/>
+      <c r="NP5" s="14"/>
+      <c r="NQ5" s="14"/>
+      <c r="NR5" s="14"/>
+      <c r="NS5" s="14"/>
+      <c r="NT5" s="14"/>
+      <c r="NU5" s="14"/>
+      <c r="NV5" s="14"/>
+      <c r="NW5" s="14"/>
+      <c r="NX5" s="14"/>
+      <c r="NY5" s="14"/>
+      <c r="NZ5" s="14"/>
+      <c r="OA5" s="14"/>
+      <c r="OB5" s="14"/>
+      <c r="OC5" s="14"/>
+      <c r="OD5" s="14"/>
+      <c r="OE5" s="14"/>
+      <c r="OF5" s="14"/>
+      <c r="OG5" s="14"/>
+      <c r="OH5" s="14"/>
+      <c r="OI5" s="14"/>
+      <c r="OJ5" s="14"/>
+      <c r="OK5" s="14"/>
+      <c r="OL5" s="14"/>
+      <c r="OM5" s="14"/>
+      <c r="ON5" s="14"/>
+      <c r="OO5" s="14"/>
+      <c r="OP5" s="14"/>
+      <c r="OQ5" s="14"/>
+      <c r="OR5" s="14"/>
+      <c r="OS5" s="14"/>
+      <c r="OT5" s="14"/>
+      <c r="OU5" s="14"/>
+      <c r="OV5" s="14"/>
+      <c r="OW5" s="14"/>
+      <c r="OX5" s="14"/>
+      <c r="OY5" s="14"/>
+      <c r="OZ5" s="14"/>
+      <c r="PA5" s="14"/>
+      <c r="PB5" s="14"/>
+      <c r="PC5" s="14"/>
+      <c r="PD5" s="14"/>
+      <c r="PE5" s="14"/>
+      <c r="PF5" s="14"/>
+      <c r="PG5" s="14"/>
+      <c r="PH5" s="14"/>
+      <c r="PI5" s="14"/>
+      <c r="PJ5" s="14"/>
+      <c r="PK5" s="14"/>
+      <c r="PL5" s="14"/>
+      <c r="PM5" s="14"/>
+      <c r="PN5" s="14"/>
+      <c r="PO5" s="14"/>
+      <c r="PP5" s="14"/>
+      <c r="PQ5" s="14"/>
+      <c r="PR5" s="14"/>
+      <c r="PS5" s="14"/>
+      <c r="PT5" s="14"/>
+      <c r="PU5" s="14"/>
+      <c r="PV5" s="14"/>
+      <c r="PW5" s="14"/>
+      <c r="PX5" s="14"/>
+      <c r="PY5" s="14"/>
+      <c r="PZ5" s="14"/>
+      <c r="QA5" s="14"/>
+      <c r="QB5" s="14"/>
+      <c r="QC5" s="14"/>
+      <c r="QD5" s="14"/>
+      <c r="QE5" s="14"/>
+      <c r="QF5" s="14"/>
+      <c r="QG5" s="14"/>
+      <c r="QH5" s="14"/>
+      <c r="QI5" s="14"/>
+      <c r="QJ5" s="14"/>
+      <c r="QK5" s="14"/>
+      <c r="QL5" s="14"/>
+      <c r="QM5" s="14"/>
+      <c r="QN5" s="14"/>
+      <c r="QO5" s="14"/>
+      <c r="QP5" s="14"/>
+      <c r="QQ5" s="14"/>
+      <c r="QR5" s="14"/>
+      <c r="QS5" s="14"/>
+      <c r="QT5" s="14"/>
+      <c r="QU5" s="14"/>
+      <c r="QV5" s="14"/>
+      <c r="QW5" s="14"/>
+      <c r="QX5" s="14"/>
+      <c r="QY5" s="14"/>
+      <c r="QZ5" s="14"/>
+      <c r="RA5" s="14"/>
+      <c r="RB5" s="14"/>
+      <c r="RC5" s="14"/>
+      <c r="RD5" s="14"/>
+      <c r="RE5" s="14"/>
+      <c r="RF5" s="14"/>
+      <c r="RG5" s="14"/>
+      <c r="RH5" s="14"/>
+      <c r="RI5" s="14"/>
+      <c r="RJ5" s="14"/>
+      <c r="RK5" s="14"/>
+      <c r="RL5" s="14"/>
+      <c r="RM5" s="14"/>
+      <c r="RN5" s="14"/>
+      <c r="RO5" s="14"/>
+      <c r="RP5" s="14"/>
+      <c r="RQ5" s="14"/>
+      <c r="RR5" s="14"/>
+      <c r="RS5" s="14"/>
+      <c r="RT5" s="14"/>
+      <c r="RU5" s="14"/>
+      <c r="RV5" s="14"/>
+      <c r="RW5" s="14"/>
+      <c r="RX5" s="14"/>
+      <c r="RY5" s="14"/>
+      <c r="RZ5" s="14"/>
+      <c r="SA5" s="14"/>
+      <c r="SB5" s="14"/>
+      <c r="SC5" s="14"/>
+      <c r="SD5" s="14"/>
+      <c r="SE5" s="14"/>
+      <c r="SF5" s="14"/>
     </row>
     <row r="65" spans="13:16">
       <c r="M65" s="1" t="s">

</xml_diff>

<commit_message>
Recently updated test cases
test-case file.xlsx
</commit_message>
<xml_diff>
--- a/Test-Case file.xlsx
+++ b/Test-Case file.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30602"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8CBDC179-EC9C-4F01-A09C-6113236CD700}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{73D2279A-FB4B-4474-9B56-7FA582018E60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="shubh" sheetId="1" r:id="rId1"/>
-    <sheet name="saksham singh" sheetId="2" r:id="rId2"/>
+    <sheet name="saksham singh" sheetId="2" r:id="rId1"/>
+    <sheet name="shubh " sheetId="1" r:id="rId2"/>
     <sheet name="saksham koutsa" sheetId="3" r:id="rId3"/>
     <sheet name="samridhi pattel" sheetId="4" r:id="rId4"/>
   </sheets>
@@ -37,7 +37,163 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="157">
+  <si>
+    <t>functionality</t>
+  </si>
+  <si>
+    <t>test case</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>test steps</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Login API</t>
+  </si>
+  <si>
+    <t>POST /api/auth/login returns token</t>
+  </si>
+  <si>
+    <t>Valid credentials return a 200 response with a session token.</t>
+  </si>
+  <si>
+    <t>1. Send POST /api/auth/login with valid credentials.
+2. Confirm status 200.
+3. Confirm the response contains a sessionToken.</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>Register API</t>
+  </si>
+  <si>
+    <t>POST /api/auth/register creates a user</t>
+  </si>
+  <si>
+    <t>A new user is created and stored in the database.</t>
+  </si>
+  <si>
+    <t>1. Send POST /api/auth/register with new user data._x000D_
+2. Confirm status 200._x000D_
+3. Confirm the user now exists in the database.</t>
+  </si>
+  <si>
+    <t>Remote Session</t>
+  </si>
+  <si>
+    <t>Create and validate session code</t>
+  </si>
+  <si>
+    <t>Remote sender and receiver connect using a session code.</t>
+  </si>
+  <si>
+    <t>1. Create a remote session and note the code._x000D_
+2. Validate the code._x000D_
+3. Confirm the session is active.</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Emergency SOS API</t>
+  </si>
+  <si>
+    <t>POST /api/emergency/sos records alert</t>
+  </si>
+  <si>
+    <t>An SOS submission is accepted and stored.</t>
+  </si>
+  <si>
+    <t>1. POST an SOS payload._x000D_
+2. Confirm status 200._x000D_
+3. Confirm the alert is stored/logged.</t>
+  </si>
+  <si>
+    <t>Password Matching</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify password matching error during registration
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Registration form validates that password and confirmation password match before submitting.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to the frontend registration page.
+2. Enter valid name, email, and password.
+3. Enter a mismatched confirmation password.
+4. Click the register button.
+5. Confirm "Passwords do not match." error is displayed.
+</t>
+  </si>
+  <si>
+    <t>pass</t>
+  </si>
+  <si>
+    <t>Active test highlight</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify active tab is highlighted when clicked
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clicking on a navigation tab updates its styling to indicate it is the active tab.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to the application homepage.
+2. Click on the 'Sign' tab.
+3. Confirm the tab's CSS class is updated to include the active highlight color (e.g., 'indigo').
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">backend API testing </t>
+  </si>
+  <si>
+    <t xml:space="preserve">GET /api/quick-phrases returns quick phrases list
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The quick phrases API endpoint successfully returns a valid JSON array containing phrase labels.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to the API endpoint http://localhost:3000/api/quick-phrases.
+2. Wait for the page response to load.
+3. Extract the body text from the page.
+4. Confirm the response contains a JSON array format (e.g., "[") and the key "label".
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pass
+</t>
+  </si>
+  <si>
+    <t>unauthenticaed user testing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unauthenticated user is redirected to login
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A user attempting to access the /dashboard route without an active session is automatically redirected to the /login page.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate directly to http://localhost:3000/dashboard.
+2. Wait for the application to evaluate authentication status.
+3. Confirm the URL updates to contain /login.
+4. Confirm the login form is displayed on the screen.
+</t>
+  </si>
   <si>
     <t>Functionality</t>
   </si>
@@ -105,83 +261,6 @@
 2. Confirm the buffer commits sooner than on 'Slow (2.5s)'.</t>
   </si>
   <si>
-    <t>functionality</t>
-  </si>
-  <si>
-    <t>test case</t>
-  </si>
-  <si>
-    <t>description</t>
-  </si>
-  <si>
-    <t>test steps</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Login API</t>
-  </si>
-  <si>
-    <t>POST /api/auth/login returns token</t>
-  </si>
-  <si>
-    <t>Valid credentials return a 200 response with a session token.</t>
-  </si>
-  <si>
-    <t>1. Send POST /api/auth/login with valid credentials.
-2. Confirm status 200.
-3. Confirm the response contains a sessionToken.</t>
-  </si>
-  <si>
-    <t>Fail</t>
-  </si>
-  <si>
-    <t>Register API</t>
-  </si>
-  <si>
-    <t>POST /api/auth/register creates a user</t>
-  </si>
-  <si>
-    <t>A new user is created and stored in the database.</t>
-  </si>
-  <si>
-    <t>1. Send POST /api/auth/register with new user data._x000D_
-2. Confirm status 200._x000D_
-3. Confirm the user now exists in the database.</t>
-  </si>
-  <si>
-    <t>Remote Session</t>
-  </si>
-  <si>
-    <t>Create and validate session code</t>
-  </si>
-  <si>
-    <t>Remote sender and receiver connect using a session code.</t>
-  </si>
-  <si>
-    <t>1. Create a remote session and note the code._x000D_
-2. Validate the code._x000D_
-3. Confirm the session is active.</t>
-  </si>
-  <si>
-    <t>Pass</t>
-  </si>
-  <si>
-    <t>Emergency SOS API</t>
-  </si>
-  <si>
-    <t>POST /api/emergency/sos records alert</t>
-  </si>
-  <si>
-    <t>An SOS submission is accepted and stored.</t>
-  </si>
-  <si>
-    <t>1. POST an SOS payload._x000D_
-2. Confirm status 200._x000D_
-3. Confirm the alert is stored/logged.</t>
-  </si>
-  <si>
     <t>status</t>
   </si>
   <si>
@@ -194,14 +273,11 @@
     <t>A detected hand shows the landmark skeleton on the camera feed.</t>
   </si>
   <si>
-    <t>1. Open the Sign tab and enable the webcam._x000D_
-2. Show your hand to the camera._x000D_
+    <t>1. Open the Sign tab and enable the webcam.
+2. Show your hand to the camera.
 3. Confirm the skeleton overlay is drawn on the hand.</t>
   </si>
   <si>
-    <t>pass</t>
-  </si>
-  <si>
     <t>Gesture Recognition</t>
   </si>
   <si>
@@ -211,7 +287,7 @@
     <t>A flat open palm is classified as the HELLO gesture.</t>
   </si>
   <si>
-    <t>1. Show a flat open palm to the camera._x000D_
+    <t>1. Show a flat open palm to the camera.
 2. Confirm 'HELLO' is shown as the current gesture.</t>
   </si>
   <si>
@@ -224,43 +300,186 @@
     <t>Extended fingers light up in the live finger readout.</t>
   </si>
   <si>
-    <t>1. Extend only the index finger._x000D_
+    <t>1. Extend only the index finger.
 2. Confirm only the 'Index' pill is lit and the others are off.</t>
   </si>
   <si>
-    <t>Open hand recognized as YES</t>
-  </si>
-  <si>
-    <t>A  closed front palm is classified as the YES gesture.</t>
+    <t>Closed fist recognized as YES</t>
+  </si>
+  <si>
+    <t>A closed front palm / fist is classified as the YES gesture.</t>
   </si>
   <si>
     <t>1. Show a closed front palm to the camera.
 2. Confirm 'YES' is shown as the current gesture.</t>
   </si>
   <si>
-    <t>Open hand recognized as HELP</t>
-  </si>
-  <si>
-    <t>A  closed front palm with open/straight thumb and pinky finger
- is classified as the SLEEP gesture.</t>
+    <t>Hand sign recognized as HELP</t>
+  </si>
+  <si>
+    <t>A closed fist with thumb upright over the base palm is classified as the HELP gesture.</t>
   </si>
   <si>
     <t>1. Show a HELP gesture hand sign.
 2. Confirm 'HELP' is shown as the current gesture.</t>
   </si>
   <si>
-    <t>Open hand recognized as FOOD</t>
-  </si>
-  <si>
-    <t>A  closed front palm with open/straight thumb and pinky finger
- is classified as the FOOD gesture.</t>
+    <t>Hand sign recognized as FOOD</t>
+  </si>
+  <si>
+    <t>Curved fingers brought towards the mouth forming a cup shape is classified as the FOOD gesture.</t>
   </si>
   <si>
     <t>1. Show a FOOD gesture hand sign.
 2. Confirm 'FOOD' is shown as the current gesture.</t>
   </si>
   <si>
-    <t>fail</t>
+    <t>Snapping index and thumb recognized as NO</t>
+  </si>
+  <si>
+    <t>Index and middle fingers extended and snapping against the thumb is classified as the NO gesture.</t>
+  </si>
+  <si>
+    <t>1. Show a NO gesture hand sign to the camera.
+2. Confirm 'NO' is shown as the current gesture.</t>
+  </si>
+  <si>
+    <t>Flat hand from chin recognized as THANK YOU</t>
+  </si>
+  <si>
+    <t>Flat hand touching fingers to chin and moving forward is classified as the THANK YOU gesture.</t>
+  </si>
+  <si>
+    <t>1. Show a THANK YOU gesture hand sign.
+2. Confirm 'THANK YOU' is shown as the current gesture.</t>
+  </si>
+  <si>
+    <t>Sentence Construction</t>
+  </si>
+  <si>
+    <t>Multi-gesture concatenation in phrase buffer</t>
+  </si>
+  <si>
+    <t>Sequentially detected gestures are appended into a complete sentence separated by spaces.</t>
+  </si>
+  <si>
+    <t>1. Perform 'HELLO' gesture.
+2. Perform 'HELP' gesture.
+3. Perform 'NEED WATER' gesture.
+4. Confirm phrase buffer displays 'HELLO HELP NEED WATER'.</t>
+  </si>
+  <si>
+    <t>Phrase Buffer Control</t>
+  </si>
+  <si>
+    <t>Delete Word removes last appended gesture</t>
+  </si>
+  <si>
+    <t>Clicking 'Delete Word' removes only the last word/gesture without clearing the entire sentence.</t>
+  </si>
+  <si>
+    <t>1. Construct a multi-word phrase (e.g., 'HELLO HELP').
+2. Click the 'Delete Word' button.
+3. Confirm 'HELP' is deleted and 'HELLO' remains.</t>
+  </si>
+  <si>
+    <t>Clear All completely resets constructed phrase</t>
+  </si>
+  <si>
+    <t>Clicking 'Clear All' clears all accumulated words from the phrase buffer.</t>
+  </si>
+  <si>
+    <t>1. Add gestures to the phrase buffer.
+2. Click the 'Clear All' button.
+3. Confirm buffer is cleared back to placeholder state.</t>
+  </si>
+  <si>
+    <t>Visual Overlay</t>
+  </si>
+  <si>
+    <t>Toggle landmark skeleton overlay visibility</t>
+  </si>
+  <si>
+    <t>Toggling the 'Show Skeleton Overlay' checkbox enables or disables the landmark visualizer.</t>
+  </si>
+  <si>
+    <t>1. Enable camera feed with skeleton overlay active.
+2. Uncheck 'Show Skeleton Overlay'.
+3. Confirm skeleton lines disappear from video stream.
+4. Check the box again and confirm skeleton reappears.</t>
+  </si>
+  <si>
+    <t>Audio &amp; Speech</t>
+  </si>
+  <si>
+    <t>Adjust speech speed rate and pitch sliders</t>
+  </si>
+  <si>
+    <t>Voice speed rate and pitch sliders dynamically update speech synthesis configuration and readout labels.</t>
+  </si>
+  <si>
+    <t>1. Move Speed Rate slider to 1.5x.
+2. Confirm speed display updates to '1.5x'.
+3. Move Pitch slider to 1.2x.
+4. Confirm pitch display updates to '1.2x'.</t>
+  </si>
+  <si>
+    <t>Hardware Control</t>
+  </si>
+  <si>
+    <t>Toggle Webcam feed start and stop</t>
+  </si>
+  <si>
+    <t>Clicking camera activation button starts or shuts down the live webcam stream.</t>
+  </si>
+  <si>
+    <t>1. Click 'Use Real Webcam' button.
+2. Confirm live camera feed starts.
+3. Click 'Close Camera' button.
+4. Confirm camera stream stops cleanly.</t>
+  </si>
+  <si>
+    <t>Speech Dispatch</t>
+  </si>
+  <si>
+    <t>Submit phrase for speech synthesis playback</t>
+  </si>
+  <si>
+    <t>Clicking 'Submit' plays synthesized audio of the buffer and logs the phrase to history.</t>
+  </si>
+  <si>
+    <t>1. Construct phrase 'HELLO HOW ARE YOU'.
+2. Verify 'Submit' button is enabled.
+3. Click 'Submit'.
+4. Confirm speech audio plays and phrase is logged.</t>
+  </si>
+  <si>
+    <t>Gesture Cheat Sheet</t>
+  </si>
+  <si>
+    <t>Quick select gesture from cheat sheet cards</t>
+  </si>
+  <si>
+    <t>Clicking any gesture card in the cheat sheet triggers simulated recognition and updates HUD metrics.</t>
+  </si>
+  <si>
+    <t>1. Open Hand Sign Gesture cheat sheet.
+2. Click on 'HELLO' card.
+3. Confirm current gesture updates to 'HELLO' and confidence displays 98.5%.</t>
+  </si>
+  <si>
+    <t>Performance HUD</t>
+  </si>
+  <si>
+    <t>Live FPS and Confidence score monitoring</t>
+  </si>
+  <si>
+    <t>Video feed HUD continuously tracks recognition confidence percentage and camera inference FPS.</t>
+  </si>
+  <si>
+    <t>1. Observe the top-right video HUD during active tracking.
+2. Confirm Confidence score percentage is rendered.
+3. Confirm live FPS counter is rendered and updates.</t>
   </si>
   <si>
     <t xml:space="preserve"> </t>
@@ -318,13 +537,61 @@
     <t>1. Open on desktop.
 2. Resize to phone width.
 3. Confirm content reflows with no horizontal scrollbar.</t>
+  </si>
+  <si>
+    <t>Authentication UI</t>
+  </si>
+  <si>
+    <t>Block sign-in when fields are empty</t>
+  </si>
+  <si>
+    <t>The sign-in form shows required-field feedback and stays on the login screen.</t>
+  </si>
+  <si>
+    <t>1. Open the login screen. 2. Leave email and password empty. 3. Select Sign In. 4. Confirm the required-field message appears and no loading state remains.</t>
+  </si>
+  <si>
+    <t>Switch between login and registration screens</t>
+  </si>
+  <si>
+    <t>The screen controls show the selected form and clear prior messages.</t>
+  </si>
+  <si>
+    <t>1. From Login, select the registration link. 2. Confirm registration fields appear. 3. Return to Login. 4. Confirm the login form appears without stale validation messages.</t>
+  </si>
+  <si>
+    <t>Validate email format during registration</t>
+  </si>
+  <si>
+    <t>An invalid email address displays a validation message before the form enters a loading state.</t>
+  </si>
+  <si>
+    <t>1. Open Register. 2. Enter a name, an invalid email such as `patient@`, and the other required fields. 3. Submit the form. 4. Confirm the email validation message appears and the screen remains responsive.</t>
+  </si>
+  <si>
+    <t>Show password strength feedback</t>
+  </si>
+  <si>
+    <t>A password that is too short or lacks a letter or number is rejected with clear guidance.</t>
+  </si>
+  <si>
+    <t>1. Open Register. 2. Complete the required fields with a valid email. 3. Enter a password shorter than eight characters or without both a letter and number. 4. Submit and confirm the password guidance appears.</t>
+  </si>
+  <si>
+    <t>Show confirmation mismatch feedback</t>
+  </si>
+  <si>
+    <t>Registration stays on the form and reports when password fields do not match.</t>
+  </si>
+  <si>
+    <t>1. Open Register and complete the required fields. 2. Enter a valid password and a different confirmation password. 3. Submit. 4. Confirm the mismatch message appears and the form remains visible.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -344,16 +611,19 @@
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
       <sz val="10"/>
-      <color rgb="FF1E1B2E"/>
+      <color rgb="FF1F2937"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <name val="Carlito"/>
     </font>
   </fonts>
   <fills count="3">
@@ -370,7 +640,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -417,21 +687,12 @@
     </border>
     <border>
       <left/>
-      <right style="thin">
+      <right/>
+      <top style="thin">
         <color rgb="FFD8CDB3"/>
-      </right>
-      <top/>
+      </top>
       <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
+        <color rgb="FFD8CDB3"/>
       </bottom>
       <diagonal/>
     </border>
@@ -439,7 +700,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -469,30 +730,39 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -806,6 +1076,189 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34DC9AF5-5BD4-482A-B7F9-DB033897936F}">
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="22.5703125" customWidth="1"/>
+    <col min="2" max="2" width="39" customWidth="1"/>
+    <col min="3" max="3" width="55.5703125" customWidth="1"/>
+    <col min="4" max="4" width="52.28515625" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="45.75">
+      <c r="A2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="45.75">
+      <c r="A3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="45.75">
+      <c r="A4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="5"/>
+    </row>
+    <row r="5" spans="1:6" ht="45.75">
+      <c r="A5" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="91.5">
+      <c r="A6" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="23" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="76.5">
+      <c r="A7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="106.5">
+      <c r="A8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="84" customHeight="1">
+      <c r="A9" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="4"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="2"/>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="4"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H18"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -818,16 +1271,16 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="3" t="s">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>1</v>
+        <v>42</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>2</v>
+        <v>43</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>3</v>
+        <v>44</v>
       </c>
       <c r="E1" s="5"/>
       <c r="F1" s="5"/>
@@ -836,16 +1289,16 @@
     </row>
     <row r="2" spans="1:8" ht="54" customHeight="1">
       <c r="A2" s="9" t="s">
-        <v>4</v>
+        <v>45</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>7</v>
+        <v>48</v>
       </c>
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
@@ -854,16 +1307,16 @@
     </row>
     <row r="3" spans="1:8" ht="36">
       <c r="A3" s="9" t="s">
-        <v>8</v>
+        <v>49</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>9</v>
+        <v>50</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>10</v>
+        <v>51</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
       <c r="E3" s="5"/>
       <c r="F3" s="5"/>
@@ -872,16 +1325,16 @@
     </row>
     <row r="4" spans="1:8" ht="39.75" customHeight="1">
       <c r="A4" s="9" t="s">
-        <v>12</v>
+        <v>53</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>13</v>
+        <v>54</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>14</v>
+        <v>55</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>15</v>
+        <v>56</v>
       </c>
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
@@ -890,16 +1343,16 @@
     </row>
     <row r="5" spans="1:8" ht="39" customHeight="1">
       <c r="A5" s="9" t="s">
-        <v>16</v>
+        <v>57</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>18</v>
+        <v>59</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>19</v>
+        <v>60</v>
       </c>
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
@@ -1041,276 +1494,330 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34DC9AF5-5BD4-482A-B7F9-DB033897936F}">
-  <dimension ref="A1:F11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="22.5703125" customWidth="1"/>
-    <col min="2" max="2" width="39" customWidth="1"/>
-    <col min="3" max="3" width="55.5703125" customWidth="1"/>
-    <col min="4" max="4" width="52.28515625" customWidth="1"/>
-    <col min="5" max="5" width="9.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="45.75">
-      <c r="A2" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="45.75">
-      <c r="A3" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="45.75">
-      <c r="A4" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="F4" s="5"/>
-    </row>
-    <row r="5" spans="1:6" ht="45.75">
-      <c r="A5" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" s="4"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="2"/>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" s="4"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="2"/>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" s="4"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="2"/>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" s="4"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="2"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE4EFD82-DCBD-4BB3-BA94-E9E32ACDFEC8}">
   <dimension ref="A1:E29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.42578125" customWidth="1"/>
-    <col min="2" max="2" width="29.42578125" customWidth="1"/>
-    <col min="3" max="3" width="57.7109375" customWidth="1"/>
-    <col min="4" max="4" width="57.42578125" customWidth="1"/>
+    <col min="2" max="2" width="50" customWidth="1"/>
+    <col min="3" max="3" width="82.42578125" customWidth="1"/>
+    <col min="4" max="4" width="64.85546875" customWidth="1"/>
     <col min="5" max="5" width="10.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>43</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="45.75" customHeight="1">
       <c r="A2" s="3" t="s">
-        <v>44</v>
+        <v>62</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>46</v>
+        <v>64</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="E2" t="s">
-        <v>48</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="30.75">
       <c r="A3" s="3" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>51</v>
+        <v>68</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="E3" t="s">
-        <v>48</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="30.75">
       <c r="A4" s="3" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>54</v>
+        <v>71</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>56</v>
+        <v>73</v>
       </c>
       <c r="E4" t="s">
-        <v>48</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="30.75">
       <c r="A5" s="3" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="E5" t="s">
-        <v>48</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="30.75">
       <c r="A6" s="3" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="E6" t="s">
-        <v>48</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="30.75">
       <c r="A7" s="3" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>63</v>
+        <v>80</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>64</v>
+        <v>81</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>65</v>
+        <v>82</v>
       </c>
       <c r="E7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="30.75">
+      <c r="A8" s="3" t="s">
         <v>66</v>
       </c>
+      <c r="B8" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="E8" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="8" spans="1:5">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="8"/>
+    <row r="9" spans="1:5" ht="30.75">
+      <c r="A9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C9" t="s">
+        <v>87</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E9" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="29" spans="1:4">
+    <row r="10" spans="1:5" ht="60.75">
+      <c r="A10" t="s">
+        <v>89</v>
+      </c>
+      <c r="B10" t="s">
+        <v>90</v>
+      </c>
+      <c r="C10" t="s">
+        <v>91</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="45.75">
+      <c r="A11" t="s">
+        <v>93</v>
+      </c>
+      <c r="B11" t="s">
+        <v>94</v>
+      </c>
+      <c r="C11" t="s">
+        <v>95</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="45.75">
+      <c r="A12" t="s">
+        <v>93</v>
+      </c>
+      <c r="B12" t="s">
+        <v>97</v>
+      </c>
+      <c r="C12" t="s">
+        <v>98</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="60.75">
+      <c r="A13" t="s">
+        <v>100</v>
+      </c>
+      <c r="B13" t="s">
+        <v>101</v>
+      </c>
+      <c r="C13" t="s">
+        <v>102</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="E13" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="60.75">
+      <c r="A14" t="s">
+        <v>104</v>
+      </c>
+      <c r="B14" t="s">
+        <v>105</v>
+      </c>
+      <c r="C14" t="s">
+        <v>106</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="E14" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="60.75">
+      <c r="A15" t="s">
+        <v>108</v>
+      </c>
+      <c r="B15" t="s">
+        <v>109</v>
+      </c>
+      <c r="C15" t="s">
+        <v>110</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E15" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="60.75">
+      <c r="A16" t="s">
+        <v>112</v>
+      </c>
+      <c r="B16" t="s">
+        <v>113</v>
+      </c>
+      <c r="C16" t="s">
+        <v>114</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="E16" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="60.75">
+      <c r="A17" t="s">
+        <v>116</v>
+      </c>
+      <c r="B17" t="s">
+        <v>117</v>
+      </c>
+      <c r="C17" t="s">
+        <v>118</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="45.75">
+      <c r="A18" t="s">
+        <v>120</v>
+      </c>
+      <c r="B18" t="s">
+        <v>121</v>
+      </c>
+      <c r="C18" t="s">
+        <v>122</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="E18" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
       <c r="A29" s="6" t="s">
-        <v>67</v>
+        <v>124</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>67</v>
+        <v>124</v>
       </c>
       <c r="C29" s="6"/>
       <c r="D29" s="6"/>
@@ -1333,36 +1840,36 @@
   <sheetData>
     <row r="1" spans="1:500">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>42</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>43</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>44</v>
       </c>
       <c r="E1" s="18" t="s">
-        <v>24</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:500" ht="36">
       <c r="A2" s="11" t="s">
-        <v>68</v>
+        <v>125</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>69</v>
+        <v>126</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>70</v>
+        <v>127</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>71</v>
+        <v>128</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="F2" s="14"/>
       <c r="G2" s="14"/>
@@ -1862,19 +2369,19 @@
     </row>
     <row r="3" spans="1:500" ht="36">
       <c r="A3" s="11" t="s">
-        <v>72</v>
+        <v>129</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>73</v>
+        <v>130</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>74</v>
+        <v>131</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>75</v>
+        <v>132</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="F3" s="14"/>
       <c r="G3" s="14"/>
@@ -2374,19 +2881,19 @@
     </row>
     <row r="4" spans="1:500" ht="24">
       <c r="A4" s="15" t="s">
-        <v>76</v>
+        <v>133</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>77</v>
+        <v>134</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>78</v>
+        <v>135</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>79</v>
+        <v>136</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="F4" s="14"/>
       <c r="G4" s="14"/>
@@ -2886,19 +3393,19 @@
     </row>
     <row r="5" spans="1:500" ht="36">
       <c r="A5" s="15" t="s">
-        <v>80</v>
+        <v>137</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>81</v>
+        <v>138</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="D5" s="16" t="s">
-        <v>83</v>
+        <v>139</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>140</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="F5" s="14"/>
       <c r="G5" s="14"/>
@@ -3396,21 +3903,2578 @@
       <c r="SE5" s="14"/>
       <c r="SF5" s="14"/>
     </row>
-    <row r="10" spans="1:500">
-      <c r="D10" s="20"/>
+    <row r="6" spans="1:500" ht="36">
+      <c r="A6" s="21" t="s">
+        <v>141</v>
+      </c>
+      <c r="B6" s="21" t="s">
+        <v>142</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>143</v>
+      </c>
+      <c r="D6" s="21" t="s">
+        <v>144</v>
+      </c>
+      <c r="E6" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="14"/>
+      <c r="K6" s="14"/>
+      <c r="L6" s="14"/>
+      <c r="M6" s="14"/>
+      <c r="N6" s="14"/>
+      <c r="O6" s="14"/>
+      <c r="P6" s="14"/>
+      <c r="Q6" s="14"/>
+      <c r="R6" s="14"/>
+      <c r="S6" s="14"/>
+      <c r="T6" s="14"/>
+      <c r="U6" s="14"/>
+      <c r="V6" s="14"/>
+      <c r="W6" s="14"/>
+      <c r="X6" s="14"/>
+      <c r="Y6" s="14"/>
+      <c r="Z6" s="14"/>
+      <c r="AA6" s="14"/>
+      <c r="AB6" s="14"/>
+      <c r="AC6" s="14"/>
+      <c r="AD6" s="14"/>
+      <c r="AE6" s="14"/>
+      <c r="AF6" s="14"/>
+      <c r="AG6" s="14"/>
+      <c r="AH6" s="14"/>
+      <c r="AI6" s="14"/>
+      <c r="AJ6" s="14"/>
+      <c r="AK6" s="14"/>
+      <c r="AL6" s="14"/>
+      <c r="AM6" s="14"/>
+      <c r="AN6" s="14"/>
+      <c r="AO6" s="14"/>
+      <c r="AP6" s="14"/>
+      <c r="AQ6" s="14"/>
+      <c r="AR6" s="14"/>
+      <c r="AS6" s="14"/>
+      <c r="AT6" s="14"/>
+      <c r="AU6" s="14"/>
+      <c r="AV6" s="14"/>
+      <c r="AW6" s="14"/>
+      <c r="AX6" s="14"/>
+      <c r="AY6" s="14"/>
+      <c r="AZ6" s="14"/>
+      <c r="BA6" s="14"/>
+      <c r="BB6" s="14"/>
+      <c r="BC6" s="14"/>
+      <c r="BD6" s="14"/>
+      <c r="BE6" s="14"/>
+      <c r="BF6" s="14"/>
+      <c r="BG6" s="14"/>
+      <c r="BH6" s="14"/>
+      <c r="BI6" s="14"/>
+      <c r="BJ6" s="14"/>
+      <c r="BK6" s="14"/>
+      <c r="BL6" s="14"/>
+      <c r="BM6" s="14"/>
+      <c r="BN6" s="14"/>
+      <c r="BO6" s="14"/>
+      <c r="BP6" s="14"/>
+      <c r="BQ6" s="14"/>
+      <c r="BR6" s="14"/>
+      <c r="BS6" s="14"/>
+      <c r="BT6" s="14"/>
+      <c r="BU6" s="14"/>
+      <c r="BV6" s="14"/>
+      <c r="BW6" s="14"/>
+      <c r="BX6" s="14"/>
+      <c r="BY6" s="14"/>
+      <c r="BZ6" s="14"/>
+      <c r="CA6" s="14"/>
+      <c r="CB6" s="14"/>
+      <c r="CC6" s="14"/>
+      <c r="CD6" s="14"/>
+      <c r="CE6" s="14"/>
+      <c r="CF6" s="14"/>
+      <c r="CG6" s="14"/>
+      <c r="CH6" s="14"/>
+      <c r="CI6" s="14"/>
+      <c r="CJ6" s="14"/>
+      <c r="CK6" s="14"/>
+      <c r="CL6" s="14"/>
+      <c r="CM6" s="14"/>
+      <c r="CN6" s="14"/>
+      <c r="CO6" s="14"/>
+      <c r="CP6" s="14"/>
+      <c r="CQ6" s="14"/>
+      <c r="CR6" s="14"/>
+      <c r="CS6" s="14"/>
+      <c r="CT6" s="14"/>
+      <c r="CU6" s="14"/>
+      <c r="CV6" s="14"/>
+      <c r="CW6" s="14"/>
+      <c r="CX6" s="14"/>
+      <c r="CY6" s="14"/>
+      <c r="CZ6" s="14"/>
+      <c r="DA6" s="14"/>
+      <c r="DB6" s="14"/>
+      <c r="DC6" s="14"/>
+      <c r="DD6" s="14"/>
+      <c r="DE6" s="14"/>
+      <c r="DF6" s="14"/>
+      <c r="DG6" s="14"/>
+      <c r="DH6" s="14"/>
+      <c r="DI6" s="14"/>
+      <c r="DJ6" s="14"/>
+      <c r="DK6" s="14"/>
+      <c r="DL6" s="14"/>
+      <c r="DM6" s="14"/>
+      <c r="DN6" s="14"/>
+      <c r="DO6" s="14"/>
+      <c r="DP6" s="14"/>
+      <c r="DQ6" s="14"/>
+      <c r="DR6" s="14"/>
+      <c r="DS6" s="14"/>
+      <c r="DT6" s="14"/>
+      <c r="DU6" s="14"/>
+      <c r="DV6" s="14"/>
+      <c r="DW6" s="14"/>
+      <c r="DX6" s="14"/>
+      <c r="DY6" s="14"/>
+      <c r="DZ6" s="14"/>
+      <c r="EA6" s="14"/>
+      <c r="EB6" s="14"/>
+      <c r="EC6" s="14"/>
+      <c r="ED6" s="14"/>
+      <c r="EE6" s="14"/>
+      <c r="EF6" s="14"/>
+      <c r="EG6" s="14"/>
+      <c r="EH6" s="14"/>
+      <c r="EI6" s="14"/>
+      <c r="EJ6" s="14"/>
+      <c r="EK6" s="14"/>
+      <c r="EL6" s="14"/>
+      <c r="EM6" s="14"/>
+      <c r="EN6" s="14"/>
+      <c r="EO6" s="14"/>
+      <c r="EP6" s="14"/>
+      <c r="EQ6" s="14"/>
+      <c r="ER6" s="14"/>
+      <c r="ES6" s="14"/>
+      <c r="ET6" s="14"/>
+      <c r="EU6" s="14"/>
+      <c r="EV6" s="14"/>
+      <c r="EW6" s="14"/>
+      <c r="EX6" s="14"/>
+      <c r="EY6" s="14"/>
+      <c r="EZ6" s="14"/>
+      <c r="FA6" s="14"/>
+      <c r="FB6" s="14"/>
+      <c r="FC6" s="14"/>
+      <c r="FD6" s="14"/>
+      <c r="FE6" s="14"/>
+      <c r="FF6" s="14"/>
+      <c r="FG6" s="14"/>
+      <c r="FH6" s="14"/>
+      <c r="FI6" s="14"/>
+      <c r="FJ6" s="14"/>
+      <c r="FK6" s="14"/>
+      <c r="FL6" s="14"/>
+      <c r="FM6" s="14"/>
+      <c r="FN6" s="14"/>
+      <c r="FO6" s="14"/>
+      <c r="FP6" s="14"/>
+      <c r="FQ6" s="14"/>
+      <c r="FR6" s="14"/>
+      <c r="FS6" s="14"/>
+      <c r="FT6" s="14"/>
+      <c r="FU6" s="14"/>
+      <c r="FV6" s="14"/>
+      <c r="FW6" s="14"/>
+      <c r="FX6" s="14"/>
+      <c r="FY6" s="14"/>
+      <c r="FZ6" s="14"/>
+      <c r="GA6" s="14"/>
+      <c r="GB6" s="14"/>
+      <c r="GC6" s="14"/>
+      <c r="GD6" s="14"/>
+      <c r="GE6" s="14"/>
+      <c r="GF6" s="14"/>
+      <c r="GG6" s="14"/>
+      <c r="GH6" s="14"/>
+      <c r="GI6" s="14"/>
+      <c r="GJ6" s="14"/>
+      <c r="GK6" s="14"/>
+      <c r="GL6" s="14"/>
+      <c r="GM6" s="14"/>
+      <c r="GN6" s="14"/>
+      <c r="GO6" s="14"/>
+      <c r="GP6" s="14"/>
+      <c r="GQ6" s="14"/>
+      <c r="GR6" s="14"/>
+      <c r="GS6" s="14"/>
+      <c r="GT6" s="14"/>
+      <c r="GU6" s="14"/>
+      <c r="GV6" s="14"/>
+      <c r="GW6" s="14"/>
+      <c r="GX6" s="14"/>
+      <c r="GY6" s="14"/>
+      <c r="GZ6" s="14"/>
+      <c r="HA6" s="14"/>
+      <c r="HB6" s="14"/>
+      <c r="HC6" s="14"/>
+      <c r="HD6" s="14"/>
+      <c r="HE6" s="14"/>
+      <c r="HF6" s="14"/>
+      <c r="HG6" s="14"/>
+      <c r="HH6" s="14"/>
+      <c r="HI6" s="14"/>
+      <c r="HJ6" s="14"/>
+      <c r="HK6" s="14"/>
+      <c r="HL6" s="14"/>
+      <c r="HM6" s="14"/>
+      <c r="HN6" s="14"/>
+      <c r="HO6" s="14"/>
+      <c r="HP6" s="14"/>
+      <c r="HQ6" s="14"/>
+      <c r="HR6" s="14"/>
+      <c r="HS6" s="14"/>
+      <c r="HT6" s="14"/>
+      <c r="HU6" s="14"/>
+      <c r="HV6" s="14"/>
+      <c r="HW6" s="14"/>
+      <c r="HX6" s="14"/>
+      <c r="HY6" s="14"/>
+      <c r="HZ6" s="14"/>
+      <c r="IA6" s="14"/>
+      <c r="IB6" s="14"/>
+      <c r="IC6" s="14"/>
+      <c r="ID6" s="14"/>
+      <c r="IE6" s="14"/>
+      <c r="IF6" s="14"/>
+      <c r="IG6" s="14"/>
+      <c r="IH6" s="14"/>
+      <c r="II6" s="14"/>
+      <c r="IJ6" s="14"/>
+      <c r="IK6" s="14"/>
+      <c r="IL6" s="14"/>
+      <c r="IM6" s="14"/>
+      <c r="IN6" s="14"/>
+      <c r="IO6" s="14"/>
+      <c r="IP6" s="14"/>
+      <c r="IQ6" s="14"/>
+      <c r="IR6" s="14"/>
+      <c r="IS6" s="14"/>
+      <c r="IT6" s="14"/>
+      <c r="IU6" s="14"/>
+      <c r="IV6" s="14"/>
+      <c r="IW6" s="14"/>
+      <c r="IX6" s="14"/>
+      <c r="IY6" s="14"/>
+      <c r="IZ6" s="14"/>
+      <c r="JA6" s="14"/>
+      <c r="JB6" s="14"/>
+      <c r="JC6" s="14"/>
+      <c r="JD6" s="14"/>
+      <c r="JE6" s="14"/>
+      <c r="JF6" s="14"/>
+      <c r="JG6" s="14"/>
+      <c r="JH6" s="14"/>
+      <c r="JI6" s="14"/>
+      <c r="JJ6" s="14"/>
+      <c r="JK6" s="14"/>
+      <c r="JL6" s="14"/>
+      <c r="JM6" s="14"/>
+      <c r="JN6" s="14"/>
+      <c r="JO6" s="14"/>
+      <c r="JP6" s="14"/>
+      <c r="JQ6" s="14"/>
+      <c r="JR6" s="14"/>
+      <c r="JS6" s="14"/>
+      <c r="JT6" s="14"/>
+      <c r="JU6" s="14"/>
+      <c r="JV6" s="14"/>
+      <c r="JW6" s="14"/>
+      <c r="JX6" s="14"/>
+      <c r="JY6" s="14"/>
+      <c r="JZ6" s="14"/>
+      <c r="KA6" s="14"/>
+      <c r="KB6" s="14"/>
+      <c r="KC6" s="14"/>
+      <c r="KD6" s="14"/>
+      <c r="KE6" s="14"/>
+      <c r="KF6" s="14"/>
+      <c r="KG6" s="14"/>
+      <c r="KH6" s="14"/>
+      <c r="KI6" s="14"/>
+      <c r="KJ6" s="14"/>
+      <c r="KK6" s="14"/>
+      <c r="KL6" s="14"/>
+      <c r="KM6" s="14"/>
+      <c r="KN6" s="14"/>
+      <c r="KO6" s="14"/>
+      <c r="KP6" s="14"/>
+      <c r="KQ6" s="14"/>
+      <c r="KR6" s="14"/>
+      <c r="KS6" s="14"/>
+      <c r="KT6" s="14"/>
+      <c r="KU6" s="14"/>
+      <c r="KV6" s="14"/>
+      <c r="KW6" s="14"/>
+      <c r="KX6" s="14"/>
+      <c r="KY6" s="14"/>
+      <c r="KZ6" s="14"/>
+      <c r="LA6" s="14"/>
+      <c r="LB6" s="14"/>
+      <c r="LC6" s="14"/>
+      <c r="LD6" s="14"/>
+      <c r="LE6" s="14"/>
+      <c r="LF6" s="14"/>
+      <c r="LG6" s="14"/>
+      <c r="LH6" s="14"/>
+      <c r="LI6" s="14"/>
+      <c r="LJ6" s="14"/>
+      <c r="LK6" s="14"/>
+      <c r="LL6" s="14"/>
+      <c r="LM6" s="14"/>
+      <c r="LN6" s="14"/>
+      <c r="LO6" s="14"/>
+      <c r="LP6" s="14"/>
+      <c r="LQ6" s="14"/>
+      <c r="LR6" s="14"/>
+      <c r="LS6" s="14"/>
+      <c r="LT6" s="14"/>
+      <c r="LU6" s="14"/>
+      <c r="LV6" s="14"/>
+      <c r="LW6" s="14"/>
+      <c r="LX6" s="14"/>
+      <c r="LY6" s="14"/>
+      <c r="LZ6" s="14"/>
+      <c r="MA6" s="14"/>
+      <c r="MB6" s="14"/>
+      <c r="MC6" s="14"/>
+      <c r="MD6" s="14"/>
+      <c r="ME6" s="14"/>
+      <c r="MF6" s="14"/>
+      <c r="MG6" s="14"/>
+      <c r="MH6" s="14"/>
+      <c r="MI6" s="14"/>
+      <c r="MJ6" s="14"/>
+      <c r="MK6" s="14"/>
+      <c r="ML6" s="14"/>
+      <c r="MM6" s="14"/>
+      <c r="MN6" s="14"/>
+      <c r="MO6" s="14"/>
+      <c r="MP6" s="14"/>
+      <c r="MQ6" s="14"/>
+      <c r="MR6" s="14"/>
+      <c r="MS6" s="14"/>
+      <c r="MT6" s="14"/>
+      <c r="MU6" s="14"/>
+      <c r="MV6" s="14"/>
+      <c r="MW6" s="14"/>
+      <c r="MX6" s="14"/>
+      <c r="MY6" s="14"/>
+      <c r="MZ6" s="14"/>
+      <c r="NA6" s="14"/>
+      <c r="NB6" s="14"/>
+      <c r="NC6" s="14"/>
+      <c r="ND6" s="14"/>
+      <c r="NE6" s="14"/>
+      <c r="NF6" s="14"/>
+      <c r="NG6" s="14"/>
+      <c r="NH6" s="14"/>
+      <c r="NI6" s="14"/>
+      <c r="NJ6" s="14"/>
+      <c r="NK6" s="14"/>
+      <c r="NL6" s="14"/>
+      <c r="NM6" s="14"/>
+      <c r="NN6" s="14"/>
+      <c r="NO6" s="14"/>
+      <c r="NP6" s="14"/>
+      <c r="NQ6" s="14"/>
+      <c r="NR6" s="14"/>
+      <c r="NS6" s="14"/>
+      <c r="NT6" s="14"/>
+      <c r="NU6" s="14"/>
+      <c r="NV6" s="14"/>
+      <c r="NW6" s="14"/>
+      <c r="NX6" s="14"/>
+      <c r="NY6" s="14"/>
+      <c r="NZ6" s="14"/>
+      <c r="OA6" s="14"/>
+      <c r="OB6" s="14"/>
+      <c r="OC6" s="14"/>
+      <c r="OD6" s="14"/>
+      <c r="OE6" s="14"/>
+      <c r="OF6" s="14"/>
+      <c r="OG6" s="14"/>
+      <c r="OH6" s="14"/>
+      <c r="OI6" s="14"/>
+      <c r="OJ6" s="14"/>
+      <c r="OK6" s="14"/>
+      <c r="OL6" s="14"/>
+      <c r="OM6" s="14"/>
+      <c r="ON6" s="14"/>
+      <c r="OO6" s="14"/>
+      <c r="OP6" s="14"/>
+      <c r="OQ6" s="14"/>
+      <c r="OR6" s="14"/>
+      <c r="OS6" s="14"/>
+      <c r="OT6" s="14"/>
+      <c r="OU6" s="14"/>
+      <c r="OV6" s="14"/>
+      <c r="OW6" s="14"/>
+      <c r="OX6" s="14"/>
+      <c r="OY6" s="14"/>
+      <c r="OZ6" s="14"/>
+      <c r="PA6" s="14"/>
+      <c r="PB6" s="14"/>
+      <c r="PC6" s="14"/>
+      <c r="PD6" s="14"/>
+      <c r="PE6" s="14"/>
+      <c r="PF6" s="14"/>
+      <c r="PG6" s="14"/>
+      <c r="PH6" s="14"/>
+      <c r="PI6" s="14"/>
+      <c r="PJ6" s="14"/>
+      <c r="PK6" s="14"/>
+      <c r="PL6" s="14"/>
+      <c r="PM6" s="14"/>
+      <c r="PN6" s="14"/>
+      <c r="PO6" s="14"/>
+      <c r="PP6" s="14"/>
+      <c r="PQ6" s="14"/>
+      <c r="PR6" s="14"/>
+      <c r="PS6" s="14"/>
+      <c r="PT6" s="14"/>
+      <c r="PU6" s="14"/>
+      <c r="PV6" s="14"/>
+      <c r="PW6" s="14"/>
+      <c r="PX6" s="14"/>
+      <c r="PY6" s="14"/>
+      <c r="PZ6" s="14"/>
+      <c r="QA6" s="14"/>
+      <c r="QB6" s="14"/>
+      <c r="QC6" s="14"/>
+      <c r="QD6" s="14"/>
+      <c r="QE6" s="14"/>
+      <c r="QF6" s="14"/>
+      <c r="QG6" s="14"/>
+      <c r="QH6" s="14"/>
+      <c r="QI6" s="14"/>
+      <c r="QJ6" s="14"/>
+      <c r="QK6" s="14"/>
+      <c r="QL6" s="14"/>
+      <c r="QM6" s="14"/>
+      <c r="QN6" s="14"/>
+      <c r="QO6" s="14"/>
+      <c r="QP6" s="14"/>
+      <c r="QQ6" s="14"/>
+      <c r="QR6" s="14"/>
+      <c r="QS6" s="14"/>
+      <c r="QT6" s="14"/>
+      <c r="QU6" s="14"/>
+      <c r="QV6" s="14"/>
+      <c r="QW6" s="14"/>
+      <c r="QX6" s="14"/>
+      <c r="QY6" s="14"/>
+      <c r="QZ6" s="14"/>
+      <c r="RA6" s="14"/>
+      <c r="RB6" s="14"/>
+      <c r="RC6" s="14"/>
+      <c r="RD6" s="14"/>
+      <c r="RE6" s="14"/>
+      <c r="RF6" s="14"/>
+      <c r="RG6" s="14"/>
+      <c r="RH6" s="14"/>
+      <c r="RI6" s="14"/>
+      <c r="RJ6" s="14"/>
+      <c r="RK6" s="14"/>
+      <c r="RL6" s="14"/>
+      <c r="RM6" s="14"/>
+      <c r="RN6" s="14"/>
+      <c r="RO6" s="14"/>
+      <c r="RP6" s="14"/>
+      <c r="RQ6" s="14"/>
+      <c r="RR6" s="14"/>
+      <c r="RS6" s="14"/>
+      <c r="RT6" s="14"/>
+      <c r="RU6" s="14"/>
+      <c r="RV6" s="14"/>
+      <c r="RW6" s="14"/>
+      <c r="RX6" s="14"/>
+      <c r="RY6" s="14"/>
+      <c r="RZ6" s="14"/>
+      <c r="SA6" s="14"/>
+      <c r="SB6" s="14"/>
+      <c r="SC6" s="14"/>
+      <c r="SD6" s="14"/>
+      <c r="SE6" s="14"/>
+      <c r="SF6" s="14"/>
+    </row>
+    <row r="7" spans="1:500" ht="36">
+      <c r="A7" s="21" t="s">
+        <v>141</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>145</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>146</v>
+      </c>
+      <c r="D7" s="21" t="s">
+        <v>147</v>
+      </c>
+      <c r="E7" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="14"/>
+      <c r="K7" s="14"/>
+      <c r="L7" s="14"/>
+      <c r="M7" s="14"/>
+      <c r="N7" s="14"/>
+      <c r="O7" s="14"/>
+      <c r="P7" s="14"/>
+      <c r="Q7" s="14"/>
+      <c r="R7" s="14"/>
+      <c r="S7" s="14"/>
+      <c r="T7" s="14"/>
+      <c r="U7" s="14"/>
+      <c r="V7" s="14"/>
+      <c r="W7" s="14"/>
+      <c r="X7" s="14"/>
+      <c r="Y7" s="14"/>
+      <c r="Z7" s="14"/>
+      <c r="AA7" s="14"/>
+      <c r="AB7" s="14"/>
+      <c r="AC7" s="14"/>
+      <c r="AD7" s="14"/>
+      <c r="AE7" s="14"/>
+      <c r="AF7" s="14"/>
+      <c r="AG7" s="14"/>
+      <c r="AH7" s="14"/>
+      <c r="AI7" s="14"/>
+      <c r="AJ7" s="14"/>
+      <c r="AK7" s="14"/>
+      <c r="AL7" s="14"/>
+      <c r="AM7" s="14"/>
+      <c r="AN7" s="14"/>
+      <c r="AO7" s="14"/>
+      <c r="AP7" s="14"/>
+      <c r="AQ7" s="14"/>
+      <c r="AR7" s="14"/>
+      <c r="AS7" s="14"/>
+      <c r="AT7" s="14"/>
+      <c r="AU7" s="14"/>
+      <c r="AV7" s="14"/>
+      <c r="AW7" s="14"/>
+      <c r="AX7" s="14"/>
+      <c r="AY7" s="14"/>
+      <c r="AZ7" s="14"/>
+      <c r="BA7" s="14"/>
+      <c r="BB7" s="14"/>
+      <c r="BC7" s="14"/>
+      <c r="BD7" s="14"/>
+      <c r="BE7" s="14"/>
+      <c r="BF7" s="14"/>
+      <c r="BG7" s="14"/>
+      <c r="BH7" s="14"/>
+      <c r="BI7" s="14"/>
+      <c r="BJ7" s="14"/>
+      <c r="BK7" s="14"/>
+      <c r="BL7" s="14"/>
+      <c r="BM7" s="14"/>
+      <c r="BN7" s="14"/>
+      <c r="BO7" s="14"/>
+      <c r="BP7" s="14"/>
+      <c r="BQ7" s="14"/>
+      <c r="BR7" s="14"/>
+      <c r="BS7" s="14"/>
+      <c r="BT7" s="14"/>
+      <c r="BU7" s="14"/>
+      <c r="BV7" s="14"/>
+      <c r="BW7" s="14"/>
+      <c r="BX7" s="14"/>
+      <c r="BY7" s="14"/>
+      <c r="BZ7" s="14"/>
+      <c r="CA7" s="14"/>
+      <c r="CB7" s="14"/>
+      <c r="CC7" s="14"/>
+      <c r="CD7" s="14"/>
+      <c r="CE7" s="14"/>
+      <c r="CF7" s="14"/>
+      <c r="CG7" s="14"/>
+      <c r="CH7" s="14"/>
+      <c r="CI7" s="14"/>
+      <c r="CJ7" s="14"/>
+      <c r="CK7" s="14"/>
+      <c r="CL7" s="14"/>
+      <c r="CM7" s="14"/>
+      <c r="CN7" s="14"/>
+      <c r="CO7" s="14"/>
+      <c r="CP7" s="14"/>
+      <c r="CQ7" s="14"/>
+      <c r="CR7" s="14"/>
+      <c r="CS7" s="14"/>
+      <c r="CT7" s="14"/>
+      <c r="CU7" s="14"/>
+      <c r="CV7" s="14"/>
+      <c r="CW7" s="14"/>
+      <c r="CX7" s="14"/>
+      <c r="CY7" s="14"/>
+      <c r="CZ7" s="14"/>
+      <c r="DA7" s="14"/>
+      <c r="DB7" s="14"/>
+      <c r="DC7" s="14"/>
+      <c r="DD7" s="14"/>
+      <c r="DE7" s="14"/>
+      <c r="DF7" s="14"/>
+      <c r="DG7" s="14"/>
+      <c r="DH7" s="14"/>
+      <c r="DI7" s="14"/>
+      <c r="DJ7" s="14"/>
+      <c r="DK7" s="14"/>
+      <c r="DL7" s="14"/>
+      <c r="DM7" s="14"/>
+      <c r="DN7" s="14"/>
+      <c r="DO7" s="14"/>
+      <c r="DP7" s="14"/>
+      <c r="DQ7" s="14"/>
+      <c r="DR7" s="14"/>
+      <c r="DS7" s="14"/>
+      <c r="DT7" s="14"/>
+      <c r="DU7" s="14"/>
+      <c r="DV7" s="14"/>
+      <c r="DW7" s="14"/>
+      <c r="DX7" s="14"/>
+      <c r="DY7" s="14"/>
+      <c r="DZ7" s="14"/>
+      <c r="EA7" s="14"/>
+      <c r="EB7" s="14"/>
+      <c r="EC7" s="14"/>
+      <c r="ED7" s="14"/>
+      <c r="EE7" s="14"/>
+      <c r="EF7" s="14"/>
+      <c r="EG7" s="14"/>
+      <c r="EH7" s="14"/>
+      <c r="EI7" s="14"/>
+      <c r="EJ7" s="14"/>
+      <c r="EK7" s="14"/>
+      <c r="EL7" s="14"/>
+      <c r="EM7" s="14"/>
+      <c r="EN7" s="14"/>
+      <c r="EO7" s="14"/>
+      <c r="EP7" s="14"/>
+      <c r="EQ7" s="14"/>
+      <c r="ER7" s="14"/>
+      <c r="ES7" s="14"/>
+      <c r="ET7" s="14"/>
+      <c r="EU7" s="14"/>
+      <c r="EV7" s="14"/>
+      <c r="EW7" s="14"/>
+      <c r="EX7" s="14"/>
+      <c r="EY7" s="14"/>
+      <c r="EZ7" s="14"/>
+      <c r="FA7" s="14"/>
+      <c r="FB7" s="14"/>
+      <c r="FC7" s="14"/>
+      <c r="FD7" s="14"/>
+      <c r="FE7" s="14"/>
+      <c r="FF7" s="14"/>
+      <c r="FG7" s="14"/>
+      <c r="FH7" s="14"/>
+      <c r="FI7" s="14"/>
+      <c r="FJ7" s="14"/>
+      <c r="FK7" s="14"/>
+      <c r="FL7" s="14"/>
+      <c r="FM7" s="14"/>
+      <c r="FN7" s="14"/>
+      <c r="FO7" s="14"/>
+      <c r="FP7" s="14"/>
+      <c r="FQ7" s="14"/>
+      <c r="FR7" s="14"/>
+      <c r="FS7" s="14"/>
+      <c r="FT7" s="14"/>
+      <c r="FU7" s="14"/>
+      <c r="FV7" s="14"/>
+      <c r="FW7" s="14"/>
+      <c r="FX7" s="14"/>
+      <c r="FY7" s="14"/>
+      <c r="FZ7" s="14"/>
+      <c r="GA7" s="14"/>
+      <c r="GB7" s="14"/>
+      <c r="GC7" s="14"/>
+      <c r="GD7" s="14"/>
+      <c r="GE7" s="14"/>
+      <c r="GF7" s="14"/>
+      <c r="GG7" s="14"/>
+      <c r="GH7" s="14"/>
+      <c r="GI7" s="14"/>
+      <c r="GJ7" s="14"/>
+      <c r="GK7" s="14"/>
+      <c r="GL7" s="14"/>
+      <c r="GM7" s="14"/>
+      <c r="GN7" s="14"/>
+      <c r="GO7" s="14"/>
+      <c r="GP7" s="14"/>
+      <c r="GQ7" s="14"/>
+      <c r="GR7" s="14"/>
+      <c r="GS7" s="14"/>
+      <c r="GT7" s="14"/>
+      <c r="GU7" s="14"/>
+      <c r="GV7" s="14"/>
+      <c r="GW7" s="14"/>
+      <c r="GX7" s="14"/>
+      <c r="GY7" s="14"/>
+      <c r="GZ7" s="14"/>
+      <c r="HA7" s="14"/>
+      <c r="HB7" s="14"/>
+      <c r="HC7" s="14"/>
+      <c r="HD7" s="14"/>
+      <c r="HE7" s="14"/>
+      <c r="HF7" s="14"/>
+      <c r="HG7" s="14"/>
+      <c r="HH7" s="14"/>
+      <c r="HI7" s="14"/>
+      <c r="HJ7" s="14"/>
+      <c r="HK7" s="14"/>
+      <c r="HL7" s="14"/>
+      <c r="HM7" s="14"/>
+      <c r="HN7" s="14"/>
+      <c r="HO7" s="14"/>
+      <c r="HP7" s="14"/>
+      <c r="HQ7" s="14"/>
+      <c r="HR7" s="14"/>
+      <c r="HS7" s="14"/>
+      <c r="HT7" s="14"/>
+      <c r="HU7" s="14"/>
+      <c r="HV7" s="14"/>
+      <c r="HW7" s="14"/>
+      <c r="HX7" s="14"/>
+      <c r="HY7" s="14"/>
+      <c r="HZ7" s="14"/>
+      <c r="IA7" s="14"/>
+      <c r="IB7" s="14"/>
+      <c r="IC7" s="14"/>
+      <c r="ID7" s="14"/>
+      <c r="IE7" s="14"/>
+      <c r="IF7" s="14"/>
+      <c r="IG7" s="14"/>
+      <c r="IH7" s="14"/>
+      <c r="II7" s="14"/>
+      <c r="IJ7" s="14"/>
+      <c r="IK7" s="14"/>
+      <c r="IL7" s="14"/>
+      <c r="IM7" s="14"/>
+      <c r="IN7" s="14"/>
+      <c r="IO7" s="14"/>
+      <c r="IP7" s="14"/>
+      <c r="IQ7" s="14"/>
+      <c r="IR7" s="14"/>
+      <c r="IS7" s="14"/>
+      <c r="IT7" s="14"/>
+      <c r="IU7" s="14"/>
+      <c r="IV7" s="14"/>
+      <c r="IW7" s="14"/>
+      <c r="IX7" s="14"/>
+      <c r="IY7" s="14"/>
+      <c r="IZ7" s="14"/>
+      <c r="JA7" s="14"/>
+      <c r="JB7" s="14"/>
+      <c r="JC7" s="14"/>
+      <c r="JD7" s="14"/>
+      <c r="JE7" s="14"/>
+      <c r="JF7" s="14"/>
+      <c r="JG7" s="14"/>
+      <c r="JH7" s="14"/>
+      <c r="JI7" s="14"/>
+      <c r="JJ7" s="14"/>
+      <c r="JK7" s="14"/>
+      <c r="JL7" s="14"/>
+      <c r="JM7" s="14"/>
+      <c r="JN7" s="14"/>
+      <c r="JO7" s="14"/>
+      <c r="JP7" s="14"/>
+      <c r="JQ7" s="14"/>
+      <c r="JR7" s="14"/>
+      <c r="JS7" s="14"/>
+      <c r="JT7" s="14"/>
+      <c r="JU7" s="14"/>
+      <c r="JV7" s="14"/>
+      <c r="JW7" s="14"/>
+      <c r="JX7" s="14"/>
+      <c r="JY7" s="14"/>
+      <c r="JZ7" s="14"/>
+      <c r="KA7" s="14"/>
+      <c r="KB7" s="14"/>
+      <c r="KC7" s="14"/>
+      <c r="KD7" s="14"/>
+      <c r="KE7" s="14"/>
+      <c r="KF7" s="14"/>
+      <c r="KG7" s="14"/>
+      <c r="KH7" s="14"/>
+      <c r="KI7" s="14"/>
+      <c r="KJ7" s="14"/>
+      <c r="KK7" s="14"/>
+      <c r="KL7" s="14"/>
+      <c r="KM7" s="14"/>
+      <c r="KN7" s="14"/>
+      <c r="KO7" s="14"/>
+      <c r="KP7" s="14"/>
+      <c r="KQ7" s="14"/>
+      <c r="KR7" s="14"/>
+      <c r="KS7" s="14"/>
+      <c r="KT7" s="14"/>
+      <c r="KU7" s="14"/>
+      <c r="KV7" s="14"/>
+      <c r="KW7" s="14"/>
+      <c r="KX7" s="14"/>
+      <c r="KY7" s="14"/>
+      <c r="KZ7" s="14"/>
+      <c r="LA7" s="14"/>
+      <c r="LB7" s="14"/>
+      <c r="LC7" s="14"/>
+      <c r="LD7" s="14"/>
+      <c r="LE7" s="14"/>
+      <c r="LF7" s="14"/>
+      <c r="LG7" s="14"/>
+      <c r="LH7" s="14"/>
+      <c r="LI7" s="14"/>
+      <c r="LJ7" s="14"/>
+      <c r="LK7" s="14"/>
+      <c r="LL7" s="14"/>
+      <c r="LM7" s="14"/>
+      <c r="LN7" s="14"/>
+      <c r="LO7" s="14"/>
+      <c r="LP7" s="14"/>
+      <c r="LQ7" s="14"/>
+      <c r="LR7" s="14"/>
+      <c r="LS7" s="14"/>
+      <c r="LT7" s="14"/>
+      <c r="LU7" s="14"/>
+      <c r="LV7" s="14"/>
+      <c r="LW7" s="14"/>
+      <c r="LX7" s="14"/>
+      <c r="LY7" s="14"/>
+      <c r="LZ7" s="14"/>
+      <c r="MA7" s="14"/>
+      <c r="MB7" s="14"/>
+      <c r="MC7" s="14"/>
+      <c r="MD7" s="14"/>
+      <c r="ME7" s="14"/>
+      <c r="MF7" s="14"/>
+      <c r="MG7" s="14"/>
+      <c r="MH7" s="14"/>
+      <c r="MI7" s="14"/>
+      <c r="MJ7" s="14"/>
+      <c r="MK7" s="14"/>
+      <c r="ML7" s="14"/>
+      <c r="MM7" s="14"/>
+      <c r="MN7" s="14"/>
+      <c r="MO7" s="14"/>
+      <c r="MP7" s="14"/>
+      <c r="MQ7" s="14"/>
+      <c r="MR7" s="14"/>
+      <c r="MS7" s="14"/>
+      <c r="MT7" s="14"/>
+      <c r="MU7" s="14"/>
+      <c r="MV7" s="14"/>
+      <c r="MW7" s="14"/>
+      <c r="MX7" s="14"/>
+      <c r="MY7" s="14"/>
+      <c r="MZ7" s="14"/>
+      <c r="NA7" s="14"/>
+      <c r="NB7" s="14"/>
+      <c r="NC7" s="14"/>
+      <c r="ND7" s="14"/>
+      <c r="NE7" s="14"/>
+      <c r="NF7" s="14"/>
+      <c r="NG7" s="14"/>
+      <c r="NH7" s="14"/>
+      <c r="NI7" s="14"/>
+      <c r="NJ7" s="14"/>
+      <c r="NK7" s="14"/>
+      <c r="NL7" s="14"/>
+      <c r="NM7" s="14"/>
+      <c r="NN7" s="14"/>
+      <c r="NO7" s="14"/>
+      <c r="NP7" s="14"/>
+      <c r="NQ7" s="14"/>
+      <c r="NR7" s="14"/>
+      <c r="NS7" s="14"/>
+      <c r="NT7" s="14"/>
+      <c r="NU7" s="14"/>
+      <c r="NV7" s="14"/>
+      <c r="NW7" s="14"/>
+      <c r="NX7" s="14"/>
+      <c r="NY7" s="14"/>
+      <c r="NZ7" s="14"/>
+      <c r="OA7" s="14"/>
+      <c r="OB7" s="14"/>
+      <c r="OC7" s="14"/>
+      <c r="OD7" s="14"/>
+      <c r="OE7" s="14"/>
+      <c r="OF7" s="14"/>
+      <c r="OG7" s="14"/>
+      <c r="OH7" s="14"/>
+      <c r="OI7" s="14"/>
+      <c r="OJ7" s="14"/>
+      <c r="OK7" s="14"/>
+      <c r="OL7" s="14"/>
+      <c r="OM7" s="14"/>
+      <c r="ON7" s="14"/>
+      <c r="OO7" s="14"/>
+      <c r="OP7" s="14"/>
+      <c r="OQ7" s="14"/>
+      <c r="OR7" s="14"/>
+      <c r="OS7" s="14"/>
+      <c r="OT7" s="14"/>
+      <c r="OU7" s="14"/>
+      <c r="OV7" s="14"/>
+      <c r="OW7" s="14"/>
+      <c r="OX7" s="14"/>
+      <c r="OY7" s="14"/>
+      <c r="OZ7" s="14"/>
+      <c r="PA7" s="14"/>
+      <c r="PB7" s="14"/>
+      <c r="PC7" s="14"/>
+      <c r="PD7" s="14"/>
+      <c r="PE7" s="14"/>
+      <c r="PF7" s="14"/>
+      <c r="PG7" s="14"/>
+      <c r="PH7" s="14"/>
+      <c r="PI7" s="14"/>
+      <c r="PJ7" s="14"/>
+      <c r="PK7" s="14"/>
+      <c r="PL7" s="14"/>
+      <c r="PM7" s="14"/>
+      <c r="PN7" s="14"/>
+      <c r="PO7" s="14"/>
+      <c r="PP7" s="14"/>
+      <c r="PQ7" s="14"/>
+      <c r="PR7" s="14"/>
+      <c r="PS7" s="14"/>
+      <c r="PT7" s="14"/>
+      <c r="PU7" s="14"/>
+      <c r="PV7" s="14"/>
+      <c r="PW7" s="14"/>
+      <c r="PX7" s="14"/>
+      <c r="PY7" s="14"/>
+      <c r="PZ7" s="14"/>
+      <c r="QA7" s="14"/>
+      <c r="QB7" s="14"/>
+      <c r="QC7" s="14"/>
+      <c r="QD7" s="14"/>
+      <c r="QE7" s="14"/>
+      <c r="QF7" s="14"/>
+      <c r="QG7" s="14"/>
+      <c r="QH7" s="14"/>
+      <c r="QI7" s="14"/>
+      <c r="QJ7" s="14"/>
+      <c r="QK7" s="14"/>
+      <c r="QL7" s="14"/>
+      <c r="QM7" s="14"/>
+      <c r="QN7" s="14"/>
+      <c r="QO7" s="14"/>
+      <c r="QP7" s="14"/>
+      <c r="QQ7" s="14"/>
+      <c r="QR7" s="14"/>
+      <c r="QS7" s="14"/>
+      <c r="QT7" s="14"/>
+      <c r="QU7" s="14"/>
+      <c r="QV7" s="14"/>
+      <c r="QW7" s="14"/>
+      <c r="QX7" s="14"/>
+      <c r="QY7" s="14"/>
+      <c r="QZ7" s="14"/>
+      <c r="RA7" s="14"/>
+      <c r="RB7" s="14"/>
+      <c r="RC7" s="14"/>
+      <c r="RD7" s="14"/>
+      <c r="RE7" s="14"/>
+      <c r="RF7" s="14"/>
+      <c r="RG7" s="14"/>
+      <c r="RH7" s="14"/>
+      <c r="RI7" s="14"/>
+      <c r="RJ7" s="14"/>
+      <c r="RK7" s="14"/>
+      <c r="RL7" s="14"/>
+      <c r="RM7" s="14"/>
+      <c r="RN7" s="14"/>
+      <c r="RO7" s="14"/>
+      <c r="RP7" s="14"/>
+      <c r="RQ7" s="14"/>
+      <c r="RR7" s="14"/>
+      <c r="RS7" s="14"/>
+      <c r="RT7" s="14"/>
+      <c r="RU7" s="14"/>
+      <c r="RV7" s="14"/>
+      <c r="RW7" s="14"/>
+      <c r="RX7" s="14"/>
+      <c r="RY7" s="14"/>
+      <c r="RZ7" s="14"/>
+      <c r="SA7" s="14"/>
+      <c r="SB7" s="14"/>
+      <c r="SC7" s="14"/>
+      <c r="SD7" s="14"/>
+      <c r="SE7" s="14"/>
+      <c r="SF7" s="14"/>
+    </row>
+    <row r="8" spans="1:500" ht="36">
+      <c r="A8" s="21" t="s">
+        <v>141</v>
+      </c>
+      <c r="B8" s="21" t="s">
+        <v>148</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>149</v>
+      </c>
+      <c r="D8" s="21" t="s">
+        <v>150</v>
+      </c>
+      <c r="E8" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
+      <c r="I8" s="14"/>
+      <c r="J8" s="14"/>
+      <c r="K8" s="14"/>
+      <c r="L8" s="14"/>
+      <c r="M8" s="14"/>
+      <c r="N8" s="14"/>
+      <c r="O8" s="14"/>
+      <c r="P8" s="14"/>
+      <c r="Q8" s="14"/>
+      <c r="R8" s="14"/>
+      <c r="S8" s="14"/>
+      <c r="T8" s="14"/>
+      <c r="U8" s="14"/>
+      <c r="V8" s="14"/>
+      <c r="W8" s="14"/>
+      <c r="X8" s="14"/>
+      <c r="Y8" s="14"/>
+      <c r="Z8" s="14"/>
+      <c r="AA8" s="14"/>
+      <c r="AB8" s="14"/>
+      <c r="AC8" s="14"/>
+      <c r="AD8" s="14"/>
+      <c r="AE8" s="14"/>
+      <c r="AF8" s="14"/>
+      <c r="AG8" s="14"/>
+      <c r="AH8" s="14"/>
+      <c r="AI8" s="14"/>
+      <c r="AJ8" s="14"/>
+      <c r="AK8" s="14"/>
+      <c r="AL8" s="14"/>
+      <c r="AM8" s="14"/>
+      <c r="AN8" s="14"/>
+      <c r="AO8" s="14"/>
+      <c r="AP8" s="14"/>
+      <c r="AQ8" s="14"/>
+      <c r="AR8" s="14"/>
+      <c r="AS8" s="14"/>
+      <c r="AT8" s="14"/>
+      <c r="AU8" s="14"/>
+      <c r="AV8" s="14"/>
+      <c r="AW8" s="14"/>
+      <c r="AX8" s="14"/>
+      <c r="AY8" s="14"/>
+      <c r="AZ8" s="14"/>
+      <c r="BA8" s="14"/>
+      <c r="BB8" s="14"/>
+      <c r="BC8" s="14"/>
+      <c r="BD8" s="14"/>
+      <c r="BE8" s="14"/>
+      <c r="BF8" s="14"/>
+      <c r="BG8" s="14"/>
+      <c r="BH8" s="14"/>
+      <c r="BI8" s="14"/>
+      <c r="BJ8" s="14"/>
+      <c r="BK8" s="14"/>
+      <c r="BL8" s="14"/>
+      <c r="BM8" s="14"/>
+      <c r="BN8" s="14"/>
+      <c r="BO8" s="14"/>
+      <c r="BP8" s="14"/>
+      <c r="BQ8" s="14"/>
+      <c r="BR8" s="14"/>
+      <c r="BS8" s="14"/>
+      <c r="BT8" s="14"/>
+      <c r="BU8" s="14"/>
+      <c r="BV8" s="14"/>
+      <c r="BW8" s="14"/>
+      <c r="BX8" s="14"/>
+      <c r="BY8" s="14"/>
+      <c r="BZ8" s="14"/>
+      <c r="CA8" s="14"/>
+      <c r="CB8" s="14"/>
+      <c r="CC8" s="14"/>
+      <c r="CD8" s="14"/>
+      <c r="CE8" s="14"/>
+      <c r="CF8" s="14"/>
+      <c r="CG8" s="14"/>
+      <c r="CH8" s="14"/>
+      <c r="CI8" s="14"/>
+      <c r="CJ8" s="14"/>
+      <c r="CK8" s="14"/>
+      <c r="CL8" s="14"/>
+      <c r="CM8" s="14"/>
+      <c r="CN8" s="14"/>
+      <c r="CO8" s="14"/>
+      <c r="CP8" s="14"/>
+      <c r="CQ8" s="14"/>
+      <c r="CR8" s="14"/>
+      <c r="CS8" s="14"/>
+      <c r="CT8" s="14"/>
+      <c r="CU8" s="14"/>
+      <c r="CV8" s="14"/>
+      <c r="CW8" s="14"/>
+      <c r="CX8" s="14"/>
+      <c r="CY8" s="14"/>
+      <c r="CZ8" s="14"/>
+      <c r="DA8" s="14"/>
+      <c r="DB8" s="14"/>
+      <c r="DC8" s="14"/>
+      <c r="DD8" s="14"/>
+      <c r="DE8" s="14"/>
+      <c r="DF8" s="14"/>
+      <c r="DG8" s="14"/>
+      <c r="DH8" s="14"/>
+      <c r="DI8" s="14"/>
+      <c r="DJ8" s="14"/>
+      <c r="DK8" s="14"/>
+      <c r="DL8" s="14"/>
+      <c r="DM8" s="14"/>
+      <c r="DN8" s="14"/>
+      <c r="DO8" s="14"/>
+      <c r="DP8" s="14"/>
+      <c r="DQ8" s="14"/>
+      <c r="DR8" s="14"/>
+      <c r="DS8" s="14"/>
+      <c r="DT8" s="14"/>
+      <c r="DU8" s="14"/>
+      <c r="DV8" s="14"/>
+      <c r="DW8" s="14"/>
+      <c r="DX8" s="14"/>
+      <c r="DY8" s="14"/>
+      <c r="DZ8" s="14"/>
+      <c r="EA8" s="14"/>
+      <c r="EB8" s="14"/>
+      <c r="EC8" s="14"/>
+      <c r="ED8" s="14"/>
+      <c r="EE8" s="14"/>
+      <c r="EF8" s="14"/>
+      <c r="EG8" s="14"/>
+      <c r="EH8" s="14"/>
+      <c r="EI8" s="14"/>
+      <c r="EJ8" s="14"/>
+      <c r="EK8" s="14"/>
+      <c r="EL8" s="14"/>
+      <c r="EM8" s="14"/>
+      <c r="EN8" s="14"/>
+      <c r="EO8" s="14"/>
+      <c r="EP8" s="14"/>
+      <c r="EQ8" s="14"/>
+      <c r="ER8" s="14"/>
+      <c r="ES8" s="14"/>
+      <c r="ET8" s="14"/>
+      <c r="EU8" s="14"/>
+      <c r="EV8" s="14"/>
+      <c r="EW8" s="14"/>
+      <c r="EX8" s="14"/>
+      <c r="EY8" s="14"/>
+      <c r="EZ8" s="14"/>
+      <c r="FA8" s="14"/>
+      <c r="FB8" s="14"/>
+      <c r="FC8" s="14"/>
+      <c r="FD8" s="14"/>
+      <c r="FE8" s="14"/>
+      <c r="FF8" s="14"/>
+      <c r="FG8" s="14"/>
+      <c r="FH8" s="14"/>
+      <c r="FI8" s="14"/>
+      <c r="FJ8" s="14"/>
+      <c r="FK8" s="14"/>
+      <c r="FL8" s="14"/>
+      <c r="FM8" s="14"/>
+      <c r="FN8" s="14"/>
+      <c r="FO8" s="14"/>
+      <c r="FP8" s="14"/>
+      <c r="FQ8" s="14"/>
+      <c r="FR8" s="14"/>
+      <c r="FS8" s="14"/>
+      <c r="FT8" s="14"/>
+      <c r="FU8" s="14"/>
+      <c r="FV8" s="14"/>
+      <c r="FW8" s="14"/>
+      <c r="FX8" s="14"/>
+      <c r="FY8" s="14"/>
+      <c r="FZ8" s="14"/>
+      <c r="GA8" s="14"/>
+      <c r="GB8" s="14"/>
+      <c r="GC8" s="14"/>
+      <c r="GD8" s="14"/>
+      <c r="GE8" s="14"/>
+      <c r="GF8" s="14"/>
+      <c r="GG8" s="14"/>
+      <c r="GH8" s="14"/>
+      <c r="GI8" s="14"/>
+      <c r="GJ8" s="14"/>
+      <c r="GK8" s="14"/>
+      <c r="GL8" s="14"/>
+      <c r="GM8" s="14"/>
+      <c r="GN8" s="14"/>
+      <c r="GO8" s="14"/>
+      <c r="GP8" s="14"/>
+      <c r="GQ8" s="14"/>
+      <c r="GR8" s="14"/>
+      <c r="GS8" s="14"/>
+      <c r="GT8" s="14"/>
+      <c r="GU8" s="14"/>
+      <c r="GV8" s="14"/>
+      <c r="GW8" s="14"/>
+      <c r="GX8" s="14"/>
+      <c r="GY8" s="14"/>
+      <c r="GZ8" s="14"/>
+      <c r="HA8" s="14"/>
+      <c r="HB8" s="14"/>
+      <c r="HC8" s="14"/>
+      <c r="HD8" s="14"/>
+      <c r="HE8" s="14"/>
+      <c r="HF8" s="14"/>
+      <c r="HG8" s="14"/>
+      <c r="HH8" s="14"/>
+      <c r="HI8" s="14"/>
+      <c r="HJ8" s="14"/>
+      <c r="HK8" s="14"/>
+      <c r="HL8" s="14"/>
+      <c r="HM8" s="14"/>
+      <c r="HN8" s="14"/>
+      <c r="HO8" s="14"/>
+      <c r="HP8" s="14"/>
+      <c r="HQ8" s="14"/>
+      <c r="HR8" s="14"/>
+      <c r="HS8" s="14"/>
+      <c r="HT8" s="14"/>
+      <c r="HU8" s="14"/>
+      <c r="HV8" s="14"/>
+      <c r="HW8" s="14"/>
+      <c r="HX8" s="14"/>
+      <c r="HY8" s="14"/>
+      <c r="HZ8" s="14"/>
+      <c r="IA8" s="14"/>
+      <c r="IB8" s="14"/>
+      <c r="IC8" s="14"/>
+      <c r="ID8" s="14"/>
+      <c r="IE8" s="14"/>
+      <c r="IF8" s="14"/>
+      <c r="IG8" s="14"/>
+      <c r="IH8" s="14"/>
+      <c r="II8" s="14"/>
+      <c r="IJ8" s="14"/>
+      <c r="IK8" s="14"/>
+      <c r="IL8" s="14"/>
+      <c r="IM8" s="14"/>
+      <c r="IN8" s="14"/>
+      <c r="IO8" s="14"/>
+      <c r="IP8" s="14"/>
+      <c r="IQ8" s="14"/>
+      <c r="IR8" s="14"/>
+      <c r="IS8" s="14"/>
+      <c r="IT8" s="14"/>
+      <c r="IU8" s="14"/>
+      <c r="IV8" s="14"/>
+      <c r="IW8" s="14"/>
+      <c r="IX8" s="14"/>
+      <c r="IY8" s="14"/>
+      <c r="IZ8" s="14"/>
+      <c r="JA8" s="14"/>
+      <c r="JB8" s="14"/>
+      <c r="JC8" s="14"/>
+      <c r="JD8" s="14"/>
+      <c r="JE8" s="14"/>
+      <c r="JF8" s="14"/>
+      <c r="JG8" s="14"/>
+      <c r="JH8" s="14"/>
+      <c r="JI8" s="14"/>
+      <c r="JJ8" s="14"/>
+      <c r="JK8" s="14"/>
+      <c r="JL8" s="14"/>
+      <c r="JM8" s="14"/>
+      <c r="JN8" s="14"/>
+      <c r="JO8" s="14"/>
+      <c r="JP8" s="14"/>
+      <c r="JQ8" s="14"/>
+      <c r="JR8" s="14"/>
+      <c r="JS8" s="14"/>
+      <c r="JT8" s="14"/>
+      <c r="JU8" s="14"/>
+      <c r="JV8" s="14"/>
+      <c r="JW8" s="14"/>
+      <c r="JX8" s="14"/>
+      <c r="JY8" s="14"/>
+      <c r="JZ8" s="14"/>
+      <c r="KA8" s="14"/>
+      <c r="KB8" s="14"/>
+      <c r="KC8" s="14"/>
+      <c r="KD8" s="14"/>
+      <c r="KE8" s="14"/>
+      <c r="KF8" s="14"/>
+      <c r="KG8" s="14"/>
+      <c r="KH8" s="14"/>
+      <c r="KI8" s="14"/>
+      <c r="KJ8" s="14"/>
+      <c r="KK8" s="14"/>
+      <c r="KL8" s="14"/>
+      <c r="KM8" s="14"/>
+      <c r="KN8" s="14"/>
+      <c r="KO8" s="14"/>
+      <c r="KP8" s="14"/>
+      <c r="KQ8" s="14"/>
+      <c r="KR8" s="14"/>
+      <c r="KS8" s="14"/>
+      <c r="KT8" s="14"/>
+      <c r="KU8" s="14"/>
+      <c r="KV8" s="14"/>
+      <c r="KW8" s="14"/>
+      <c r="KX8" s="14"/>
+      <c r="KY8" s="14"/>
+      <c r="KZ8" s="14"/>
+      <c r="LA8" s="14"/>
+      <c r="LB8" s="14"/>
+      <c r="LC8" s="14"/>
+      <c r="LD8" s="14"/>
+      <c r="LE8" s="14"/>
+      <c r="LF8" s="14"/>
+      <c r="LG8" s="14"/>
+      <c r="LH8" s="14"/>
+      <c r="LI8" s="14"/>
+      <c r="LJ8" s="14"/>
+      <c r="LK8" s="14"/>
+      <c r="LL8" s="14"/>
+      <c r="LM8" s="14"/>
+      <c r="LN8" s="14"/>
+      <c r="LO8" s="14"/>
+      <c r="LP8" s="14"/>
+      <c r="LQ8" s="14"/>
+      <c r="LR8" s="14"/>
+      <c r="LS8" s="14"/>
+      <c r="LT8" s="14"/>
+      <c r="LU8" s="14"/>
+      <c r="LV8" s="14"/>
+      <c r="LW8" s="14"/>
+      <c r="LX8" s="14"/>
+      <c r="LY8" s="14"/>
+      <c r="LZ8" s="14"/>
+      <c r="MA8" s="14"/>
+      <c r="MB8" s="14"/>
+      <c r="MC8" s="14"/>
+      <c r="MD8" s="14"/>
+      <c r="ME8" s="14"/>
+      <c r="MF8" s="14"/>
+      <c r="MG8" s="14"/>
+      <c r="MH8" s="14"/>
+      <c r="MI8" s="14"/>
+      <c r="MJ8" s="14"/>
+      <c r="MK8" s="14"/>
+      <c r="ML8" s="14"/>
+      <c r="MM8" s="14"/>
+      <c r="MN8" s="14"/>
+      <c r="MO8" s="14"/>
+      <c r="MP8" s="14"/>
+      <c r="MQ8" s="14"/>
+      <c r="MR8" s="14"/>
+      <c r="MS8" s="14"/>
+      <c r="MT8" s="14"/>
+      <c r="MU8" s="14"/>
+      <c r="MV8" s="14"/>
+      <c r="MW8" s="14"/>
+      <c r="MX8" s="14"/>
+      <c r="MY8" s="14"/>
+      <c r="MZ8" s="14"/>
+      <c r="NA8" s="14"/>
+      <c r="NB8" s="14"/>
+      <c r="NC8" s="14"/>
+      <c r="ND8" s="14"/>
+      <c r="NE8" s="14"/>
+      <c r="NF8" s="14"/>
+      <c r="NG8" s="14"/>
+      <c r="NH8" s="14"/>
+      <c r="NI8" s="14"/>
+      <c r="NJ8" s="14"/>
+      <c r="NK8" s="14"/>
+      <c r="NL8" s="14"/>
+      <c r="NM8" s="14"/>
+      <c r="NN8" s="14"/>
+      <c r="NO8" s="14"/>
+      <c r="NP8" s="14"/>
+      <c r="NQ8" s="14"/>
+      <c r="NR8" s="14"/>
+      <c r="NS8" s="14"/>
+      <c r="NT8" s="14"/>
+      <c r="NU8" s="14"/>
+      <c r="NV8" s="14"/>
+      <c r="NW8" s="14"/>
+      <c r="NX8" s="14"/>
+      <c r="NY8" s="14"/>
+      <c r="NZ8" s="14"/>
+      <c r="OA8" s="14"/>
+      <c r="OB8" s="14"/>
+      <c r="OC8" s="14"/>
+      <c r="OD8" s="14"/>
+      <c r="OE8" s="14"/>
+      <c r="OF8" s="14"/>
+      <c r="OG8" s="14"/>
+      <c r="OH8" s="14"/>
+      <c r="OI8" s="14"/>
+      <c r="OJ8" s="14"/>
+      <c r="OK8" s="14"/>
+      <c r="OL8" s="14"/>
+      <c r="OM8" s="14"/>
+      <c r="ON8" s="14"/>
+      <c r="OO8" s="14"/>
+      <c r="OP8" s="14"/>
+      <c r="OQ8" s="14"/>
+      <c r="OR8" s="14"/>
+      <c r="OS8" s="14"/>
+      <c r="OT8" s="14"/>
+      <c r="OU8" s="14"/>
+      <c r="OV8" s="14"/>
+      <c r="OW8" s="14"/>
+      <c r="OX8" s="14"/>
+      <c r="OY8" s="14"/>
+      <c r="OZ8" s="14"/>
+      <c r="PA8" s="14"/>
+      <c r="PB8" s="14"/>
+      <c r="PC8" s="14"/>
+      <c r="PD8" s="14"/>
+      <c r="PE8" s="14"/>
+      <c r="PF8" s="14"/>
+      <c r="PG8" s="14"/>
+      <c r="PH8" s="14"/>
+      <c r="PI8" s="14"/>
+      <c r="PJ8" s="14"/>
+      <c r="PK8" s="14"/>
+      <c r="PL8" s="14"/>
+      <c r="PM8" s="14"/>
+      <c r="PN8" s="14"/>
+      <c r="PO8" s="14"/>
+      <c r="PP8" s="14"/>
+      <c r="PQ8" s="14"/>
+      <c r="PR8" s="14"/>
+      <c r="PS8" s="14"/>
+      <c r="PT8" s="14"/>
+      <c r="PU8" s="14"/>
+      <c r="PV8" s="14"/>
+      <c r="PW8" s="14"/>
+      <c r="PX8" s="14"/>
+      <c r="PY8" s="14"/>
+      <c r="PZ8" s="14"/>
+      <c r="QA8" s="14"/>
+      <c r="QB8" s="14"/>
+      <c r="QC8" s="14"/>
+      <c r="QD8" s="14"/>
+      <c r="QE8" s="14"/>
+      <c r="QF8" s="14"/>
+      <c r="QG8" s="14"/>
+      <c r="QH8" s="14"/>
+      <c r="QI8" s="14"/>
+      <c r="QJ8" s="14"/>
+      <c r="QK8" s="14"/>
+      <c r="QL8" s="14"/>
+      <c r="QM8" s="14"/>
+      <c r="QN8" s="14"/>
+      <c r="QO8" s="14"/>
+      <c r="QP8" s="14"/>
+      <c r="QQ8" s="14"/>
+      <c r="QR8" s="14"/>
+      <c r="QS8" s="14"/>
+      <c r="QT8" s="14"/>
+      <c r="QU8" s="14"/>
+      <c r="QV8" s="14"/>
+      <c r="QW8" s="14"/>
+      <c r="QX8" s="14"/>
+      <c r="QY8" s="14"/>
+      <c r="QZ8" s="14"/>
+      <c r="RA8" s="14"/>
+      <c r="RB8" s="14"/>
+      <c r="RC8" s="14"/>
+      <c r="RD8" s="14"/>
+      <c r="RE8" s="14"/>
+      <c r="RF8" s="14"/>
+      <c r="RG8" s="14"/>
+      <c r="RH8" s="14"/>
+      <c r="RI8" s="14"/>
+      <c r="RJ8" s="14"/>
+      <c r="RK8" s="14"/>
+      <c r="RL8" s="14"/>
+      <c r="RM8" s="14"/>
+      <c r="RN8" s="14"/>
+      <c r="RO8" s="14"/>
+      <c r="RP8" s="14"/>
+      <c r="RQ8" s="14"/>
+      <c r="RR8" s="14"/>
+      <c r="RS8" s="14"/>
+      <c r="RT8" s="14"/>
+      <c r="RU8" s="14"/>
+      <c r="RV8" s="14"/>
+      <c r="RW8" s="14"/>
+      <c r="RX8" s="14"/>
+      <c r="RY8" s="14"/>
+      <c r="RZ8" s="14"/>
+      <c r="SA8" s="14"/>
+      <c r="SB8" s="14"/>
+      <c r="SC8" s="14"/>
+      <c r="SD8" s="14"/>
+      <c r="SE8" s="14"/>
+      <c r="SF8" s="14"/>
+    </row>
+    <row r="9" spans="1:500" ht="36">
+      <c r="A9" s="21" t="s">
+        <v>141</v>
+      </c>
+      <c r="B9" s="21" t="s">
+        <v>151</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>152</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>153</v>
+      </c>
+      <c r="E9" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" s="22"/>
+      <c r="G9" s="22"/>
+      <c r="H9" s="22"/>
+      <c r="I9" s="22"/>
+      <c r="J9" s="22"/>
+      <c r="K9" s="22"/>
+      <c r="L9" s="22"/>
+      <c r="M9" s="22"/>
+      <c r="N9" s="22"/>
+      <c r="O9" s="22"/>
+      <c r="P9" s="22"/>
+      <c r="Q9" s="22"/>
+      <c r="R9" s="22"/>
+      <c r="S9" s="22"/>
+      <c r="T9" s="22"/>
+      <c r="U9" s="22"/>
+      <c r="V9" s="22"/>
+      <c r="W9" s="22"/>
+      <c r="X9" s="22"/>
+      <c r="Y9" s="22"/>
+      <c r="Z9" s="22"/>
+      <c r="AA9" s="22"/>
+      <c r="AB9" s="22"/>
+      <c r="AC9" s="22"/>
+      <c r="AD9" s="22"/>
+      <c r="AE9" s="22"/>
+      <c r="AF9" s="22"/>
+      <c r="AG9" s="22"/>
+      <c r="AH9" s="22"/>
+      <c r="AI9" s="22"/>
+      <c r="AJ9" s="22"/>
+      <c r="AK9" s="22"/>
+      <c r="AL9" s="22"/>
+      <c r="AM9" s="22"/>
+      <c r="AN9" s="22"/>
+      <c r="AO9" s="22"/>
+      <c r="AP9" s="22"/>
+      <c r="AQ9" s="22"/>
+      <c r="AR9" s="22"/>
+      <c r="AS9" s="22"/>
+      <c r="AT9" s="22"/>
+      <c r="AU9" s="22"/>
+      <c r="AV9" s="22"/>
+      <c r="AW9" s="22"/>
+      <c r="AX9" s="22"/>
+      <c r="AY9" s="22"/>
+      <c r="AZ9" s="22"/>
+      <c r="BA9" s="22"/>
+      <c r="BB9" s="22"/>
+      <c r="BC9" s="22"/>
+      <c r="BD9" s="22"/>
+      <c r="BE9" s="22"/>
+      <c r="BF9" s="22"/>
+      <c r="BG9" s="22"/>
+      <c r="BH9" s="22"/>
+      <c r="BI9" s="22"/>
+      <c r="BJ9" s="22"/>
+      <c r="BK9" s="22"/>
+      <c r="BL9" s="22"/>
+      <c r="BM9" s="22"/>
+      <c r="BN9" s="22"/>
+      <c r="BO9" s="22"/>
+      <c r="BP9" s="22"/>
+      <c r="BQ9" s="22"/>
+      <c r="BR9" s="22"/>
+      <c r="BS9" s="22"/>
+      <c r="BT9" s="22"/>
+      <c r="BU9" s="22"/>
+      <c r="BV9" s="22"/>
+      <c r="BW9" s="22"/>
+      <c r="BX9" s="22"/>
+      <c r="BY9" s="22"/>
+      <c r="BZ9" s="22"/>
+      <c r="CA9" s="22"/>
+      <c r="CB9" s="22"/>
+      <c r="CC9" s="22"/>
+      <c r="CD9" s="22"/>
+      <c r="CE9" s="22"/>
+      <c r="CF9" s="22"/>
+      <c r="CG9" s="22"/>
+      <c r="CH9" s="22"/>
+      <c r="CI9" s="22"/>
+      <c r="CJ9" s="22"/>
+      <c r="CK9" s="22"/>
+      <c r="CL9" s="22"/>
+      <c r="CM9" s="22"/>
+      <c r="CN9" s="22"/>
+      <c r="CO9" s="22"/>
+      <c r="CP9" s="22"/>
+      <c r="CQ9" s="22"/>
+      <c r="CR9" s="22"/>
+      <c r="CS9" s="22"/>
+      <c r="CT9" s="22"/>
+      <c r="CU9" s="22"/>
+      <c r="CV9" s="22"/>
+      <c r="CW9" s="22"/>
+      <c r="CX9" s="22"/>
+      <c r="CY9" s="22"/>
+      <c r="CZ9" s="22"/>
+      <c r="DA9" s="22"/>
+      <c r="DB9" s="22"/>
+      <c r="DC9" s="22"/>
+      <c r="DD9" s="22"/>
+      <c r="DE9" s="22"/>
+      <c r="DF9" s="22"/>
+      <c r="DG9" s="22"/>
+      <c r="DH9" s="22"/>
+      <c r="DI9" s="22"/>
+      <c r="DJ9" s="22"/>
+      <c r="DK9" s="22"/>
+      <c r="DL9" s="22"/>
+      <c r="DM9" s="22"/>
+      <c r="DN9" s="22"/>
+      <c r="DO9" s="22"/>
+      <c r="DP9" s="22"/>
+      <c r="DQ9" s="22"/>
+      <c r="DR9" s="22"/>
+      <c r="DS9" s="22"/>
+      <c r="DT9" s="22"/>
+      <c r="DU9" s="22"/>
+      <c r="DV9" s="22"/>
+      <c r="DW9" s="22"/>
+      <c r="DX9" s="22"/>
+      <c r="DY9" s="22"/>
+      <c r="DZ9" s="22"/>
+      <c r="EA9" s="22"/>
+      <c r="EB9" s="22"/>
+      <c r="EC9" s="22"/>
+      <c r="ED9" s="22"/>
+      <c r="EE9" s="22"/>
+      <c r="EF9" s="22"/>
+      <c r="EG9" s="22"/>
+      <c r="EH9" s="22"/>
+      <c r="EI9" s="22"/>
+      <c r="EJ9" s="22"/>
+      <c r="EK9" s="22"/>
+      <c r="EL9" s="22"/>
+      <c r="EM9" s="22"/>
+      <c r="EN9" s="22"/>
+      <c r="EO9" s="22"/>
+      <c r="EP9" s="22"/>
+      <c r="EQ9" s="22"/>
+      <c r="ER9" s="22"/>
+      <c r="ES9" s="22"/>
+      <c r="ET9" s="22"/>
+      <c r="EU9" s="22"/>
+      <c r="EV9" s="22"/>
+      <c r="EW9" s="22"/>
+      <c r="EX9" s="22"/>
+      <c r="EY9" s="22"/>
+      <c r="EZ9" s="22"/>
+      <c r="FA9" s="22"/>
+      <c r="FB9" s="22"/>
+      <c r="FC9" s="22"/>
+      <c r="FD9" s="22"/>
+      <c r="FE9" s="22"/>
+      <c r="FF9" s="22"/>
+      <c r="FG9" s="22"/>
+      <c r="FH9" s="22"/>
+      <c r="FI9" s="22"/>
+      <c r="FJ9" s="22"/>
+      <c r="FK9" s="22"/>
+      <c r="FL9" s="22"/>
+      <c r="FM9" s="22"/>
+      <c r="FN9" s="22"/>
+      <c r="FO9" s="22"/>
+      <c r="FP9" s="22"/>
+      <c r="FQ9" s="22"/>
+      <c r="FR9" s="22"/>
+      <c r="FS9" s="22"/>
+      <c r="FT9" s="22"/>
+      <c r="FU9" s="22"/>
+      <c r="FV9" s="22"/>
+      <c r="FW9" s="22"/>
+      <c r="FX9" s="22"/>
+      <c r="FY9" s="22"/>
+      <c r="FZ9" s="22"/>
+      <c r="GA9" s="22"/>
+      <c r="GB9" s="22"/>
+      <c r="GC9" s="22"/>
+      <c r="GD9" s="22"/>
+      <c r="GE9" s="22"/>
+      <c r="GF9" s="22"/>
+      <c r="GG9" s="22"/>
+      <c r="GH9" s="22"/>
+      <c r="GI9" s="22"/>
+      <c r="GJ9" s="22"/>
+      <c r="GK9" s="22"/>
+      <c r="GL9" s="22"/>
+      <c r="GM9" s="22"/>
+      <c r="GN9" s="22"/>
+      <c r="GO9" s="22"/>
+      <c r="GP9" s="22"/>
+      <c r="GQ9" s="22"/>
+      <c r="GR9" s="22"/>
+      <c r="GS9" s="22"/>
+      <c r="GT9" s="22"/>
+      <c r="GU9" s="22"/>
+      <c r="GV9" s="22"/>
+      <c r="GW9" s="22"/>
+      <c r="GX9" s="22"/>
+      <c r="GY9" s="22"/>
+      <c r="GZ9" s="22"/>
+      <c r="HA9" s="22"/>
+      <c r="HB9" s="22"/>
+      <c r="HC9" s="22"/>
+      <c r="HD9" s="22"/>
+      <c r="HE9" s="22"/>
+      <c r="HF9" s="22"/>
+      <c r="HG9" s="22"/>
+      <c r="HH9" s="22"/>
+      <c r="HI9" s="22"/>
+      <c r="HJ9" s="22"/>
+      <c r="HK9" s="22"/>
+      <c r="HL9" s="22"/>
+      <c r="HM9" s="22"/>
+      <c r="HN9" s="22"/>
+      <c r="HO9" s="22"/>
+      <c r="HP9" s="22"/>
+      <c r="HQ9" s="22"/>
+      <c r="HR9" s="22"/>
+      <c r="HS9" s="22"/>
+      <c r="HT9" s="22"/>
+      <c r="HU9" s="22"/>
+      <c r="HV9" s="22"/>
+      <c r="HW9" s="22"/>
+      <c r="HX9" s="22"/>
+      <c r="HY9" s="22"/>
+      <c r="HZ9" s="22"/>
+      <c r="IA9" s="22"/>
+      <c r="IB9" s="22"/>
+      <c r="IC9" s="22"/>
+      <c r="ID9" s="22"/>
+      <c r="IE9" s="22"/>
+      <c r="IF9" s="22"/>
+      <c r="IG9" s="22"/>
+      <c r="IH9" s="22"/>
+      <c r="II9" s="22"/>
+      <c r="IJ9" s="22"/>
+      <c r="IK9" s="22"/>
+      <c r="IL9" s="22"/>
+      <c r="IM9" s="22"/>
+      <c r="IN9" s="22"/>
+      <c r="IO9" s="22"/>
+      <c r="IP9" s="22"/>
+      <c r="IQ9" s="22"/>
+      <c r="IR9" s="22"/>
+      <c r="IS9" s="22"/>
+      <c r="IT9" s="22"/>
+      <c r="IU9" s="22"/>
+      <c r="IV9" s="22"/>
+      <c r="IW9" s="22"/>
+      <c r="IX9" s="22"/>
+      <c r="IY9" s="22"/>
+      <c r="IZ9" s="22"/>
+      <c r="JA9" s="22"/>
+      <c r="JB9" s="22"/>
+      <c r="JC9" s="22"/>
+      <c r="JD9" s="22"/>
+      <c r="JE9" s="22"/>
+      <c r="JF9" s="22"/>
+      <c r="JG9" s="22"/>
+      <c r="JH9" s="22"/>
+      <c r="JI9" s="22"/>
+      <c r="JJ9" s="22"/>
+      <c r="JK9" s="22"/>
+      <c r="JL9" s="22"/>
+      <c r="JM9" s="22"/>
+      <c r="JN9" s="22"/>
+      <c r="JO9" s="22"/>
+      <c r="JP9" s="22"/>
+      <c r="JQ9" s="22"/>
+      <c r="JR9" s="22"/>
+      <c r="JS9" s="22"/>
+      <c r="JT9" s="22"/>
+      <c r="JU9" s="22"/>
+      <c r="JV9" s="22"/>
+      <c r="JW9" s="22"/>
+      <c r="JX9" s="22"/>
+      <c r="JY9" s="22"/>
+      <c r="JZ9" s="22"/>
+      <c r="KA9" s="22"/>
+      <c r="KB9" s="22"/>
+      <c r="KC9" s="22"/>
+      <c r="KD9" s="22"/>
+      <c r="KE9" s="22"/>
+      <c r="KF9" s="22"/>
+      <c r="KG9" s="22"/>
+      <c r="KH9" s="22"/>
+      <c r="KI9" s="22"/>
+      <c r="KJ9" s="22"/>
+      <c r="KK9" s="22"/>
+      <c r="KL9" s="22"/>
+      <c r="KM9" s="22"/>
+      <c r="KN9" s="22"/>
+      <c r="KO9" s="22"/>
+      <c r="KP9" s="22"/>
+      <c r="KQ9" s="22"/>
+      <c r="KR9" s="22"/>
+      <c r="KS9" s="22"/>
+      <c r="KT9" s="22"/>
+      <c r="KU9" s="22"/>
+      <c r="KV9" s="22"/>
+      <c r="KW9" s="22"/>
+      <c r="KX9" s="22"/>
+      <c r="KY9" s="22"/>
+      <c r="KZ9" s="22"/>
+      <c r="LA9" s="22"/>
+      <c r="LB9" s="22"/>
+      <c r="LC9" s="22"/>
+      <c r="LD9" s="22"/>
+      <c r="LE9" s="22"/>
+      <c r="LF9" s="22"/>
+      <c r="LG9" s="22"/>
+      <c r="LH9" s="22"/>
+      <c r="LI9" s="22"/>
+      <c r="LJ9" s="22"/>
+      <c r="LK9" s="22"/>
+      <c r="LL9" s="22"/>
+      <c r="LM9" s="22"/>
+      <c r="LN9" s="22"/>
+      <c r="LO9" s="22"/>
+      <c r="LP9" s="22"/>
+      <c r="LQ9" s="22"/>
+      <c r="LR9" s="22"/>
+      <c r="LS9" s="22"/>
+      <c r="LT9" s="22"/>
+      <c r="LU9" s="22"/>
+      <c r="LV9" s="22"/>
+      <c r="LW9" s="22"/>
+      <c r="LX9" s="22"/>
+      <c r="LY9" s="22"/>
+      <c r="LZ9" s="22"/>
+      <c r="MA9" s="22"/>
+      <c r="MB9" s="22"/>
+      <c r="MC9" s="22"/>
+      <c r="MD9" s="22"/>
+      <c r="ME9" s="22"/>
+      <c r="MF9" s="22"/>
+      <c r="MG9" s="22"/>
+      <c r="MH9" s="22"/>
+      <c r="MI9" s="22"/>
+      <c r="MJ9" s="22"/>
+      <c r="MK9" s="22"/>
+      <c r="ML9" s="22"/>
+      <c r="MM9" s="22"/>
+      <c r="MN9" s="22"/>
+      <c r="MO9" s="22"/>
+      <c r="MP9" s="22"/>
+      <c r="MQ9" s="22"/>
+      <c r="MR9" s="22"/>
+      <c r="MS9" s="22"/>
+      <c r="MT9" s="22"/>
+      <c r="MU9" s="22"/>
+      <c r="MV9" s="22"/>
+      <c r="MW9" s="22"/>
+      <c r="MX9" s="22"/>
+      <c r="MY9" s="22"/>
+      <c r="MZ9" s="22"/>
+      <c r="NA9" s="22"/>
+      <c r="NB9" s="22"/>
+      <c r="NC9" s="22"/>
+      <c r="ND9" s="22"/>
+      <c r="NE9" s="22"/>
+      <c r="NF9" s="22"/>
+      <c r="NG9" s="22"/>
+      <c r="NH9" s="22"/>
+      <c r="NI9" s="22"/>
+      <c r="NJ9" s="22"/>
+      <c r="NK9" s="22"/>
+      <c r="NL9" s="22"/>
+      <c r="NM9" s="22"/>
+      <c r="NN9" s="22"/>
+      <c r="NO9" s="22"/>
+      <c r="NP9" s="22"/>
+      <c r="NQ9" s="22"/>
+      <c r="NR9" s="22"/>
+      <c r="NS9" s="22"/>
+      <c r="NT9" s="22"/>
+      <c r="NU9" s="22"/>
+      <c r="NV9" s="22"/>
+      <c r="NW9" s="22"/>
+      <c r="NX9" s="22"/>
+      <c r="NY9" s="22"/>
+      <c r="NZ9" s="22"/>
+      <c r="OA9" s="22"/>
+      <c r="OB9" s="22"/>
+      <c r="OC9" s="22"/>
+      <c r="OD9" s="22"/>
+      <c r="OE9" s="22"/>
+      <c r="OF9" s="22"/>
+      <c r="OG9" s="22"/>
+      <c r="OH9" s="22"/>
+      <c r="OI9" s="22"/>
+      <c r="OJ9" s="22"/>
+      <c r="OK9" s="22"/>
+      <c r="OL9" s="22"/>
+      <c r="OM9" s="22"/>
+      <c r="ON9" s="22"/>
+      <c r="OO9" s="22"/>
+      <c r="OP9" s="22"/>
+      <c r="OQ9" s="22"/>
+      <c r="OR9" s="22"/>
+      <c r="OS9" s="22"/>
+      <c r="OT9" s="22"/>
+      <c r="OU9" s="22"/>
+      <c r="OV9" s="22"/>
+      <c r="OW9" s="22"/>
+      <c r="OX9" s="22"/>
+      <c r="OY9" s="22"/>
+      <c r="OZ9" s="22"/>
+      <c r="PA9" s="22"/>
+      <c r="PB9" s="22"/>
+      <c r="PC9" s="22"/>
+      <c r="PD9" s="22"/>
+      <c r="PE9" s="22"/>
+      <c r="PF9" s="22"/>
+      <c r="PG9" s="22"/>
+      <c r="PH9" s="22"/>
+      <c r="PI9" s="22"/>
+      <c r="PJ9" s="22"/>
+      <c r="PK9" s="22"/>
+      <c r="PL9" s="22"/>
+      <c r="PM9" s="22"/>
+      <c r="PN9" s="22"/>
+      <c r="PO9" s="22"/>
+      <c r="PP9" s="22"/>
+      <c r="PQ9" s="22"/>
+      <c r="PR9" s="22"/>
+      <c r="PS9" s="22"/>
+      <c r="PT9" s="22"/>
+      <c r="PU9" s="22"/>
+      <c r="PV9" s="22"/>
+      <c r="PW9" s="22"/>
+      <c r="PX9" s="22"/>
+      <c r="PY9" s="22"/>
+      <c r="PZ9" s="22"/>
+      <c r="QA9" s="22"/>
+      <c r="QB9" s="22"/>
+      <c r="QC9" s="22"/>
+      <c r="QD9" s="22"/>
+      <c r="QE9" s="22"/>
+      <c r="QF9" s="22"/>
+      <c r="QG9" s="22"/>
+      <c r="QH9" s="22"/>
+      <c r="QI9" s="22"/>
+      <c r="QJ9" s="22"/>
+      <c r="QK9" s="22"/>
+      <c r="QL9" s="22"/>
+      <c r="QM9" s="22"/>
+      <c r="QN9" s="22"/>
+      <c r="QO9" s="22"/>
+      <c r="QP9" s="22"/>
+      <c r="QQ9" s="22"/>
+      <c r="QR9" s="22"/>
+      <c r="QS9" s="22"/>
+      <c r="QT9" s="22"/>
+      <c r="QU9" s="22"/>
+      <c r="QV9" s="22"/>
+      <c r="QW9" s="22"/>
+      <c r="QX9" s="22"/>
+      <c r="QY9" s="22"/>
+      <c r="QZ9" s="22"/>
+      <c r="RA9" s="22"/>
+      <c r="RB9" s="22"/>
+      <c r="RC9" s="22"/>
+      <c r="RD9" s="22"/>
+      <c r="RE9" s="22"/>
+      <c r="RF9" s="22"/>
+      <c r="RG9" s="22"/>
+      <c r="RH9" s="22"/>
+      <c r="RI9" s="22"/>
+      <c r="RJ9" s="22"/>
+      <c r="RK9" s="22"/>
+      <c r="RL9" s="22"/>
+      <c r="RM9" s="22"/>
+      <c r="RN9" s="22"/>
+      <c r="RO9" s="22"/>
+      <c r="RP9" s="22"/>
+      <c r="RQ9" s="22"/>
+      <c r="RR9" s="22"/>
+      <c r="RS9" s="22"/>
+      <c r="RT9" s="22"/>
+      <c r="RU9" s="22"/>
+      <c r="RV9" s="22"/>
+      <c r="RW9" s="22"/>
+      <c r="RX9" s="22"/>
+      <c r="RY9" s="22"/>
+      <c r="RZ9" s="22"/>
+      <c r="SA9" s="22"/>
+      <c r="SB9" s="22"/>
+      <c r="SC9" s="22"/>
+      <c r="SD9" s="22"/>
+      <c r="SE9" s="22"/>
+      <c r="SF9" s="22"/>
+    </row>
+    <row r="10" spans="1:500" ht="36">
+      <c r="A10" s="21" t="s">
+        <v>141</v>
+      </c>
+      <c r="B10" s="21" t="s">
+        <v>154</v>
+      </c>
+      <c r="C10" s="21" t="s">
+        <v>155</v>
+      </c>
+      <c r="D10" s="21" t="s">
+        <v>156</v>
+      </c>
+      <c r="E10" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" s="22"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="22"/>
+      <c r="I10" s="22"/>
+      <c r="J10" s="22"/>
+      <c r="K10" s="22"/>
+      <c r="L10" s="22"/>
+      <c r="M10" s="22"/>
+      <c r="N10" s="22"/>
+      <c r="O10" s="22"/>
+      <c r="P10" s="22"/>
+      <c r="Q10" s="22"/>
+      <c r="R10" s="22"/>
+      <c r="S10" s="22"/>
+      <c r="T10" s="22"/>
+      <c r="U10" s="22"/>
+      <c r="V10" s="22"/>
+      <c r="W10" s="22"/>
+      <c r="X10" s="22"/>
+      <c r="Y10" s="22"/>
+      <c r="Z10" s="22"/>
+      <c r="AA10" s="22"/>
+      <c r="AB10" s="22"/>
+      <c r="AC10" s="22"/>
+      <c r="AD10" s="22"/>
+      <c r="AE10" s="22"/>
+      <c r="AF10" s="22"/>
+      <c r="AG10" s="22"/>
+      <c r="AH10" s="22"/>
+      <c r="AI10" s="22"/>
+      <c r="AJ10" s="22"/>
+      <c r="AK10" s="22"/>
+      <c r="AL10" s="22"/>
+      <c r="AM10" s="22"/>
+      <c r="AN10" s="22"/>
+      <c r="AO10" s="22"/>
+      <c r="AP10" s="22"/>
+      <c r="AQ10" s="22"/>
+      <c r="AR10" s="22"/>
+      <c r="AS10" s="22"/>
+      <c r="AT10" s="22"/>
+      <c r="AU10" s="22"/>
+      <c r="AV10" s="22"/>
+      <c r="AW10" s="22"/>
+      <c r="AX10" s="22"/>
+      <c r="AY10" s="22"/>
+      <c r="AZ10" s="22"/>
+      <c r="BA10" s="22"/>
+      <c r="BB10" s="22"/>
+      <c r="BC10" s="22"/>
+      <c r="BD10" s="22"/>
+      <c r="BE10" s="22"/>
+      <c r="BF10" s="22"/>
+      <c r="BG10" s="22"/>
+      <c r="BH10" s="22"/>
+      <c r="BI10" s="22"/>
+      <c r="BJ10" s="22"/>
+      <c r="BK10" s="22"/>
+      <c r="BL10" s="22"/>
+      <c r="BM10" s="22"/>
+      <c r="BN10" s="22"/>
+      <c r="BO10" s="22"/>
+      <c r="BP10" s="22"/>
+      <c r="BQ10" s="22"/>
+      <c r="BR10" s="22"/>
+      <c r="BS10" s="22"/>
+      <c r="BT10" s="22"/>
+      <c r="BU10" s="22"/>
+      <c r="BV10" s="22"/>
+      <c r="BW10" s="22"/>
+      <c r="BX10" s="22"/>
+      <c r="BY10" s="22"/>
+      <c r="BZ10" s="22"/>
+      <c r="CA10" s="22"/>
+      <c r="CB10" s="22"/>
+      <c r="CC10" s="22"/>
+      <c r="CD10" s="22"/>
+      <c r="CE10" s="22"/>
+      <c r="CF10" s="22"/>
+      <c r="CG10" s="22"/>
+      <c r="CH10" s="22"/>
+      <c r="CI10" s="22"/>
+      <c r="CJ10" s="22"/>
+      <c r="CK10" s="22"/>
+      <c r="CL10" s="22"/>
+      <c r="CM10" s="22"/>
+      <c r="CN10" s="22"/>
+      <c r="CO10" s="22"/>
+      <c r="CP10" s="22"/>
+      <c r="CQ10" s="22"/>
+      <c r="CR10" s="22"/>
+      <c r="CS10" s="22"/>
+      <c r="CT10" s="22"/>
+      <c r="CU10" s="22"/>
+      <c r="CV10" s="22"/>
+      <c r="CW10" s="22"/>
+      <c r="CX10" s="22"/>
+      <c r="CY10" s="22"/>
+      <c r="CZ10" s="22"/>
+      <c r="DA10" s="22"/>
+      <c r="DB10" s="22"/>
+      <c r="DC10" s="22"/>
+      <c r="DD10" s="22"/>
+      <c r="DE10" s="22"/>
+      <c r="DF10" s="22"/>
+      <c r="DG10" s="22"/>
+      <c r="DH10" s="22"/>
+      <c r="DI10" s="22"/>
+      <c r="DJ10" s="22"/>
+      <c r="DK10" s="22"/>
+      <c r="DL10" s="22"/>
+      <c r="DM10" s="22"/>
+      <c r="DN10" s="22"/>
+      <c r="DO10" s="22"/>
+      <c r="DP10" s="22"/>
+      <c r="DQ10" s="22"/>
+      <c r="DR10" s="22"/>
+      <c r="DS10" s="22"/>
+      <c r="DT10" s="22"/>
+      <c r="DU10" s="22"/>
+      <c r="DV10" s="22"/>
+      <c r="DW10" s="22"/>
+      <c r="DX10" s="22"/>
+      <c r="DY10" s="22"/>
+      <c r="DZ10" s="22"/>
+      <c r="EA10" s="22"/>
+      <c r="EB10" s="22"/>
+      <c r="EC10" s="22"/>
+      <c r="ED10" s="22"/>
+      <c r="EE10" s="22"/>
+      <c r="EF10" s="22"/>
+      <c r="EG10" s="22"/>
+      <c r="EH10" s="22"/>
+      <c r="EI10" s="22"/>
+      <c r="EJ10" s="22"/>
+      <c r="EK10" s="22"/>
+      <c r="EL10" s="22"/>
+      <c r="EM10" s="22"/>
+      <c r="EN10" s="22"/>
+      <c r="EO10" s="22"/>
+      <c r="EP10" s="22"/>
+      <c r="EQ10" s="22"/>
+      <c r="ER10" s="22"/>
+      <c r="ES10" s="22"/>
+      <c r="ET10" s="22"/>
+      <c r="EU10" s="22"/>
+      <c r="EV10" s="22"/>
+      <c r="EW10" s="22"/>
+      <c r="EX10" s="22"/>
+      <c r="EY10" s="22"/>
+      <c r="EZ10" s="22"/>
+      <c r="FA10" s="22"/>
+      <c r="FB10" s="22"/>
+      <c r="FC10" s="22"/>
+      <c r="FD10" s="22"/>
+      <c r="FE10" s="22"/>
+      <c r="FF10" s="22"/>
+      <c r="FG10" s="22"/>
+      <c r="FH10" s="22"/>
+      <c r="FI10" s="22"/>
+      <c r="FJ10" s="22"/>
+      <c r="FK10" s="22"/>
+      <c r="FL10" s="22"/>
+      <c r="FM10" s="22"/>
+      <c r="FN10" s="22"/>
+      <c r="FO10" s="22"/>
+      <c r="FP10" s="22"/>
+      <c r="FQ10" s="22"/>
+      <c r="FR10" s="22"/>
+      <c r="FS10" s="22"/>
+      <c r="FT10" s="22"/>
+      <c r="FU10" s="22"/>
+      <c r="FV10" s="22"/>
+      <c r="FW10" s="22"/>
+      <c r="FX10" s="22"/>
+      <c r="FY10" s="22"/>
+      <c r="FZ10" s="22"/>
+      <c r="GA10" s="22"/>
+      <c r="GB10" s="22"/>
+      <c r="GC10" s="22"/>
+      <c r="GD10" s="22"/>
+      <c r="GE10" s="22"/>
+      <c r="GF10" s="22"/>
+      <c r="GG10" s="22"/>
+      <c r="GH10" s="22"/>
+      <c r="GI10" s="22"/>
+      <c r="GJ10" s="22"/>
+      <c r="GK10" s="22"/>
+      <c r="GL10" s="22"/>
+      <c r="GM10" s="22"/>
+      <c r="GN10" s="22"/>
+      <c r="GO10" s="22"/>
+      <c r="GP10" s="22"/>
+      <c r="GQ10" s="22"/>
+      <c r="GR10" s="22"/>
+      <c r="GS10" s="22"/>
+      <c r="GT10" s="22"/>
+      <c r="GU10" s="22"/>
+      <c r="GV10" s="22"/>
+      <c r="GW10" s="22"/>
+      <c r="GX10" s="22"/>
+      <c r="GY10" s="22"/>
+      <c r="GZ10" s="22"/>
+      <c r="HA10" s="22"/>
+      <c r="HB10" s="22"/>
+      <c r="HC10" s="22"/>
+      <c r="HD10" s="22"/>
+      <c r="HE10" s="22"/>
+      <c r="HF10" s="22"/>
+      <c r="HG10" s="22"/>
+      <c r="HH10" s="22"/>
+      <c r="HI10" s="22"/>
+      <c r="HJ10" s="22"/>
+      <c r="HK10" s="22"/>
+      <c r="HL10" s="22"/>
+      <c r="HM10" s="22"/>
+      <c r="HN10" s="22"/>
+      <c r="HO10" s="22"/>
+      <c r="HP10" s="22"/>
+      <c r="HQ10" s="22"/>
+      <c r="HR10" s="22"/>
+      <c r="HS10" s="22"/>
+      <c r="HT10" s="22"/>
+      <c r="HU10" s="22"/>
+      <c r="HV10" s="22"/>
+      <c r="HW10" s="22"/>
+      <c r="HX10" s="22"/>
+      <c r="HY10" s="22"/>
+      <c r="HZ10" s="22"/>
+      <c r="IA10" s="22"/>
+      <c r="IB10" s="22"/>
+      <c r="IC10" s="22"/>
+      <c r="ID10" s="22"/>
+      <c r="IE10" s="22"/>
+      <c r="IF10" s="22"/>
+      <c r="IG10" s="22"/>
+      <c r="IH10" s="22"/>
+      <c r="II10" s="22"/>
+      <c r="IJ10" s="22"/>
+      <c r="IK10" s="22"/>
+      <c r="IL10" s="22"/>
+      <c r="IM10" s="22"/>
+      <c r="IN10" s="22"/>
+      <c r="IO10" s="22"/>
+      <c r="IP10" s="22"/>
+      <c r="IQ10" s="22"/>
+      <c r="IR10" s="22"/>
+      <c r="IS10" s="22"/>
+      <c r="IT10" s="22"/>
+      <c r="IU10" s="22"/>
+      <c r="IV10" s="22"/>
+      <c r="IW10" s="22"/>
+      <c r="IX10" s="22"/>
+      <c r="IY10" s="22"/>
+      <c r="IZ10" s="22"/>
+      <c r="JA10" s="22"/>
+      <c r="JB10" s="22"/>
+      <c r="JC10" s="22"/>
+      <c r="JD10" s="22"/>
+      <c r="JE10" s="22"/>
+      <c r="JF10" s="22"/>
+      <c r="JG10" s="22"/>
+      <c r="JH10" s="22"/>
+      <c r="JI10" s="22"/>
+      <c r="JJ10" s="22"/>
+      <c r="JK10" s="22"/>
+      <c r="JL10" s="22"/>
+      <c r="JM10" s="22"/>
+      <c r="JN10" s="22"/>
+      <c r="JO10" s="22"/>
+      <c r="JP10" s="22"/>
+      <c r="JQ10" s="22"/>
+      <c r="JR10" s="22"/>
+      <c r="JS10" s="22"/>
+      <c r="JT10" s="22"/>
+      <c r="JU10" s="22"/>
+      <c r="JV10" s="22"/>
+      <c r="JW10" s="22"/>
+      <c r="JX10" s="22"/>
+      <c r="JY10" s="22"/>
+      <c r="JZ10" s="22"/>
+      <c r="KA10" s="22"/>
+      <c r="KB10" s="22"/>
+      <c r="KC10" s="22"/>
+      <c r="KD10" s="22"/>
+      <c r="KE10" s="22"/>
+      <c r="KF10" s="22"/>
+      <c r="KG10" s="22"/>
+      <c r="KH10" s="22"/>
+      <c r="KI10" s="22"/>
+      <c r="KJ10" s="22"/>
+      <c r="KK10" s="22"/>
+      <c r="KL10" s="22"/>
+      <c r="KM10" s="22"/>
+      <c r="KN10" s="22"/>
+      <c r="KO10" s="22"/>
+      <c r="KP10" s="22"/>
+      <c r="KQ10" s="22"/>
+      <c r="KR10" s="22"/>
+      <c r="KS10" s="22"/>
+      <c r="KT10" s="22"/>
+      <c r="KU10" s="22"/>
+      <c r="KV10" s="22"/>
+      <c r="KW10" s="22"/>
+      <c r="KX10" s="22"/>
+      <c r="KY10" s="22"/>
+      <c r="KZ10" s="22"/>
+      <c r="LA10" s="22"/>
+      <c r="LB10" s="22"/>
+      <c r="LC10" s="22"/>
+      <c r="LD10" s="22"/>
+      <c r="LE10" s="22"/>
+      <c r="LF10" s="22"/>
+      <c r="LG10" s="22"/>
+      <c r="LH10" s="22"/>
+      <c r="LI10" s="22"/>
+      <c r="LJ10" s="22"/>
+      <c r="LK10" s="22"/>
+      <c r="LL10" s="22"/>
+      <c r="LM10" s="22"/>
+      <c r="LN10" s="22"/>
+      <c r="LO10" s="22"/>
+      <c r="LP10" s="22"/>
+      <c r="LQ10" s="22"/>
+      <c r="LR10" s="22"/>
+      <c r="LS10" s="22"/>
+      <c r="LT10" s="22"/>
+      <c r="LU10" s="22"/>
+      <c r="LV10" s="22"/>
+      <c r="LW10" s="22"/>
+      <c r="LX10" s="22"/>
+      <c r="LY10" s="22"/>
+      <c r="LZ10" s="22"/>
+      <c r="MA10" s="22"/>
+      <c r="MB10" s="22"/>
+      <c r="MC10" s="22"/>
+      <c r="MD10" s="22"/>
+      <c r="ME10" s="22"/>
+      <c r="MF10" s="22"/>
+      <c r="MG10" s="22"/>
+      <c r="MH10" s="22"/>
+      <c r="MI10" s="22"/>
+      <c r="MJ10" s="22"/>
+      <c r="MK10" s="22"/>
+      <c r="ML10" s="22"/>
+      <c r="MM10" s="22"/>
+      <c r="MN10" s="22"/>
+      <c r="MO10" s="22"/>
+      <c r="MP10" s="22"/>
+      <c r="MQ10" s="22"/>
+      <c r="MR10" s="22"/>
+      <c r="MS10" s="22"/>
+      <c r="MT10" s="22"/>
+      <c r="MU10" s="22"/>
+      <c r="MV10" s="22"/>
+      <c r="MW10" s="22"/>
+      <c r="MX10" s="22"/>
+      <c r="MY10" s="22"/>
+      <c r="MZ10" s="22"/>
+      <c r="NA10" s="22"/>
+      <c r="NB10" s="22"/>
+      <c r="NC10" s="22"/>
+      <c r="ND10" s="22"/>
+      <c r="NE10" s="22"/>
+      <c r="NF10" s="22"/>
+      <c r="NG10" s="22"/>
+      <c r="NH10" s="22"/>
+      <c r="NI10" s="22"/>
+      <c r="NJ10" s="22"/>
+      <c r="NK10" s="22"/>
+      <c r="NL10" s="22"/>
+      <c r="NM10" s="22"/>
+      <c r="NN10" s="22"/>
+      <c r="NO10" s="22"/>
+      <c r="NP10" s="22"/>
+      <c r="NQ10" s="22"/>
+      <c r="NR10" s="22"/>
+      <c r="NS10" s="22"/>
+      <c r="NT10" s="22"/>
+      <c r="NU10" s="22"/>
+      <c r="NV10" s="22"/>
+      <c r="NW10" s="22"/>
+      <c r="NX10" s="22"/>
+      <c r="NY10" s="22"/>
+      <c r="NZ10" s="22"/>
+      <c r="OA10" s="22"/>
+      <c r="OB10" s="22"/>
+      <c r="OC10" s="22"/>
+      <c r="OD10" s="22"/>
+      <c r="OE10" s="22"/>
+      <c r="OF10" s="22"/>
+      <c r="OG10" s="22"/>
+      <c r="OH10" s="22"/>
+      <c r="OI10" s="22"/>
+      <c r="OJ10" s="22"/>
+      <c r="OK10" s="22"/>
+      <c r="OL10" s="22"/>
+      <c r="OM10" s="22"/>
+      <c r="ON10" s="22"/>
+      <c r="OO10" s="22"/>
+      <c r="OP10" s="22"/>
+      <c r="OQ10" s="22"/>
+      <c r="OR10" s="22"/>
+      <c r="OS10" s="22"/>
+      <c r="OT10" s="22"/>
+      <c r="OU10" s="22"/>
+      <c r="OV10" s="22"/>
+      <c r="OW10" s="22"/>
+      <c r="OX10" s="22"/>
+      <c r="OY10" s="22"/>
+      <c r="OZ10" s="22"/>
+      <c r="PA10" s="22"/>
+      <c r="PB10" s="22"/>
+      <c r="PC10" s="22"/>
+      <c r="PD10" s="22"/>
+      <c r="PE10" s="22"/>
+      <c r="PF10" s="22"/>
+      <c r="PG10" s="22"/>
+      <c r="PH10" s="22"/>
+      <c r="PI10" s="22"/>
+      <c r="PJ10" s="22"/>
+      <c r="PK10" s="22"/>
+      <c r="PL10" s="22"/>
+      <c r="PM10" s="22"/>
+      <c r="PN10" s="22"/>
+      <c r="PO10" s="22"/>
+      <c r="PP10" s="22"/>
+      <c r="PQ10" s="22"/>
+      <c r="PR10" s="22"/>
+      <c r="PS10" s="22"/>
+      <c r="PT10" s="22"/>
+      <c r="PU10" s="22"/>
+      <c r="PV10" s="22"/>
+      <c r="PW10" s="22"/>
+      <c r="PX10" s="22"/>
+      <c r="PY10" s="22"/>
+      <c r="PZ10" s="22"/>
+      <c r="QA10" s="22"/>
+      <c r="QB10" s="22"/>
+      <c r="QC10" s="22"/>
+      <c r="QD10" s="22"/>
+      <c r="QE10" s="22"/>
+      <c r="QF10" s="22"/>
+      <c r="QG10" s="22"/>
+      <c r="QH10" s="22"/>
+      <c r="QI10" s="22"/>
+      <c r="QJ10" s="22"/>
+      <c r="QK10" s="22"/>
+      <c r="QL10" s="22"/>
+      <c r="QM10" s="22"/>
+      <c r="QN10" s="22"/>
+      <c r="QO10" s="22"/>
+      <c r="QP10" s="22"/>
+      <c r="QQ10" s="22"/>
+      <c r="QR10" s="22"/>
+      <c r="QS10" s="22"/>
+      <c r="QT10" s="22"/>
+      <c r="QU10" s="22"/>
+      <c r="QV10" s="22"/>
+      <c r="QW10" s="22"/>
+      <c r="QX10" s="22"/>
+      <c r="QY10" s="22"/>
+      <c r="QZ10" s="22"/>
+      <c r="RA10" s="22"/>
+      <c r="RB10" s="22"/>
+      <c r="RC10" s="22"/>
+      <c r="RD10" s="22"/>
+      <c r="RE10" s="22"/>
+      <c r="RF10" s="22"/>
+      <c r="RG10" s="22"/>
+      <c r="RH10" s="22"/>
+      <c r="RI10" s="22"/>
+      <c r="RJ10" s="22"/>
+      <c r="RK10" s="22"/>
+      <c r="RL10" s="22"/>
+      <c r="RM10" s="22"/>
+      <c r="RN10" s="22"/>
+      <c r="RO10" s="22"/>
+      <c r="RP10" s="22"/>
+      <c r="RQ10" s="22"/>
+      <c r="RR10" s="22"/>
+      <c r="RS10" s="22"/>
+      <c r="RT10" s="22"/>
+      <c r="RU10" s="22"/>
+      <c r="RV10" s="22"/>
+      <c r="RW10" s="22"/>
+      <c r="RX10" s="22"/>
+      <c r="RY10" s="22"/>
+      <c r="RZ10" s="22"/>
+      <c r="SA10" s="22"/>
+      <c r="SB10" s="22"/>
+      <c r="SC10" s="22"/>
+      <c r="SD10" s="22"/>
+      <c r="SE10" s="22"/>
+      <c r="SF10" s="22"/>
     </row>
     <row r="65" spans="13:16">
       <c r="M65" s="1" t="s">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="N65" s="1" t="s">
-        <v>1</v>
+        <v>42</v>
       </c>
       <c r="O65" s="1" t="s">
-        <v>2</v>
+        <v>43</v>
       </c>
       <c r="P65" s="1" t="s">
-        <v>3</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated the excel sheet
updated the excel sheet with latest added test case files.
</commit_message>
<xml_diff>
--- a/Test-Case file.xlsx
+++ b/Test-Case file.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30602"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E6D7DF27-F011-4AD0-9F0B-E2B40A8C9629}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7377E0D1-3D10-4192-8D69-9DE013F68E74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="3" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="shubh " sheetId="1" r:id="rId1"/>
@@ -268,9 +268,6 @@
 2. Confirm status is 401 (Unauthorized) or 404 (Not Found).</t>
   </si>
   <si>
-    <t>not uploaded</t>
-  </si>
-  <si>
     <t>Missing email returns bad request</t>
   </si>
   <si>
@@ -320,6 +317,9 @@
 2. Enter valid username and password.
 3. Click the Login button.
 4. Assert that the patient-profile-name element is visible in the DOM.</t>
+  </si>
+  <si>
+    <t>not uploaded</t>
   </si>
   <si>
     <t>Register API</t>
@@ -832,7 +832,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -865,6 +865,12 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -941,7 +947,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1015,6 +1021,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6289,7 +6298,7 @@
         <v>70</v>
       </c>
       <c r="E3" s="26" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="48" customHeight="1">
@@ -6297,16 +6306,16 @@
         <v>63</v>
       </c>
       <c r="B4" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="C4" s="26" t="s">
         <v>72</v>
       </c>
-      <c r="C4" s="26" t="s">
+      <c r="D4" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="D4" s="7" t="s">
-        <v>74</v>
-      </c>
       <c r="E4" s="26" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="F4" s="5"/>
     </row>
@@ -6315,51 +6324,51 @@
         <v>63</v>
       </c>
       <c r="B5" s="26" t="s">
+        <v>74</v>
+      </c>
+      <c r="C5" s="26" t="s">
         <v>75</v>
       </c>
-      <c r="C5" s="26" t="s">
+      <c r="D5" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="D5" s="7" t="s">
-        <v>77</v>
-      </c>
       <c r="E5" s="26" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="F5" s="26"/>
     </row>
     <row r="6" spans="1:7" ht="73.5" customHeight="1">
       <c r="A6" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B6" s="26" t="s">
         <v>78</v>
       </c>
-      <c r="B6" s="26" t="s">
+      <c r="C6" s="26" t="s">
         <v>79</v>
       </c>
-      <c r="C6" s="26" t="s">
+      <c r="D6" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="D6" s="7" t="s">
-        <v>81</v>
-      </c>
       <c r="E6" s="26" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="79.5" customHeight="1">
       <c r="A7" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B7" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="B7" s="26" t="s">
+      <c r="C7" s="26" t="s">
         <v>83</v>
       </c>
-      <c r="C7" s="26" t="s">
+      <c r="D7" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="E7" s="26" t="s">
         <v>85</v>
-      </c>
-      <c r="E7" s="26" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="51" customHeight="1">
@@ -6393,7 +6402,7 @@
         <v>92</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="59.25" customHeight="1">
@@ -6410,7 +6419,7 @@
         <v>95</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="48" customHeight="1">
@@ -6427,7 +6436,7 @@
         <v>98</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="51.75" customHeight="1">
@@ -6461,7 +6470,7 @@
         <v>105</v>
       </c>
       <c r="E13" s="26" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="40.5" customHeight="1">
@@ -6478,7 +6487,7 @@
         <v>108</v>
       </c>
       <c r="E14" s="26" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="63.75" customHeight="1">
@@ -6512,7 +6521,7 @@
         <v>115</v>
       </c>
       <c r="E16" s="26" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="55.5" customHeight="1">
@@ -6529,7 +6538,7 @@
         <v>118</v>
       </c>
       <c r="E17" s="26" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="113.25" customHeight="1">
@@ -6563,7 +6572,7 @@
         <v>126</v>
       </c>
       <c r="E19" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="80.25" customHeight="1">
@@ -6580,7 +6589,7 @@
         <v>130</v>
       </c>
       <c r="E20" s="26" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="97.5" customHeight="1">
@@ -6614,7 +6623,7 @@
         <v>138</v>
       </c>
       <c r="E22" s="26" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="57.75" customHeight="1">
@@ -6631,7 +6640,7 @@
         <v>141</v>
       </c>
       <c r="E23" s="26" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="68.25" customHeight="1">
@@ -6665,7 +6674,7 @@
         <v>148</v>
       </c>
       <c r="E25" s="26" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="56.25" customHeight="1">
@@ -6682,7 +6691,7 @@
         <v>152</v>
       </c>
       <c r="E26" s="26" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="47.25" customHeight="1">
@@ -6699,7 +6708,7 @@
         <v>155</v>
       </c>
       <c r="E27" s="26" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="48.75" customHeight="1">
@@ -6716,7 +6725,7 @@
         <v>159</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="44.25" customHeight="1">
@@ -6733,7 +6742,7 @@
         <v>162</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -6850,7 +6859,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -6986,7 +6995,7 @@
       </c>
     </row>
     <row r="9" spans="1:5" ht="30.75">
-      <c r="A9" t="s">
+      <c r="A9" s="1" t="s">
         <v>169</v>
       </c>
       <c r="B9" t="s">
@@ -7003,7 +7012,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" ht="60.75">
-      <c r="A10" t="s">
+      <c r="A10" s="1" t="s">
         <v>192</v>
       </c>
       <c r="B10" t="s">
@@ -7017,7 +7026,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" ht="45.75">
-      <c r="A11" t="s">
+      <c r="A11" s="1" t="s">
         <v>196</v>
       </c>
       <c r="B11" t="s">
@@ -7031,7 +7040,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" ht="45.75">
-      <c r="A12" t="s">
+      <c r="A12" s="1" t="s">
         <v>196</v>
       </c>
       <c r="B12" t="s">
@@ -7045,7 +7054,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" ht="60.75">
-      <c r="A13" t="s">
+      <c r="A13" s="1" t="s">
         <v>203</v>
       </c>
       <c r="B13" t="s">
@@ -7062,7 +7071,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="60.75">
-      <c r="A14" t="s">
+      <c r="A14" s="1" t="s">
         <v>207</v>
       </c>
       <c r="B14" t="s">
@@ -7079,7 +7088,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="60.75">
-      <c r="A15" t="s">
+      <c r="A15" s="1" t="s">
         <v>211</v>
       </c>
       <c r="B15" t="s">
@@ -7096,7 +7105,7 @@
       </c>
     </row>
     <row r="16" spans="1:5" ht="60.75">
-      <c r="A16" t="s">
+      <c r="A16" s="1" t="s">
         <v>215</v>
       </c>
       <c r="B16" t="s">
@@ -7113,7 +7122,7 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="45.75">
-      <c r="A17" t="s">
+      <c r="A17" s="1" t="s">
         <v>219</v>
       </c>
       <c r="B17" t="s">
@@ -7130,7 +7139,7 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="45.75">
-      <c r="A18" t="s">
+      <c r="A18" s="1" t="s">
         <v>223</v>
       </c>
       <c r="B18" t="s">

</xml_diff>

<commit_message>
updated excel file with latest uploaded test cases
</commit_message>
<xml_diff>
--- a/Test-Case file.xlsx
+++ b/Test-Case file.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30602"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7377E0D1-3D10-4192-8D69-9DE013F68E74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{48ECEE47-3B9D-4214-B14D-9F97DB228857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="3" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="shubh " sheetId="1" r:id="rId1"/>
@@ -319,9 +319,6 @@
 4. Assert that the patient-profile-name element is visible in the DOM.</t>
   </si>
   <si>
-    <t>not uploaded</t>
-  </si>
-  <si>
     <t>Register API</t>
   </si>
   <si>
@@ -365,6 +362,9 @@
     <t>1. Generate a unique mock email.
 2. Send POST to /api/auth/register with name, email, and password.
 3. Confirm status is 200 or 201.</t>
+  </si>
+  <si>
+    <t>not uploaded</t>
   </si>
   <si>
     <t>Remote Session</t>
@@ -6368,21 +6368,21 @@
         <v>84</v>
       </c>
       <c r="E7" s="26" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="51" customHeight="1">
       <c r="A8" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B8" s="26" t="s">
         <v>86</v>
       </c>
-      <c r="B8" s="26" t="s">
+      <c r="C8" s="26" t="s">
         <v>87</v>
       </c>
-      <c r="C8" s="26" t="s">
+      <c r="D8" s="7" t="s">
         <v>88</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>89</v>
       </c>
       <c r="E8" s="26" t="s">
         <v>67</v>
@@ -6390,53 +6390,53 @@
     </row>
     <row r="9" spans="1:7" ht="66.75" customHeight="1">
       <c r="A9" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B9" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="D9" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="D9" s="23" t="s">
-        <v>92</v>
-      </c>
       <c r="E9" s="5" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="59.25" customHeight="1">
       <c r="A10" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B10" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="D10" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="D10" s="23" t="s">
-        <v>95</v>
-      </c>
       <c r="E10" s="5" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="48" customHeight="1">
       <c r="A11" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="D11" s="23" t="s">
         <v>97</v>
       </c>
-      <c r="D11" s="23" t="s">
+      <c r="E11" s="5" t="s">
         <v>98</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="51.75" customHeight="1">
@@ -6470,7 +6470,7 @@
         <v>105</v>
       </c>
       <c r="E13" s="26" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="40.5" customHeight="1">
@@ -6487,7 +6487,7 @@
         <v>108</v>
       </c>
       <c r="E14" s="26" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="63.75" customHeight="1">
@@ -6521,7 +6521,7 @@
         <v>115</v>
       </c>
       <c r="E16" s="26" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="55.5" customHeight="1">
@@ -6538,7 +6538,7 @@
         <v>118</v>
       </c>
       <c r="E17" s="26" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="113.25" customHeight="1">
@@ -6572,7 +6572,7 @@
         <v>126</v>
       </c>
       <c r="E19" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="80.25" customHeight="1">
@@ -6589,7 +6589,7 @@
         <v>130</v>
       </c>
       <c r="E20" s="26" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="97.5" customHeight="1">
@@ -6623,7 +6623,7 @@
         <v>138</v>
       </c>
       <c r="E22" s="26" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="57.75" customHeight="1">
@@ -6640,7 +6640,7 @@
         <v>141</v>
       </c>
       <c r="E23" s="26" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="68.25" customHeight="1">
@@ -6674,7 +6674,7 @@
         <v>148</v>
       </c>
       <c r="E25" s="26" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="56.25" customHeight="1">
@@ -6691,7 +6691,7 @@
         <v>152</v>
       </c>
       <c r="E26" s="26" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="47.25" customHeight="1">
@@ -6708,7 +6708,7 @@
         <v>155</v>
       </c>
       <c r="E27" s="26" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="48.75" customHeight="1">
@@ -6725,7 +6725,7 @@
         <v>159</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="44.25" customHeight="1">
@@ -6742,7 +6742,7 @@
         <v>162</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
     </row>
     <row r="30" spans="1:5">

</xml_diff>

<commit_message>
updated the Test-cases file.xlsx
updated the Test cases with latest uploaded test cases.
</commit_message>
<xml_diff>
--- a/Test-Case file.xlsx
+++ b/Test-Case file.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30602"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30606"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{48ECEE47-3B9D-4214-B14D-9F97DB228857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1AEFA8C5-D101-433C-B9B2-C744625475BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6725,7 +6725,7 @@
         <v>159</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>98</v>
+        <v>67</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="44.25" customHeight="1">
@@ -6742,7 +6742,7 @@
         <v>162</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>98</v>
+        <v>67</v>
       </c>
     </row>
     <row r="30" spans="1:5">

</xml_diff>

<commit_message>
Updated Test-case file.xlsx with latest uploads
</commit_message>
<xml_diff>
--- a/Test-Case file.xlsx
+++ b/Test-Case file.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30606"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1AEFA8C5-D101-433C-B9B2-C744625475BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{65384FEC-3DDC-4BB4-99AB-F2C10F679390}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6470,7 +6470,7 @@
         <v>105</v>
       </c>
       <c r="E13" s="26" t="s">
-        <v>98</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="40.5" customHeight="1">
@@ -6487,7 +6487,7 @@
         <v>108</v>
       </c>
       <c r="E14" s="26" t="s">
-        <v>98</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="63.75" customHeight="1">

</xml_diff>

<commit_message>
updated the Test-Case file.xlsx with latest uploads
</commit_message>
<xml_diff>
--- a/Test-Case file.xlsx
+++ b/Test-Case file.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30606"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{65384FEC-3DDC-4BB4-99AB-F2C10F679390}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CE8C6843-C4E5-4D7B-842F-703E50A34318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6674,7 +6674,7 @@
         <v>148</v>
       </c>
       <c r="E25" s="26" t="s">
-        <v>98</v>
+        <v>67</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="56.25" customHeight="1">
@@ -6691,7 +6691,7 @@
         <v>152</v>
       </c>
       <c r="E26" s="26" t="s">
-        <v>98</v>
+        <v>67</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="47.25" customHeight="1">
@@ -6708,7 +6708,7 @@
         <v>155</v>
       </c>
       <c r="E27" s="26" t="s">
-        <v>98</v>
+        <v>67</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="48.75" customHeight="1">

</xml_diff>

<commit_message>
updated the 'Test-Case file.xlsx
updated the 'Test-Case file.xlsx with new uploaded test cases
</commit_message>
<xml_diff>
--- a/Test-Case file.xlsx
+++ b/Test-Case file.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30606"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30611"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6B7A9027-2B57-4C50-A2DA-ECA65E9F0CE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4875DB6E-8DF6-4C2C-86C4-51BAE26ADB0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="shubh " sheetId="1" r:id="rId1"/>
@@ -6611,7 +6611,7 @@
         <v>134</v>
       </c>
       <c r="E20" s="26" t="s">
-        <v>102</v>
+        <v>71</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="97.5" customHeight="1">

</xml_diff>

<commit_message>
updated the 'Test-Case file.xlsx'
updated the 'Test-Case file.xlsx' with new uploaded test cases
</commit_message>
<xml_diff>
--- a/Test-Case file.xlsx
+++ b/Test-Case file.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30610"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9B54E361-E3E7-4E71-B0A9-84EEB4492F7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6EB508ED-603D-4EF7-AF9A-124203995FB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="239">
   <si>
     <t>Functionality</t>
   </si>
@@ -494,9 +494,6 @@
   <si>
     <t>1. Send POST to /api/auth/forgot-password with email bad-email-format.
 2. Confirm status is 400 (Bad Request).</t>
-  </si>
-  <si>
-    <t>not uploaded</t>
   </si>
   <si>
     <t>Active Tab highlight</t>
@@ -6641,21 +6638,21 @@
         <v>133</v>
       </c>
       <c r="E20" s="22" t="s">
-        <v>134</v>
+        <v>71</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="97.5" customHeight="1">
       <c r="A21" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="B21" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="C21" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="D21" s="6" t="s">
         <v>137</v>
-      </c>
-      <c r="D21" s="6" t="s">
-        <v>138</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>71</v>
@@ -6663,16 +6660,16 @@
     </row>
     <row r="22" spans="1:5" ht="93" customHeight="1">
       <c r="A22" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="B22" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="C22" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="D22" s="7" t="s">
         <v>141</v>
-      </c>
-      <c r="D22" s="7" t="s">
-        <v>142</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>71</v>
@@ -6680,16 +6677,16 @@
     </row>
     <row r="23" spans="1:5" ht="57.75" customHeight="1">
       <c r="A23" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="C23" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="D23" s="6" t="s">
         <v>145</v>
-      </c>
-      <c r="D23" s="6" t="s">
-        <v>146</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>71</v>
@@ -6697,16 +6694,16 @@
     </row>
     <row r="24" spans="1:5" ht="68.25" customHeight="1">
       <c r="A24" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B24" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="C24" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="D24" s="6" t="s">
         <v>148</v>
-      </c>
-      <c r="D24" s="6" t="s">
-        <v>149</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>71</v>
@@ -6714,16 +6711,16 @@
     </row>
     <row r="25" spans="1:5" ht="72.75" customHeight="1">
       <c r="A25" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="B25" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="C25" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="D25" s="26" t="s">
         <v>152</v>
-      </c>
-      <c r="D25" s="26" t="s">
-        <v>153</v>
       </c>
       <c r="E25" s="6" t="s">
         <v>71</v>
@@ -6731,16 +6728,16 @@
     </row>
     <row r="26" spans="1:5" ht="56.25" customHeight="1">
       <c r="A26" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B26" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="C26" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="D26" s="6" t="s">
         <v>155</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>156</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>71</v>
@@ -6748,16 +6745,16 @@
     </row>
     <row r="27" spans="1:5" ht="47.25" customHeight="1">
       <c r="A27" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="B27" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="C27" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="D27" s="6" t="s">
         <v>159</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>160</v>
       </c>
       <c r="E27" s="6" t="s">
         <v>71</v>
@@ -6765,16 +6762,16 @@
     </row>
     <row r="28" spans="1:5" ht="48.75" customHeight="1">
       <c r="A28" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B28" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C28" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="D28" s="6" t="s">
         <v>162</v>
-      </c>
-      <c r="D28" s="6" t="s">
-        <v>163</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>71</v>
@@ -6782,16 +6779,16 @@
     </row>
     <row r="29" spans="1:5" ht="44.25" customHeight="1">
       <c r="A29" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B29" s="22" t="s">
         <v>164</v>
       </c>
-      <c r="B29" s="22" t="s">
+      <c r="C29" s="22" t="s">
         <v>165</v>
       </c>
-      <c r="C29" s="22" t="s">
+      <c r="D29" s="22" t="s">
         <v>166</v>
-      </c>
-      <c r="D29" s="22" t="s">
-        <v>167</v>
       </c>
       <c r="E29" s="22" t="s">
         <v>71</v>
@@ -6799,16 +6796,16 @@
     </row>
     <row r="30" spans="1:5" ht="42.75" customHeight="1">
       <c r="A30" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B30" s="22" t="s">
+        <v>167</v>
+      </c>
+      <c r="C30" s="22" t="s">
         <v>168</v>
       </c>
-      <c r="C30" s="22" t="s">
+      <c r="D30" s="22" t="s">
         <v>169</v>
-      </c>
-      <c r="D30" s="22" t="s">
-        <v>170</v>
       </c>
       <c r="E30" s="22" t="s">
         <v>71</v>
@@ -6816,19 +6813,19 @@
     </row>
     <row r="31" spans="1:5" ht="117.75" customHeight="1">
       <c r="A31" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="B31" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="C31" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="D31" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="D31" s="6" t="s">
+      <c r="E31" s="6" t="s">
         <v>174</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -6957,282 +6954,282 @@
     </row>
     <row r="2" spans="1:5" ht="54.75" customHeight="1">
       <c r="A2" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="B2" s="25" t="s">
         <v>176</v>
       </c>
-      <c r="B2" s="25" t="s">
+      <c r="C2" s="25" t="s">
         <v>177</v>
       </c>
-      <c r="C2" s="25" t="s">
+      <c r="D2" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="E2" s="25" t="s">
         <v>179</v>
-      </c>
-      <c r="E2" s="25" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="39" customHeight="1">
       <c r="A3" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B3" s="25" t="s">
         <v>181</v>
       </c>
-      <c r="B3" s="25" t="s">
+      <c r="C3" s="25" t="s">
         <v>182</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="D3" s="6" t="s">
         <v>183</v>
       </c>
-      <c r="D3" s="6" t="s">
-        <v>184</v>
-      </c>
       <c r="E3" s="25" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="42" customHeight="1">
       <c r="A4" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="B4" s="25" t="s">
         <v>185</v>
       </c>
-      <c r="B4" s="25" t="s">
+      <c r="C4" s="25" t="s">
         <v>186</v>
       </c>
-      <c r="C4" s="25" t="s">
+      <c r="D4" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="D4" s="6" t="s">
-        <v>188</v>
-      </c>
       <c r="E4" s="25" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="39" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B5" s="25" t="s">
+        <v>188</v>
+      </c>
+      <c r="C5" s="25" t="s">
         <v>189</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="D5" s="6" t="s">
         <v>190</v>
       </c>
-      <c r="D5" s="6" t="s">
-        <v>191</v>
-      </c>
       <c r="E5" s="25" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="40.5" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B6" s="25" t="s">
+        <v>191</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="D6" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="D6" s="6" t="s">
-        <v>194</v>
-      </c>
       <c r="E6" s="25" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="43.5" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B7" s="25" t="s">
+        <v>194</v>
+      </c>
+      <c r="C7" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="D7" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="D7" s="6" t="s">
-        <v>197</v>
-      </c>
       <c r="E7" s="25" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="37.5" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B8" s="25" t="s">
+        <v>197</v>
+      </c>
+      <c r="C8" s="25" t="s">
         <v>198</v>
       </c>
-      <c r="C8" s="25" t="s">
+      <c r="D8" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="D8" s="6" t="s">
-        <v>200</v>
-      </c>
       <c r="E8" s="25" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="38.25" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B9" s="25" t="s">
+        <v>200</v>
+      </c>
+      <c r="C9" s="25" t="s">
         <v>201</v>
       </c>
-      <c r="C9" s="25" t="s">
+      <c r="D9" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="D9" s="6" t="s">
-        <v>203</v>
-      </c>
       <c r="E9" s="25" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="68.25" customHeight="1">
       <c r="A10" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="B10" s="25" t="s">
         <v>204</v>
       </c>
-      <c r="B10" s="25" t="s">
+      <c r="C10" s="25" t="s">
         <v>205</v>
       </c>
-      <c r="C10" s="25" t="s">
+      <c r="D10" s="6" t="s">
         <v>206</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>207</v>
       </c>
       <c r="E10" s="25"/>
     </row>
     <row r="11" spans="1:5" ht="58.5" customHeight="1">
       <c r="A11" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B11" s="25" t="s">
         <v>208</v>
       </c>
-      <c r="B11" s="25" t="s">
+      <c r="C11" s="25" t="s">
         <v>209</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="D11" s="6" t="s">
         <v>210</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>211</v>
       </c>
       <c r="E11" s="25"/>
     </row>
     <row r="12" spans="1:5" ht="55.5" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B12" s="25" t="s">
+        <v>211</v>
+      </c>
+      <c r="C12" s="25" t="s">
         <v>212</v>
       </c>
-      <c r="C12" s="25" t="s">
+      <c r="D12" s="6" t="s">
         <v>213</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>214</v>
       </c>
       <c r="E12" s="25"/>
     </row>
     <row r="13" spans="1:5" ht="72" customHeight="1">
       <c r="A13" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="B13" s="25" t="s">
         <v>215</v>
       </c>
-      <c r="B13" s="25" t="s">
+      <c r="C13" s="25" t="s">
         <v>216</v>
       </c>
-      <c r="C13" s="25" t="s">
+      <c r="D13" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="D13" s="6" t="s">
-        <v>218</v>
-      </c>
       <c r="E13" s="25" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="69" customHeight="1">
       <c r="A14" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="B14" s="25" t="s">
         <v>219</v>
       </c>
-      <c r="B14" s="25" t="s">
+      <c r="C14" s="25" t="s">
         <v>220</v>
       </c>
-      <c r="C14" s="25" t="s">
+      <c r="D14" s="6" t="s">
         <v>221</v>
       </c>
-      <c r="D14" s="6" t="s">
-        <v>222</v>
-      </c>
       <c r="E14" s="25" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="73.5" customHeight="1">
       <c r="A15" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="B15" s="25" t="s">
         <v>223</v>
       </c>
-      <c r="B15" s="25" t="s">
+      <c r="C15" s="25" t="s">
         <v>224</v>
       </c>
-      <c r="C15" s="25" t="s">
+      <c r="D15" s="6" t="s">
         <v>225</v>
       </c>
-      <c r="D15" s="6" t="s">
-        <v>226</v>
-      </c>
       <c r="E15" s="25" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="74.25" customHeight="1">
       <c r="A16" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B16" s="25" t="s">
         <v>227</v>
       </c>
-      <c r="B16" s="25" t="s">
+      <c r="C16" s="25" t="s">
         <v>228</v>
       </c>
-      <c r="C16" s="25" t="s">
+      <c r="D16" s="6" t="s">
         <v>229</v>
       </c>
-      <c r="D16" s="6" t="s">
-        <v>230</v>
-      </c>
       <c r="E16" s="25" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="57" customHeight="1">
       <c r="A17" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="B17" s="25" t="s">
         <v>231</v>
       </c>
-      <c r="B17" s="25" t="s">
+      <c r="C17" s="25" t="s">
         <v>232</v>
       </c>
-      <c r="C17" s="25" t="s">
+      <c r="D17" s="6" t="s">
         <v>233</v>
       </c>
-      <c r="D17" s="6" t="s">
-        <v>234</v>
-      </c>
       <c r="E17" s="25" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="60" customHeight="1">
       <c r="A18" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B18" s="25" t="s">
         <v>235</v>
       </c>
-      <c r="B18" s="25" t="s">
+      <c r="C18" s="25" t="s">
         <v>236</v>
       </c>
-      <c r="C18" s="25" t="s">
+      <c r="D18" s="6" t="s">
         <v>237</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>238</v>
       </c>
       <c r="E18" s="25"/>
     </row>
@@ -7244,10 +7241,10 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="5" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C29" s="5"/>
       <c r="D29" s="5"/>

</xml_diff>